<commit_message>
Actualizar metrados.xlsx detallando alturas de montaje, recorridos verticales y curvas en canalizaciones
</commit_message>
<xml_diff>
--- a/proyecto_vivienda_unifamiliar_por_RENZO/metrados/metrados.xlsx
+++ b/proyecto_vivienda_unifamiliar_por_RENZO/metrados/metrados.xlsx
@@ -1098,7 +1098,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M97"/>
+  <dimension ref="A1:M164"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="15" customWidth="1" style="1" min="1" max="1"/>
@@ -1486,7 +1486,10 @@
       <c r="D20" s="127" t="n"/>
       <c r="E20" s="127" t="n"/>
       <c r="F20" s="127" t="n"/>
-      <c r="G20" s="127" t="n"/>
+      <c r="G20" s="127">
+        <f>C20</f>
+        <v/>
+      </c>
       <c r="H20" s="127" t="n"/>
       <c r="I20" s="125" t="n"/>
     </row>
@@ -1503,7 +1506,10 @@
       <c r="D21" s="127" t="n"/>
       <c r="E21" s="127" t="n"/>
       <c r="F21" s="127" t="n"/>
-      <c r="G21" s="127" t="n"/>
+      <c r="G21" s="127">
+        <f>C21</f>
+        <v/>
+      </c>
       <c r="H21" s="127" t="n"/>
       <c r="I21" s="125" t="n"/>
     </row>
@@ -1520,7 +1526,10 @@
       <c r="D22" s="127" t="n"/>
       <c r="E22" s="127" t="n"/>
       <c r="F22" s="127" t="n"/>
-      <c r="G22" s="127" t="n"/>
+      <c r="G22" s="127">
+        <f>C22</f>
+        <v/>
+      </c>
       <c r="H22" s="127" t="n"/>
       <c r="I22" s="125" t="n"/>
     </row>
@@ -1537,7 +1546,10 @@
       <c r="D23" s="127" t="n"/>
       <c r="E23" s="127" t="n"/>
       <c r="F23" s="127" t="n"/>
-      <c r="G23" s="127" t="n"/>
+      <c r="G23" s="127">
+        <f>C23</f>
+        <v/>
+      </c>
       <c r="H23" s="127" t="n"/>
       <c r="I23" s="125" t="n"/>
     </row>
@@ -1554,7 +1566,10 @@
       <c r="D24" s="127" t="n"/>
       <c r="E24" s="127" t="n"/>
       <c r="F24" s="127" t="n"/>
-      <c r="G24" s="127" t="n"/>
+      <c r="G24" s="127">
+        <f>C24</f>
+        <v/>
+      </c>
       <c r="H24" s="127" t="n"/>
       <c r="I24" s="125" t="n"/>
     </row>
@@ -1589,7 +1604,10 @@
       <c r="D26" s="127" t="n"/>
       <c r="E26" s="127" t="n"/>
       <c r="F26" s="127" t="n"/>
-      <c r="G26" s="127" t="n"/>
+      <c r="G26" s="127">
+        <f>C26</f>
+        <v/>
+      </c>
       <c r="H26" s="127" t="n"/>
       <c r="I26" s="125" t="n"/>
     </row>
@@ -1606,7 +1624,10 @@
       <c r="D27" s="127" t="n"/>
       <c r="E27" s="127" t="n"/>
       <c r="F27" s="127" t="n"/>
-      <c r="G27" s="127" t="n"/>
+      <c r="G27" s="127">
+        <f>C27</f>
+        <v/>
+      </c>
       <c r="H27" s="127" t="n"/>
       <c r="I27" s="125" t="n"/>
     </row>
@@ -1623,7 +1644,10 @@
       <c r="D28" s="127" t="n"/>
       <c r="E28" s="127" t="n"/>
       <c r="F28" s="127" t="n"/>
-      <c r="G28" s="127" t="n"/>
+      <c r="G28" s="127">
+        <f>C28</f>
+        <v/>
+      </c>
       <c r="H28" s="127" t="n"/>
       <c r="I28" s="125" t="n"/>
     </row>
@@ -1640,7 +1664,10 @@
       <c r="D29" s="127" t="n"/>
       <c r="E29" s="127" t="n"/>
       <c r="F29" s="127" t="n"/>
-      <c r="G29" s="127" t="n"/>
+      <c r="G29" s="127">
+        <f>C29</f>
+        <v/>
+      </c>
       <c r="H29" s="127" t="n"/>
       <c r="I29" s="125" t="n"/>
     </row>
@@ -1657,7 +1684,10 @@
       <c r="D30" s="127" t="n"/>
       <c r="E30" s="127" t="n"/>
       <c r="F30" s="127" t="n"/>
-      <c r="G30" s="127" t="n"/>
+      <c r="G30" s="127">
+        <f>C30</f>
+        <v/>
+      </c>
       <c r="H30" s="127" t="n"/>
       <c r="I30" s="125" t="n"/>
     </row>
@@ -1692,7 +1722,10 @@
       <c r="D32" s="127" t="n"/>
       <c r="E32" s="127" t="n"/>
       <c r="F32" s="127" t="n"/>
-      <c r="G32" s="127" t="n"/>
+      <c r="G32" s="127">
+        <f>C32</f>
+        <v/>
+      </c>
       <c r="H32" s="127" t="n"/>
       <c r="I32" s="125" t="n"/>
     </row>
@@ -1709,7 +1742,10 @@
       <c r="D33" s="127" t="n"/>
       <c r="E33" s="127" t="n"/>
       <c r="F33" s="127" t="n"/>
-      <c r="G33" s="127" t="n"/>
+      <c r="G33" s="127">
+        <f>C33</f>
+        <v/>
+      </c>
       <c r="H33" s="127" t="n"/>
       <c r="I33" s="125" t="n"/>
     </row>
@@ -1726,7 +1762,10 @@
       <c r="D34" s="127" t="n"/>
       <c r="E34" s="127" t="n"/>
       <c r="F34" s="127" t="n"/>
-      <c r="G34" s="127" t="n"/>
+      <c r="G34" s="127">
+        <f>C34</f>
+        <v/>
+      </c>
       <c r="H34" s="127" t="n"/>
       <c r="I34" s="125" t="n"/>
     </row>
@@ -1743,7 +1782,10 @@
       <c r="D35" s="127" t="n"/>
       <c r="E35" s="127" t="n"/>
       <c r="F35" s="127" t="n"/>
-      <c r="G35" s="127" t="n"/>
+      <c r="G35" s="127">
+        <f>C35</f>
+        <v/>
+      </c>
       <c r="H35" s="127" t="n"/>
       <c r="I35" s="125" t="n"/>
     </row>
@@ -1760,7 +1802,10 @@
       <c r="D36" s="127" t="n"/>
       <c r="E36" s="127" t="n"/>
       <c r="F36" s="127" t="n"/>
-      <c r="G36" s="127" t="n"/>
+      <c r="G36" s="127">
+        <f>C36</f>
+        <v/>
+      </c>
       <c r="H36" s="127" t="n"/>
       <c r="I36" s="125" t="n"/>
     </row>
@@ -1840,7 +1885,10 @@
       <c r="D40" s="127" t="n"/>
       <c r="E40" s="127" t="n"/>
       <c r="F40" s="127" t="n"/>
-      <c r="G40" s="127" t="n"/>
+      <c r="G40" s="127">
+        <f>C40</f>
+        <v/>
+      </c>
       <c r="H40" s="127" t="n"/>
       <c r="I40" s="125" t="n"/>
     </row>
@@ -1857,7 +1905,10 @@
       <c r="D41" s="127" t="n"/>
       <c r="E41" s="127" t="n"/>
       <c r="F41" s="127" t="n"/>
-      <c r="G41" s="127" t="n"/>
+      <c r="G41" s="127">
+        <f>C41</f>
+        <v/>
+      </c>
       <c r="H41" s="127" t="n"/>
       <c r="I41" s="125" t="n"/>
     </row>
@@ -1874,7 +1925,10 @@
       <c r="D42" s="127" t="n"/>
       <c r="E42" s="127" t="n"/>
       <c r="F42" s="127" t="n"/>
-      <c r="G42" s="127" t="n"/>
+      <c r="G42" s="127">
+        <f>C42</f>
+        <v/>
+      </c>
       <c r="H42" s="127" t="n"/>
       <c r="I42" s="125" t="n"/>
     </row>
@@ -1909,7 +1963,10 @@
       <c r="D44" s="127" t="n"/>
       <c r="E44" s="127" t="n"/>
       <c r="F44" s="127" t="n"/>
-      <c r="G44" s="127" t="n"/>
+      <c r="G44" s="127">
+        <f>C44</f>
+        <v/>
+      </c>
       <c r="H44" s="127" t="n"/>
       <c r="I44" s="125" t="n"/>
     </row>
@@ -1926,7 +1983,10 @@
       <c r="D45" s="127" t="n"/>
       <c r="E45" s="127" t="n"/>
       <c r="F45" s="127" t="n"/>
-      <c r="G45" s="127" t="n"/>
+      <c r="G45" s="127">
+        <f>C45</f>
+        <v/>
+      </c>
       <c r="H45" s="127" t="n"/>
       <c r="I45" s="125" t="n"/>
     </row>
@@ -1943,7 +2003,10 @@
       <c r="D46" s="127" t="n"/>
       <c r="E46" s="127" t="n"/>
       <c r="F46" s="127" t="n"/>
-      <c r="G46" s="127" t="n"/>
+      <c r="G46" s="127">
+        <f>C46</f>
+        <v/>
+      </c>
       <c r="H46" s="127" t="n"/>
       <c r="I46" s="125" t="n"/>
     </row>
@@ -1978,7 +2041,10 @@
       <c r="D48" s="127" t="n"/>
       <c r="E48" s="127" t="n"/>
       <c r="F48" s="127" t="n"/>
-      <c r="G48" s="127" t="n"/>
+      <c r="G48" s="127">
+        <f>C48</f>
+        <v/>
+      </c>
       <c r="H48" s="127" t="n"/>
       <c r="I48" s="125" t="n"/>
     </row>
@@ -1995,7 +2061,10 @@
       <c r="D49" s="127" t="n"/>
       <c r="E49" s="127" t="n"/>
       <c r="F49" s="127" t="n"/>
-      <c r="G49" s="127" t="n"/>
+      <c r="G49" s="127">
+        <f>C49</f>
+        <v/>
+      </c>
       <c r="H49" s="127" t="n"/>
       <c r="I49" s="125" t="n"/>
     </row>
@@ -2012,7 +2081,10 @@
       <c r="D50" s="127" t="n"/>
       <c r="E50" s="127" t="n"/>
       <c r="F50" s="127" t="n"/>
-      <c r="G50" s="127" t="n"/>
+      <c r="G50" s="127">
+        <f>C50</f>
+        <v/>
+      </c>
       <c r="H50" s="127" t="n"/>
       <c r="I50" s="125" t="n"/>
     </row>
@@ -2073,7 +2145,10 @@
       <c r="D53" s="127" t="n"/>
       <c r="E53" s="127" t="n"/>
       <c r="F53" s="127" t="n"/>
-      <c r="G53" s="127" t="n"/>
+      <c r="G53" s="127">
+        <f>C53</f>
+        <v/>
+      </c>
       <c r="H53" s="127" t="n"/>
       <c r="I53" s="125" t="n"/>
     </row>
@@ -2108,7 +2183,10 @@
       <c r="D55" s="127" t="n"/>
       <c r="E55" s="127" t="n"/>
       <c r="F55" s="127" t="n"/>
-      <c r="G55" s="127" t="n"/>
+      <c r="G55" s="127">
+        <f>C55</f>
+        <v/>
+      </c>
       <c r="H55" s="127" t="n"/>
       <c r="I55" s="125" t="n"/>
     </row>
@@ -2169,7 +2247,10 @@
       <c r="D58" s="127" t="n"/>
       <c r="E58" s="127" t="n"/>
       <c r="F58" s="127" t="n"/>
-      <c r="G58" s="127" t="n"/>
+      <c r="G58" s="127">
+        <f>C58</f>
+        <v/>
+      </c>
       <c r="H58" s="127" t="n"/>
       <c r="I58" s="125" t="n"/>
     </row>
@@ -2186,7 +2267,10 @@
       <c r="D59" s="127" t="n"/>
       <c r="E59" s="127" t="n"/>
       <c r="F59" s="127" t="n"/>
-      <c r="G59" s="127" t="n"/>
+      <c r="G59" s="127">
+        <f>C59</f>
+        <v/>
+      </c>
       <c r="H59" s="127" t="n"/>
       <c r="I59" s="125" t="n"/>
     </row>
@@ -2221,7 +2305,10 @@
       <c r="D61" s="127" t="n"/>
       <c r="E61" s="127" t="n"/>
       <c r="F61" s="127" t="n"/>
-      <c r="G61" s="127" t="n"/>
+      <c r="G61" s="127">
+        <f>C61</f>
+        <v/>
+      </c>
       <c r="H61" s="127" t="n"/>
       <c r="I61" s="125" t="n"/>
     </row>
@@ -2245,1049 +2332,2326 @@
       <c r="I62" s="122" t="n"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="125" t="inlineStr">
+      <c r="A63" s="131" t="inlineStr">
         <is>
           <t>OE.5.2.2.1</t>
         </is>
       </c>
-      <c r="B63" s="126" t="inlineStr">
-        <is>
-          <t>Tubería PVC Liviana (PV-L) 3/4" (Alumbrado)</t>
-        </is>
-      </c>
-      <c r="C63" s="127" t="n">
-        <v>120</v>
-      </c>
-      <c r="D63" s="127" t="n"/>
-      <c r="E63" s="127" t="n"/>
-      <c r="F63" s="127" t="n"/>
-      <c r="G63" s="127">
-        <f>C63</f>
-        <v/>
-      </c>
-      <c r="H63" s="127">
-        <f>G63</f>
-        <v/>
-      </c>
-      <c r="I63" s="125" t="inlineStr">
+      <c r="B63" s="132" t="inlineStr">
+        <is>
+          <t>Tubería PVC Liviana (PV-L) 3/4" (Canalización Alumbrado)</t>
+        </is>
+      </c>
+      <c r="C63" s="133" t="n"/>
+      <c r="D63" s="133" t="n"/>
+      <c r="E63" s="133" t="n"/>
+      <c r="F63" s="133" t="n"/>
+      <c r="G63" s="133" t="n"/>
+      <c r="H63" s="133">
+        <f>SUM(G64,G67,G70)</f>
+        <v/>
+      </c>
+      <c r="I63" s="131" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.2.2</t>
-        </is>
-      </c>
-      <c r="B64" s="126" t="inlineStr">
-        <is>
-          <t>Tubería PVC Pesada (PV-P) 3/4" (Tomacorrientes)</t>
-        </is>
-      </c>
-      <c r="C64" s="127" t="n">
-        <v>150</v>
-      </c>
-      <c r="D64" s="127" t="n"/>
-      <c r="E64" s="127" t="n"/>
-      <c r="F64" s="127" t="n"/>
-      <c r="G64" s="127">
-        <f>C64</f>
-        <v/>
-      </c>
-      <c r="H64" s="127">
-        <f>G64</f>
-        <v/>
-      </c>
-      <c r="I64" s="125" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+      <c r="A64" s="131" t="n"/>
+      <c r="B64" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C64" s="133" t="n"/>
+      <c r="D64" s="133" t="n"/>
+      <c r="E64" s="133" t="n"/>
+      <c r="F64" s="133" t="n"/>
+      <c r="G64" s="133">
+        <f>SUM(G65:G66)</f>
+        <v/>
+      </c>
+      <c r="H64" s="133" t="n"/>
+      <c r="I64" s="131" t="n"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.2.3</t>
-        </is>
-      </c>
+      <c r="A65" s="125" t="n"/>
       <c r="B65" s="126" t="inlineStr">
         <is>
-          <t>Tubería PVC Pesada (PV-P) 1" (Alimentador)</t>
+          <t>Recorrido Horizontal (En losa de techo)</t>
         </is>
       </c>
       <c r="C65" s="127" t="n">
-        <v>25</v>
-      </c>
-      <c r="D65" s="127" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D65" s="127" t="n">
+        <v>35</v>
+      </c>
       <c r="E65" s="127" t="n"/>
       <c r="F65" s="127" t="n"/>
       <c r="G65" s="127">
-        <f>C65</f>
-        <v/>
-      </c>
-      <c r="H65" s="127">
-        <f>G65</f>
-        <v/>
-      </c>
-      <c r="I65" s="125" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+        <f>C65*D65</f>
+        <v/>
+      </c>
+      <c r="H65" s="127" t="n"/>
+      <c r="I65" s="125" t="n"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.2.4</t>
-        </is>
-      </c>
+      <c r="A66" s="125" t="n"/>
       <c r="B66" s="126" t="inlineStr">
         <is>
-          <t>Accesorios de canalización (Curvas, uniones, conectores, pegamento)</t>
+          <t>Verticales: Bajadas a Cajas de Interruptores (h = 1.40 m)</t>
         </is>
       </c>
       <c r="C66" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="127" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="D66" s="127" t="n">
+        <v>1.4</v>
+      </c>
       <c r="E66" s="127" t="n"/>
       <c r="F66" s="127" t="n"/>
       <c r="G66" s="127">
-        <f>C66</f>
-        <v/>
-      </c>
-      <c r="H66" s="127">
-        <f>G66</f>
-        <v/>
-      </c>
-      <c r="I66" s="125" t="inlineStr">
-        <is>
-          <t>glb</t>
-        </is>
-      </c>
+        <f>C66*D66</f>
+        <v/>
+      </c>
+      <c r="H66" s="127" t="n"/>
+      <c r="I66" s="125" t="n"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="122" t="inlineStr">
-        <is>
-          <t>OE.5.2.3</t>
-        </is>
-      </c>
-      <c r="B67" s="123" t="inlineStr">
-        <is>
-          <t>CONDUCTORES Y CABLES</t>
-        </is>
-      </c>
-      <c r="C67" s="124" t="n"/>
-      <c r="D67" s="124" t="n"/>
-      <c r="E67" s="124" t="n"/>
-      <c r="F67" s="124" t="n"/>
-      <c r="G67" s="124" t="n"/>
-      <c r="H67" s="124" t="n"/>
-      <c r="I67" s="122" t="n"/>
+      <c r="A67" s="131" t="n"/>
+      <c r="B67" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C67" s="133" t="n"/>
+      <c r="D67" s="133" t="n"/>
+      <c r="E67" s="133" t="n"/>
+      <c r="F67" s="133" t="n"/>
+      <c r="G67" s="133">
+        <f>SUM(G68:G69)</f>
+        <v/>
+      </c>
+      <c r="H67" s="133" t="n"/>
+      <c r="I67" s="131" t="n"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
-      <c r="A68" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.3.1</t>
-        </is>
-      </c>
+      <c r="A68" s="125" t="n"/>
       <c r="B68" s="126" t="inlineStr">
         <is>
-          <t>Conductor de cobre LSOH 1.5 mm2 (Fase+Neutro Alumbrado)</t>
+          <t>Recorrido Horizontal (En losa de techo)</t>
         </is>
       </c>
       <c r="C68" s="127" t="n">
-        <v>240</v>
-      </c>
-      <c r="D68" s="127" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D68" s="127" t="n">
+        <v>35</v>
+      </c>
       <c r="E68" s="127" t="n"/>
       <c r="F68" s="127" t="n"/>
       <c r="G68" s="127">
-        <f>C68</f>
-        <v/>
-      </c>
-      <c r="H68" s="127">
-        <f>G68</f>
-        <v/>
-      </c>
-      <c r="I68" s="125" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+        <f>C68*D68</f>
+        <v/>
+      </c>
+      <c r="H68" s="127" t="n"/>
+      <c r="I68" s="125" t="n"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.3.2</t>
-        </is>
-      </c>
+      <c r="A69" s="125" t="n"/>
       <c r="B69" s="126" t="inlineStr">
         <is>
-          <t>Conductor de cobre LSOH 1.5 mm2 (Protección a Tierra Alumbrado)</t>
+          <t>Verticales: Bajadas a Cajas de Interruptores (h = 1.40 m)</t>
         </is>
       </c>
       <c r="C69" s="127" t="n">
-        <v>110</v>
-      </c>
-      <c r="D69" s="127" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="D69" s="127" t="n">
+        <v>1.4</v>
+      </c>
       <c r="E69" s="127" t="n"/>
       <c r="F69" s="127" t="n"/>
       <c r="G69" s="127">
-        <f>C69</f>
-        <v/>
-      </c>
-      <c r="H69" s="127">
-        <f>G69</f>
-        <v/>
-      </c>
-      <c r="I69" s="125" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+        <f>C69*D69</f>
+        <v/>
+      </c>
+      <c r="H69" s="127" t="n"/>
+      <c r="I69" s="125" t="n"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.3.3</t>
-        </is>
-      </c>
-      <c r="B70" s="126" t="inlineStr">
-        <is>
-          <t>Conductor de cobre LSOH 2.5 mm2 (Fase+Neutro Tomacorrientes)</t>
-        </is>
-      </c>
-      <c r="C70" s="127" t="n">
-        <v>300</v>
-      </c>
-      <c r="D70" s="127" t="n"/>
-      <c r="E70" s="127" t="n"/>
-      <c r="F70" s="127" t="n"/>
-      <c r="G70" s="127">
-        <f>C70</f>
-        <v/>
-      </c>
-      <c r="H70" s="127">
-        <f>G70</f>
-        <v/>
-      </c>
-      <c r="I70" s="125" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+      <c r="A70" s="131" t="n"/>
+      <c r="B70" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C70" s="133" t="n"/>
+      <c r="D70" s="133" t="n"/>
+      <c r="E70" s="133" t="n"/>
+      <c r="F70" s="133" t="n"/>
+      <c r="G70" s="133">
+        <f>SUM(G71:G72)</f>
+        <v/>
+      </c>
+      <c r="H70" s="133" t="n"/>
+      <c r="I70" s="131" t="n"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.3.4</t>
-        </is>
-      </c>
+      <c r="A71" s="125" t="n"/>
       <c r="B71" s="126" t="inlineStr">
         <is>
-          <t>Conductor de cobre LSOH 2.5 mm2 (Protección a Tierra Tomacorrientes)</t>
+          <t>Recorrido Horizontal (En losa de techo)</t>
         </is>
       </c>
       <c r="C71" s="127" t="n">
-        <v>150</v>
-      </c>
-      <c r="D71" s="127" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D71" s="127" t="n">
+        <v>36.4</v>
+      </c>
       <c r="E71" s="127" t="n"/>
       <c r="F71" s="127" t="n"/>
       <c r="G71" s="127">
-        <f>C71</f>
-        <v/>
-      </c>
-      <c r="H71" s="127">
-        <f>G71</f>
-        <v/>
-      </c>
-      <c r="I71" s="125" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+        <f>C71*D71</f>
+        <v/>
+      </c>
+      <c r="H71" s="127" t="n"/>
+      <c r="I71" s="125" t="n"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.3.5</t>
-        </is>
-      </c>
+      <c r="A72" s="125" t="n"/>
       <c r="B72" s="126" t="inlineStr">
         <is>
-          <t>Conductor de cobre LSOH 2.5 mm2 (Alimentación Electrobomba)</t>
+          <t>Verticales: Bajadas a Cajas de Interruptores (h = 1.40 m)</t>
         </is>
       </c>
       <c r="C72" s="127" t="n">
-        <v>35</v>
-      </c>
-      <c r="D72" s="127" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="D72" s="127" t="n">
+        <v>1.4</v>
+      </c>
       <c r="E72" s="127" t="n"/>
       <c r="F72" s="127" t="n"/>
       <c r="G72" s="127">
-        <f>C72</f>
-        <v/>
-      </c>
-      <c r="H72" s="127">
-        <f>G72</f>
-        <v/>
-      </c>
-      <c r="I72" s="125" t="inlineStr">
+        <f>C72*D72</f>
+        <v/>
+      </c>
+      <c r="H72" s="127" t="n"/>
+      <c r="I72" s="125" t="n"/>
+    </row>
+    <row r="73" ht="15.75" customHeight="1">
+      <c r="A73" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.2.2</t>
+        </is>
+      </c>
+      <c r="B73" s="132" t="inlineStr">
+        <is>
+          <t>Tubería PVC Pesada (PV-P) 3/4" (Canalización Tomacorrientes)</t>
+        </is>
+      </c>
+      <c r="C73" s="133" t="n"/>
+      <c r="D73" s="133" t="n"/>
+      <c r="E73" s="133" t="n"/>
+      <c r="F73" s="133" t="n"/>
+      <c r="G73" s="133" t="n"/>
+      <c r="H73" s="133">
+        <f>SUM(G74,G78,G82)</f>
+        <v/>
+      </c>
+      <c r="I73" s="131" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.3.6</t>
-        </is>
-      </c>
-      <c r="B73" s="126" t="inlineStr">
-        <is>
-          <t>Conductor de cobre LSOH 10 mm2 (Alimentador General)</t>
-        </is>
-      </c>
-      <c r="C73" s="127" t="n">
-        <v>60</v>
-      </c>
-      <c r="D73" s="127" t="n"/>
-      <c r="E73" s="127" t="n"/>
-      <c r="F73" s="127" t="n"/>
-      <c r="G73" s="127">
-        <f>C73</f>
-        <v/>
-      </c>
-      <c r="H73" s="127">
-        <f>G73</f>
-        <v/>
-      </c>
-      <c r="I73" s="125" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.3.7</t>
-        </is>
-      </c>
-      <c r="B74" s="126" t="inlineStr">
-        <is>
-          <t>Conductor de cobre temple blando 6 mm2 (Conexión Puesta a Tierra)</t>
-        </is>
-      </c>
-      <c r="C74" s="127" t="n">
-        <v>25</v>
-      </c>
-      <c r="D74" s="127" t="n"/>
-      <c r="E74" s="127" t="n"/>
-      <c r="F74" s="127" t="n"/>
-      <c r="G74" s="127">
-        <f>C74</f>
-        <v/>
-      </c>
-      <c r="H74" s="127">
-        <f>G74</f>
-        <v/>
-      </c>
-      <c r="I74" s="125" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+      <c r="A74" s="131" t="n"/>
+      <c r="B74" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C74" s="133" t="n"/>
+      <c r="D74" s="133" t="n"/>
+      <c r="E74" s="133" t="n"/>
+      <c r="F74" s="133" t="n"/>
+      <c r="G74" s="133">
+        <f>SUM(G75:G77)</f>
+        <v/>
+      </c>
+      <c r="H74" s="133" t="n"/>
+      <c r="I74" s="131" t="n"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="122" t="inlineStr">
-        <is>
-          <t>OE.5.2.4</t>
-        </is>
-      </c>
-      <c r="B75" s="123" t="inlineStr">
-        <is>
-          <t>CAJAS DE PASO Y DERIVACION</t>
-        </is>
-      </c>
-      <c r="C75" s="124" t="n"/>
-      <c r="D75" s="124" t="n"/>
-      <c r="E75" s="124" t="n"/>
-      <c r="F75" s="124" t="n"/>
-      <c r="G75" s="124" t="n"/>
-      <c r="H75" s="124" t="n"/>
-      <c r="I75" s="122" t="n"/>
+      <c r="A75" s="125" t="n"/>
+      <c r="B75" s="126" t="inlineStr">
+        <is>
+          <t>Recorrido Horizontal (En contrapiso de piso 1)</t>
+        </is>
+      </c>
+      <c r="C75" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" s="127" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="E75" s="127" t="n"/>
+      <c r="F75" s="127" t="n"/>
+      <c r="G75" s="127">
+        <f>C75*D75</f>
+        <v/>
+      </c>
+      <c r="H75" s="127" t="n"/>
+      <c r="I75" s="125" t="n"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.4.1</t>
-        </is>
-      </c>
+      <c r="A76" s="125" t="n"/>
       <c r="B76" s="126" t="inlineStr">
         <is>
-          <t>Caja de pase rectangular 4"x2" FG (Derivaciones y cambios)</t>
+          <t>Verticales: Subidas a Tomacorrientes Dobles (h = 0.30 m)</t>
         </is>
       </c>
       <c r="C76" s="127" t="n">
-        <v>6</v>
-      </c>
-      <c r="D76" s="127" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="D76" s="127" t="n">
+        <v>0.3</v>
+      </c>
       <c r="E76" s="127" t="n"/>
       <c r="F76" s="127" t="n"/>
       <c r="G76" s="127">
-        <f>C76</f>
-        <v/>
-      </c>
-      <c r="H76" s="127">
-        <f>G76</f>
-        <v/>
-      </c>
-      <c r="I76" s="125" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+        <f>C76*D76</f>
+        <v/>
+      </c>
+      <c r="H76" s="127" t="n"/>
+      <c r="I76" s="125" t="n"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="122" t="inlineStr">
-        <is>
-          <t>OE.5.2.6</t>
-        </is>
-      </c>
-      <c r="B77" s="123" t="inlineStr">
-        <is>
-          <t>TABLEROS DE DISTRIBUCION Y DETALLES</t>
-        </is>
-      </c>
-      <c r="C77" s="124" t="n"/>
-      <c r="D77" s="124" t="n"/>
-      <c r="E77" s="124" t="n"/>
-      <c r="F77" s="124" t="n"/>
-      <c r="G77" s="124" t="n"/>
-      <c r="H77" s="124" t="n"/>
-      <c r="I77" s="122" t="n"/>
+      <c r="A77" s="125" t="n"/>
+      <c r="B77" s="126" t="inlineStr">
+        <is>
+          <t>Verticales: Subidas a Cocina/Bomba (Especiales h = 1.10 m)</t>
+        </is>
+      </c>
+      <c r="C77" s="127" t="n">
+        <v>5</v>
+      </c>
+      <c r="D77" s="127" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E77" s="127" t="n"/>
+      <c r="F77" s="127" t="n"/>
+      <c r="G77" s="127">
+        <f>C77*D77</f>
+        <v/>
+      </c>
+      <c r="H77" s="127" t="n"/>
+      <c r="I77" s="125" t="n"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.6.1</t>
-        </is>
-      </c>
-      <c r="B78" s="126" t="inlineStr">
-        <is>
-          <t>Tablero General TG-01 (12 polos, metálico empotrable, primer piso)</t>
-        </is>
-      </c>
-      <c r="C78" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D78" s="127" t="n"/>
-      <c r="E78" s="127" t="n"/>
-      <c r="F78" s="127" t="n"/>
-      <c r="G78" s="127">
-        <f>C78</f>
-        <v/>
-      </c>
-      <c r="H78" s="127">
-        <f>G78</f>
-        <v/>
-      </c>
-      <c r="I78" s="125" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
+      <c r="A78" s="131" t="n"/>
+      <c r="B78" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C78" s="133" t="n"/>
+      <c r="D78" s="133" t="n"/>
+      <c r="E78" s="133" t="n"/>
+      <c r="F78" s="133" t="n"/>
+      <c r="G78" s="133">
+        <f>SUM(G79:G81)</f>
+        <v/>
+      </c>
+      <c r="H78" s="133" t="n"/>
+      <c r="I78" s="131" t="n"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
-      <c r="A79" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.6.2</t>
-        </is>
-      </c>
+      <c r="A79" s="125" t="n"/>
       <c r="B79" s="126" t="inlineStr">
         <is>
-          <t>Tablero de Distribución TD-01 (8 polos, metálico empotrable, segundo piso)</t>
+          <t>Recorrido Horizontal (En contrapiso de piso 2)</t>
         </is>
       </c>
       <c r="C79" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D79" s="127" t="n"/>
+      <c r="D79" s="127" t="n">
+        <v>50.4</v>
+      </c>
       <c r="E79" s="127" t="n"/>
       <c r="F79" s="127" t="n"/>
       <c r="G79" s="127">
-        <f>C79</f>
-        <v/>
-      </c>
-      <c r="H79" s="127">
-        <f>G79</f>
-        <v/>
-      </c>
-      <c r="I79" s="125" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
+        <f>C79*D79</f>
+        <v/>
+      </c>
+      <c r="H79" s="127" t="n"/>
+      <c r="I79" s="125" t="n"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="A80" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.6.3</t>
-        </is>
-      </c>
+      <c r="A80" s="125" t="n"/>
       <c r="B80" s="126" t="inlineStr">
         <is>
-          <t>Tablero de Distribución TD-02 (8 polos, metálico empotrable, tercer piso)</t>
+          <t>Verticales: Subidas a Tomacorrientes Dobles (h = 0.30 m)</t>
         </is>
       </c>
       <c r="C80" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D80" s="127" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="D80" s="127" t="n">
+        <v>0.3</v>
+      </c>
       <c r="E80" s="127" t="n"/>
       <c r="F80" s="127" t="n"/>
       <c r="G80" s="127">
-        <f>C80</f>
-        <v/>
-      </c>
-      <c r="H80" s="127">
-        <f>G80</f>
-        <v/>
-      </c>
-      <c r="I80" s="125" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
+        <f>C80*D80</f>
+        <v/>
+      </c>
+      <c r="H80" s="127" t="n"/>
+      <c r="I80" s="125" t="n"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
-      <c r="A81" s="122" t="inlineStr">
-        <is>
-          <t>OE.5.2.8</t>
-        </is>
-      </c>
-      <c r="B81" s="123" t="inlineStr">
-        <is>
-          <t>DISPOSITIVOS DE MANIOBRA Y PROTECCION</t>
-        </is>
-      </c>
-      <c r="C81" s="124" t="n"/>
-      <c r="D81" s="124" t="n"/>
-      <c r="E81" s="124" t="n"/>
-      <c r="F81" s="124" t="n"/>
-      <c r="G81" s="124" t="n"/>
-      <c r="H81" s="124" t="n"/>
-      <c r="I81" s="122" t="n"/>
+      <c r="A81" s="125" t="n"/>
+      <c r="B81" s="126" t="inlineStr">
+        <is>
+          <t>Verticales: Subidas a Baño GFCI (h = 1.10 m)</t>
+        </is>
+      </c>
+      <c r="C81" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" s="127" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E81" s="127" t="n"/>
+      <c r="F81" s="127" t="n"/>
+      <c r="G81" s="127">
+        <f>C81*D81</f>
+        <v/>
+      </c>
+      <c r="H81" s="127" t="n"/>
+      <c r="I81" s="125" t="n"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
-      <c r="A82" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.8.1</t>
-        </is>
-      </c>
-      <c r="B82" s="126" t="inlineStr">
-        <is>
-          <t>Interruptor simple unipolar (adosar/empotrar, 10A)</t>
-        </is>
-      </c>
-      <c r="C82" s="127" t="n">
-        <v>6</v>
-      </c>
-      <c r="D82" s="127" t="n"/>
-      <c r="E82" s="127" t="n"/>
-      <c r="F82" s="127" t="n"/>
-      <c r="G82" s="127">
-        <f>C82</f>
-        <v/>
-      </c>
-      <c r="H82" s="127">
-        <f>G82</f>
-        <v/>
-      </c>
-      <c r="I82" s="125" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+      <c r="A82" s="131" t="n"/>
+      <c r="B82" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C82" s="133" t="n"/>
+      <c r="D82" s="133" t="n"/>
+      <c r="E82" s="133" t="n"/>
+      <c r="F82" s="133" t="n"/>
+      <c r="G82" s="133">
+        <f>SUM(G83:G85)</f>
+        <v/>
+      </c>
+      <c r="H82" s="133" t="n"/>
+      <c r="I82" s="131" t="n"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
-      <c r="A83" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.8.2</t>
-        </is>
-      </c>
+      <c r="A83" s="125" t="n"/>
       <c r="B83" s="126" t="inlineStr">
         <is>
-          <t>Interruptor de conmutación 3 vías (S3, escaleras)</t>
+          <t>Recorrido Horizontal (En contrapiso de piso 3)</t>
         </is>
       </c>
       <c r="C83" s="127" t="n">
-        <v>4</v>
-      </c>
-      <c r="D83" s="127" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D83" s="127" t="n">
+        <v>50</v>
+      </c>
       <c r="E83" s="127" t="n"/>
       <c r="F83" s="127" t="n"/>
       <c r="G83" s="127">
-        <f>C83</f>
-        <v/>
-      </c>
-      <c r="H83" s="127">
-        <f>G83</f>
-        <v/>
-      </c>
-      <c r="I83" s="125" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+        <f>C83*D83</f>
+        <v/>
+      </c>
+      <c r="H83" s="127" t="n"/>
+      <c r="I83" s="125" t="n"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
-      <c r="A84" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.8.3</t>
-        </is>
-      </c>
+      <c r="A84" s="125" t="n"/>
       <c r="B84" s="126" t="inlineStr">
         <is>
-          <t>Interruptor termomagnetico 2P-10A (Alumbrado)</t>
+          <t>Verticales: Subidas a Tomacorrientes Dobles (h = 0.30 m)</t>
         </is>
       </c>
       <c r="C84" s="127" t="n">
-        <v>3</v>
-      </c>
-      <c r="D84" s="127" t="n"/>
+        <v>7</v>
+      </c>
+      <c r="D84" s="127" t="n">
+        <v>0.3</v>
+      </c>
       <c r="E84" s="127" t="n"/>
       <c r="F84" s="127" t="n"/>
       <c r="G84" s="127">
-        <f>C84</f>
-        <v/>
-      </c>
-      <c r="H84" s="127">
-        <f>G84</f>
-        <v/>
-      </c>
-      <c r="I84" s="125" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+        <f>C84*D84</f>
+        <v/>
+      </c>
+      <c r="H84" s="127" t="n"/>
+      <c r="I84" s="125" t="n"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
-      <c r="A85" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.8.4</t>
-        </is>
-      </c>
+      <c r="A85" s="125" t="n"/>
       <c r="B85" s="126" t="inlineStr">
         <is>
-          <t>Interruptor termomagnetico 2P-16A (Tomacorrientes)</t>
+          <t>Verticales: Subidas a Baño/Lavandería (h = 1.10 m)</t>
         </is>
       </c>
       <c r="C85" s="127" t="n">
-        <v>5</v>
-      </c>
-      <c r="D85" s="127" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="D85" s="127" t="n">
+        <v>1.1</v>
+      </c>
       <c r="E85" s="127" t="n"/>
       <c r="F85" s="127" t="n"/>
       <c r="G85" s="127">
-        <f>C85</f>
-        <v/>
-      </c>
-      <c r="H85" s="127">
-        <f>G85</f>
-        <v/>
-      </c>
-      <c r="I85" s="125" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+        <f>C85*D85</f>
+        <v/>
+      </c>
+      <c r="H85" s="127" t="n"/>
+      <c r="I85" s="125" t="n"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.8.5</t>
-        </is>
-      </c>
-      <c r="B86" s="126" t="inlineStr">
-        <is>
-          <t>Interruptor termomagnetico 2P-20A (Cocina / Cargas especiales)</t>
-        </is>
-      </c>
-      <c r="C86" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D86" s="127" t="n"/>
-      <c r="E86" s="127" t="n"/>
-      <c r="F86" s="127" t="n"/>
-      <c r="G86" s="127">
-        <f>C86</f>
-        <v/>
-      </c>
-      <c r="H86" s="127">
-        <f>G86</f>
-        <v/>
-      </c>
-      <c r="I86" s="125" t="inlineStr">
-        <is>
-          <t>pza</t>
+      <c r="A86" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.2.3</t>
+        </is>
+      </c>
+      <c r="B86" s="132" t="inlineStr">
+        <is>
+          <t>Tubería PVC Pesada (PV-P) 1" (Canalización Alimentador General)</t>
+        </is>
+      </c>
+      <c r="C86" s="133" t="n"/>
+      <c r="D86" s="133" t="n"/>
+      <c r="E86" s="133" t="n"/>
+      <c r="F86" s="133" t="n"/>
+      <c r="G86" s="133" t="n"/>
+      <c r="H86" s="133">
+        <f>SUM(G87)</f>
+        <v/>
+      </c>
+      <c r="I86" s="131" t="inlineStr">
+        <is>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15.75" customHeight="1">
-      <c r="A87" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.8.6</t>
-        </is>
-      </c>
-      <c r="B87" s="126" t="inlineStr">
-        <is>
-          <t>Interruptor termomagnetico general 2P-40A (TG-01)</t>
-        </is>
-      </c>
-      <c r="C87" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D87" s="127" t="n"/>
-      <c r="E87" s="127" t="n"/>
-      <c r="F87" s="127" t="n"/>
-      <c r="G87" s="127">
-        <f>C87</f>
-        <v/>
-      </c>
-      <c r="H87" s="127">
-        <f>G87</f>
-        <v/>
-      </c>
-      <c r="I87" s="125" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+      <c r="A87" s="131" t="n"/>
+      <c r="B87" s="132" t="inlineStr">
+        <is>
+          <t>TRAMO PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="C87" s="133" t="n"/>
+      <c r="D87" s="133" t="n"/>
+      <c r="E87" s="133" t="n"/>
+      <c r="F87" s="133" t="n"/>
+      <c r="G87" s="133">
+        <f>SUM(G88:G93)</f>
+        <v/>
+      </c>
+      <c r="H87" s="133" t="n"/>
+      <c r="I87" s="131" t="n"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
-      <c r="A88" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.8.7</t>
-        </is>
-      </c>
+      <c r="A88" s="125" t="n"/>
       <c r="B88" s="126" t="inlineStr">
         <is>
-          <t>Interruptor diferencial 2P-25A-30mA (Protección personal)</t>
+          <t>Acometida a Tablero General TG-01 (Horizontal)</t>
         </is>
       </c>
       <c r="C88" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D88" s="127" t="n"/>
+      <c r="D88" s="127" t="n">
+        <v>6.6</v>
+      </c>
       <c r="E88" s="127" t="n"/>
       <c r="F88" s="127" t="n"/>
       <c r="G88" s="127">
-        <f>C88</f>
-        <v/>
-      </c>
-      <c r="H88" s="127">
-        <f>G88</f>
-        <v/>
-      </c>
-      <c r="I88" s="125" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+        <f>C88*D88</f>
+        <v/>
+      </c>
+      <c r="H88" s="127" t="n"/>
+      <c r="I88" s="125" t="n"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
-      <c r="A89" s="119" t="inlineStr">
-        <is>
-          <t>OE.5.4</t>
-        </is>
-      </c>
-      <c r="B89" s="120" t="inlineStr">
-        <is>
-          <t>INSTALACION DE PUESTA A TIERRA</t>
-        </is>
-      </c>
-      <c r="C89" s="121" t="n"/>
-      <c r="D89" s="121" t="n"/>
-      <c r="E89" s="121" t="n"/>
-      <c r="F89" s="121" t="n"/>
-      <c r="G89" s="121" t="n"/>
-      <c r="H89" s="121" t="n"/>
-      <c r="I89" s="119" t="n"/>
+      <c r="A89" s="125" t="n"/>
+      <c r="B89" s="126" t="inlineStr">
+        <is>
+          <t>Acometida a TG-01 (Vertical subida h = 1.40 m)</t>
+        </is>
+      </c>
+      <c r="C89" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" s="127" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E89" s="127" t="n"/>
+      <c r="F89" s="127" t="n"/>
+      <c r="G89" s="127">
+        <f>C89*D89</f>
+        <v/>
+      </c>
+      <c r="H89" s="127" t="n"/>
+      <c r="I89" s="125" t="n"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
-      <c r="A90" s="122" t="inlineStr">
-        <is>
-          <t>OE.5.4.1</t>
-        </is>
-      </c>
-      <c r="B90" s="123" t="inlineStr">
-        <is>
-          <t>PUESTA A TIERRA PAT-1</t>
-        </is>
-      </c>
-      <c r="C90" s="124" t="n"/>
-      <c r="D90" s="124" t="n"/>
-      <c r="E90" s="124" t="n"/>
-      <c r="F90" s="124" t="n"/>
-      <c r="G90" s="124" t="n"/>
-      <c r="H90" s="124" t="n"/>
-      <c r="I90" s="122" t="n"/>
+      <c r="A90" s="125" t="n"/>
+      <c r="B90" s="126" t="inlineStr">
+        <is>
+          <t>TG-01 a Tablero Distribución TD-01 (Horizontal)</t>
+        </is>
+      </c>
+      <c r="C90" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" s="127" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="E90" s="127" t="n"/>
+      <c r="F90" s="127" t="n"/>
+      <c r="G90" s="127">
+        <f>C90*D90</f>
+        <v/>
+      </c>
+      <c r="H90" s="127" t="n"/>
+      <c r="I90" s="125" t="n"/>
     </row>
     <row r="91" ht="15.75" customHeight="1">
-      <c r="A91" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.4.1.1</t>
-        </is>
-      </c>
+      <c r="A91" s="125" t="n"/>
       <c r="B91" s="126" t="inlineStr">
         <is>
-          <t>Varilla de cobre 5/8" x 2.40m, conector, caja registro, gel conductor y accesorios</t>
+          <t>TG-01 / TD-01 (Vertical subida h = 1.40 m)</t>
         </is>
       </c>
       <c r="C91" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D91" s="127" t="n"/>
+      <c r="D91" s="127" t="n">
+        <v>1.4</v>
+      </c>
       <c r="E91" s="127" t="n"/>
       <c r="F91" s="127" t="n"/>
       <c r="G91" s="127">
-        <f>C91</f>
-        <v/>
-      </c>
-      <c r="H91" s="127">
-        <f>G91</f>
-        <v/>
-      </c>
-      <c r="I91" s="125" t="inlineStr">
-        <is>
-          <t>jgo</t>
-        </is>
-      </c>
+        <f>C91*D91</f>
+        <v/>
+      </c>
+      <c r="H91" s="127" t="n"/>
+      <c r="I91" s="125" t="n"/>
     </row>
     <row r="92" ht="15.75" customHeight="1">
-      <c r="A92" s="119" t="inlineStr">
-        <is>
-          <t>OE.5.5</t>
-        </is>
-      </c>
-      <c r="B92" s="120" t="inlineStr">
-        <is>
-          <t>ARTEFACTOS DE ALUMBRADO</t>
-        </is>
-      </c>
-      <c r="C92" s="121" t="n"/>
-      <c r="D92" s="121" t="n"/>
-      <c r="E92" s="121" t="n"/>
-      <c r="F92" s="121" t="n"/>
-      <c r="G92" s="121" t="n"/>
-      <c r="H92" s="121" t="n"/>
-      <c r="I92" s="119" t="n"/>
+      <c r="A92" s="125" t="n"/>
+      <c r="B92" s="126" t="inlineStr">
+        <is>
+          <t>TD-01 a Tablero Distribución TD-02 (Horizontal)</t>
+        </is>
+      </c>
+      <c r="C92" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D92" s="127" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="E92" s="127" t="n"/>
+      <c r="F92" s="127" t="n"/>
+      <c r="G92" s="127">
+        <f>C92*D92</f>
+        <v/>
+      </c>
+      <c r="H92" s="127" t="n"/>
+      <c r="I92" s="125" t="n"/>
     </row>
     <row r="93" ht="15.75" customHeight="1">
-      <c r="A93" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.5.1</t>
-        </is>
-      </c>
+      <c r="A93" s="125" t="n"/>
       <c r="B93" s="126" t="inlineStr">
         <is>
-          <t>Luminaria LED interior de adosar 12 W (Iluminación general)</t>
+          <t>TD-01 / TD-02 (Vertical subida h = 1.40 m)</t>
         </is>
       </c>
       <c r="C93" s="127" t="n">
-        <v>19</v>
-      </c>
-      <c r="D93" s="127" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D93" s="127" t="n">
+        <v>1.4</v>
+      </c>
       <c r="E93" s="127" t="n"/>
       <c r="F93" s="127" t="n"/>
       <c r="G93" s="127">
-        <f>C93</f>
-        <v/>
-      </c>
-      <c r="H93" s="127">
-        <f>G93</f>
-        <v/>
-      </c>
-      <c r="I93" s="125" t="inlineStr">
+        <f>C93*D93</f>
+        <v/>
+      </c>
+      <c r="H93" s="127" t="n"/>
+      <c r="I93" s="125" t="n"/>
+    </row>
+    <row r="94" ht="15.75" customHeight="1">
+      <c r="A94" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.2.4</t>
+        </is>
+      </c>
+      <c r="B94" s="132" t="inlineStr">
+        <is>
+          <t>Curvas de PVC Pesada (PV-P) 3/4" (Accesorios Tomacorrientes)</t>
+        </is>
+      </c>
+      <c r="C94" s="133" t="n"/>
+      <c r="D94" s="133" t="n"/>
+      <c r="E94" s="133" t="n"/>
+      <c r="F94" s="133" t="n"/>
+      <c r="G94" s="133" t="n"/>
+      <c r="H94" s="133">
+        <f>SUM(G95,G97,G99)</f>
+        <v/>
+      </c>
+      <c r="I94" s="131" t="inlineStr">
         <is>
           <t>pza</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="15.75" customHeight="1">
-      <c r="A94" s="119" t="inlineStr">
+    <row r="95" ht="15.75" customHeight="1">
+      <c r="A95" s="131" t="n"/>
+      <c r="B95" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C95" s="133" t="n"/>
+      <c r="D95" s="133" t="n"/>
+      <c r="E95" s="133" t="n"/>
+      <c r="F95" s="133" t="n"/>
+      <c r="G95" s="133">
+        <f>SUM(C96:C96)</f>
+        <v/>
+      </c>
+      <c r="H95" s="133" t="n"/>
+      <c r="I95" s="131" t="n"/>
+    </row>
+    <row r="96" ht="15.75" customHeight="1">
+      <c r="A96" s="125" t="n"/>
+      <c r="B96" s="126" t="inlineStr">
+        <is>
+          <t>Curvas en subida a cajas de tomacorrientes</t>
+        </is>
+      </c>
+      <c r="C96" s="127" t="n">
+        <v>12</v>
+      </c>
+      <c r="D96" s="127" t="n"/>
+      <c r="E96" s="127" t="n"/>
+      <c r="F96" s="127" t="n"/>
+      <c r="G96" s="127">
+        <f>C96</f>
+        <v/>
+      </c>
+      <c r="H96" s="127" t="n"/>
+      <c r="I96" s="125" t="n"/>
+    </row>
+    <row r="97" ht="15.75" customHeight="1">
+      <c r="A97" s="131" t="n"/>
+      <c r="B97" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C97" s="133" t="n"/>
+      <c r="D97" s="133" t="n"/>
+      <c r="E97" s="133" t="n"/>
+      <c r="F97" s="133" t="n"/>
+      <c r="G97" s="133">
+        <f>SUM(C98:C98)</f>
+        <v/>
+      </c>
+      <c r="H97" s="133" t="n"/>
+      <c r="I97" s="131" t="n"/>
+    </row>
+    <row r="98" ht="15.75" customHeight="1">
+      <c r="A98" s="125" t="n"/>
+      <c r="B98" s="126" t="inlineStr">
+        <is>
+          <t>Curvas en subida a cajas de tomacorrientes</t>
+        </is>
+      </c>
+      <c r="C98" s="127" t="n">
+        <v>18</v>
+      </c>
+      <c r="D98" s="127" t="n"/>
+      <c r="E98" s="127" t="n"/>
+      <c r="F98" s="127" t="n"/>
+      <c r="G98" s="127">
+        <f>C98</f>
+        <v/>
+      </c>
+      <c r="H98" s="127" t="n"/>
+      <c r="I98" s="125" t="n"/>
+    </row>
+    <row r="99" ht="15.75" customHeight="1">
+      <c r="A99" s="131" t="n"/>
+      <c r="B99" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C99" s="133" t="n"/>
+      <c r="D99" s="133" t="n"/>
+      <c r="E99" s="133" t="n"/>
+      <c r="F99" s="133" t="n"/>
+      <c r="G99" s="133">
+        <f>SUM(C100:C100)</f>
+        <v/>
+      </c>
+      <c r="H99" s="133" t="n"/>
+      <c r="I99" s="131" t="n"/>
+    </row>
+    <row r="100" ht="15.75" customHeight="1">
+      <c r="A100" s="125" t="n"/>
+      <c r="B100" s="126" t="inlineStr">
+        <is>
+          <t>Curvas en subida a cajas de tomacorrientes</t>
+        </is>
+      </c>
+      <c r="C100" s="127" t="n">
+        <v>15</v>
+      </c>
+      <c r="D100" s="127" t="n"/>
+      <c r="E100" s="127" t="n"/>
+      <c r="F100" s="127" t="n"/>
+      <c r="G100" s="127">
+        <f>C100</f>
+        <v/>
+      </c>
+      <c r="H100" s="127" t="n"/>
+      <c r="I100" s="125" t="n"/>
+    </row>
+    <row r="101" ht="15.75" customHeight="1">
+      <c r="A101" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.2.5</t>
+        </is>
+      </c>
+      <c r="B101" s="132" t="inlineStr">
+        <is>
+          <t>Curvas de PVC Liviana (PV-L) 3/4" (Accesorios Alumbrado)</t>
+        </is>
+      </c>
+      <c r="C101" s="133" t="n"/>
+      <c r="D101" s="133" t="n"/>
+      <c r="E101" s="133" t="n"/>
+      <c r="F101" s="133" t="n"/>
+      <c r="G101" s="133" t="n"/>
+      <c r="H101" s="133">
+        <f>SUM(G102,G104,G106)</f>
+        <v/>
+      </c>
+      <c r="I101" s="131" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="15.75" customHeight="1">
+      <c r="A102" s="131" t="n"/>
+      <c r="B102" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C102" s="133" t="n"/>
+      <c r="D102" s="133" t="n"/>
+      <c r="E102" s="133" t="n"/>
+      <c r="F102" s="133" t="n"/>
+      <c r="G102" s="133">
+        <f>SUM(C103:C103)</f>
+        <v/>
+      </c>
+      <c r="H102" s="133" t="n"/>
+      <c r="I102" s="131" t="n"/>
+    </row>
+    <row r="103" ht="15.75" customHeight="1">
+      <c r="A103" s="125" t="n"/>
+      <c r="B103" s="126" t="inlineStr">
+        <is>
+          <t>Curvas en bajadas a cajas de interruptores</t>
+        </is>
+      </c>
+      <c r="C103" s="127" t="n">
+        <v>4</v>
+      </c>
+      <c r="D103" s="127" t="n"/>
+      <c r="E103" s="127" t="n"/>
+      <c r="F103" s="127" t="n"/>
+      <c r="G103" s="127">
+        <f>C103</f>
+        <v/>
+      </c>
+      <c r="H103" s="127" t="n"/>
+      <c r="I103" s="125" t="n"/>
+    </row>
+    <row r="104" ht="15.75" customHeight="1">
+      <c r="A104" s="131" t="n"/>
+      <c r="B104" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C104" s="133" t="n"/>
+      <c r="D104" s="133" t="n"/>
+      <c r="E104" s="133" t="n"/>
+      <c r="F104" s="133" t="n"/>
+      <c r="G104" s="133">
+        <f>SUM(C105:C105)</f>
+        <v/>
+      </c>
+      <c r="H104" s="133" t="n"/>
+      <c r="I104" s="131" t="n"/>
+    </row>
+    <row r="105" ht="15.75" customHeight="1">
+      <c r="A105" s="125" t="n"/>
+      <c r="B105" s="126" t="inlineStr">
+        <is>
+          <t>Curvas en bajadas a cajas de interruptores</t>
+        </is>
+      </c>
+      <c r="C105" s="127" t="n">
+        <v>4</v>
+      </c>
+      <c r="D105" s="127" t="n"/>
+      <c r="E105" s="127" t="n"/>
+      <c r="F105" s="127" t="n"/>
+      <c r="G105" s="127">
+        <f>C105</f>
+        <v/>
+      </c>
+      <c r="H105" s="127" t="n"/>
+      <c r="I105" s="125" t="n"/>
+    </row>
+    <row r="106" ht="15.75" customHeight="1">
+      <c r="A106" s="131" t="n"/>
+      <c r="B106" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C106" s="133" t="n"/>
+      <c r="D106" s="133" t="n"/>
+      <c r="E106" s="133" t="n"/>
+      <c r="F106" s="133" t="n"/>
+      <c r="G106" s="133">
+        <f>SUM(C107:C107)</f>
+        <v/>
+      </c>
+      <c r="H106" s="133" t="n"/>
+      <c r="I106" s="131" t="n"/>
+    </row>
+    <row r="107" ht="15.75" customHeight="1">
+      <c r="A107" s="125" t="n"/>
+      <c r="B107" s="126" t="inlineStr">
+        <is>
+          <t>Curvas en bajadas a cajas de interruptores</t>
+        </is>
+      </c>
+      <c r="C107" s="127" t="n">
+        <v>4</v>
+      </c>
+      <c r="D107" s="127" t="n"/>
+      <c r="E107" s="127" t="n"/>
+      <c r="F107" s="127" t="n"/>
+      <c r="G107" s="127">
+        <f>C107</f>
+        <v/>
+      </c>
+      <c r="H107" s="127" t="n"/>
+      <c r="I107" s="125" t="n"/>
+    </row>
+    <row r="108" ht="15.75" customHeight="1">
+      <c r="A108" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.2.6</t>
+        </is>
+      </c>
+      <c r="B108" s="126" t="inlineStr">
+        <is>
+          <t>Curva PVC Pesada (PV-P) 1" (Accesorios Alimentadores y tableros)</t>
+        </is>
+      </c>
+      <c r="C108" s="127" t="n">
+        <v>6</v>
+      </c>
+      <c r="D108" s="127" t="n"/>
+      <c r="E108" s="127" t="n"/>
+      <c r="F108" s="127" t="n"/>
+      <c r="G108" s="127">
+        <f>C108</f>
+        <v/>
+      </c>
+      <c r="H108" s="127">
+        <f>G108</f>
+        <v/>
+      </c>
+      <c r="I108" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="15.75" customHeight="1">
+      <c r="A109" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.2.7</t>
+        </is>
+      </c>
+      <c r="B109" s="126" t="inlineStr">
+        <is>
+          <t>Accesorios de canalización (Curvas, uniones, conectores, pegamento)</t>
+        </is>
+      </c>
+      <c r="C109" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D109" s="127" t="n"/>
+      <c r="E109" s="127" t="n"/>
+      <c r="F109" s="127" t="n"/>
+      <c r="G109" s="127">
+        <f>C109</f>
+        <v/>
+      </c>
+      <c r="H109" s="127">
+        <f>G109</f>
+        <v/>
+      </c>
+      <c r="I109" s="125" t="inlineStr">
+        <is>
+          <t>glb</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="15.75" customHeight="1">
+      <c r="A110" s="122" t="inlineStr">
+        <is>
+          <t>OE.5.2.3</t>
+        </is>
+      </c>
+      <c r="B110" s="123" t="inlineStr">
+        <is>
+          <t>CONDUCTORES Y CABLES</t>
+        </is>
+      </c>
+      <c r="C110" s="124" t="n"/>
+      <c r="D110" s="124" t="n"/>
+      <c r="E110" s="124" t="n"/>
+      <c r="F110" s="124" t="n"/>
+      <c r="G110" s="124" t="n"/>
+      <c r="H110" s="124" t="n"/>
+      <c r="I110" s="122" t="n"/>
+    </row>
+    <row r="111" ht="15.75" customHeight="1">
+      <c r="A111" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.3.1</t>
+        </is>
+      </c>
+      <c r="B111" s="132" t="inlineStr">
+        <is>
+          <t>Conductor de cobre LSOH 1.5 mm2 (Fase+Neutro Alumbrado)</t>
+        </is>
+      </c>
+      <c r="C111" s="133" t="n"/>
+      <c r="D111" s="133" t="n"/>
+      <c r="E111" s="133" t="n"/>
+      <c r="F111" s="133" t="n"/>
+      <c r="G111" s="133" t="n"/>
+      <c r="H111" s="133">
+        <f>SUM(G112,G114,G116)</f>
+        <v/>
+      </c>
+      <c r="I111" s="131" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="15.75" customHeight="1">
+      <c r="A112" s="131" t="n"/>
+      <c r="B112" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C112" s="133" t="n"/>
+      <c r="D112" s="133" t="n"/>
+      <c r="E112" s="133" t="n"/>
+      <c r="F112" s="133" t="n"/>
+      <c r="G112" s="133">
+        <f>SUM(G113:G113)</f>
+        <v/>
+      </c>
+      <c r="H112" s="133" t="n"/>
+      <c r="I112" s="131" t="n"/>
+    </row>
+    <row r="113" ht="15.75" customHeight="1">
+      <c r="A113" s="125" t="n"/>
+      <c r="B113" s="126" t="inlineStr">
+        <is>
+          <t>Circuito C1 (Alumbrado 1er Piso)</t>
+        </is>
+      </c>
+      <c r="C113" s="127" t="n">
+        <v>2</v>
+      </c>
+      <c r="D113" s="127" t="n">
+        <v>40</v>
+      </c>
+      <c r="E113" s="127" t="n"/>
+      <c r="F113" s="127" t="n"/>
+      <c r="G113" s="127">
+        <f>C113*D113</f>
+        <v/>
+      </c>
+      <c r="H113" s="127" t="n"/>
+      <c r="I113" s="125" t="n"/>
+    </row>
+    <row r="114" ht="15.75" customHeight="1">
+      <c r="A114" s="131" t="n"/>
+      <c r="B114" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C114" s="133" t="n"/>
+      <c r="D114" s="133" t="n"/>
+      <c r="E114" s="133" t="n"/>
+      <c r="F114" s="133" t="n"/>
+      <c r="G114" s="133">
+        <f>SUM(G115:G115)</f>
+        <v/>
+      </c>
+      <c r="H114" s="133" t="n"/>
+      <c r="I114" s="131" t="n"/>
+    </row>
+    <row r="115" ht="15.75" customHeight="1">
+      <c r="A115" s="125" t="n"/>
+      <c r="B115" s="126" t="inlineStr">
+        <is>
+          <t>Circuito C4 (Alumbrado 2do Piso)</t>
+        </is>
+      </c>
+      <c r="C115" s="127" t="n">
+        <v>2</v>
+      </c>
+      <c r="D115" s="127" t="n">
+        <v>40</v>
+      </c>
+      <c r="E115" s="127" t="n"/>
+      <c r="F115" s="127" t="n"/>
+      <c r="G115" s="127">
+        <f>C115*D115</f>
+        <v/>
+      </c>
+      <c r="H115" s="127" t="n"/>
+      <c r="I115" s="125" t="n"/>
+    </row>
+    <row r="116" ht="15.75" customHeight="1">
+      <c r="A116" s="131" t="n"/>
+      <c r="B116" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C116" s="133" t="n"/>
+      <c r="D116" s="133" t="n"/>
+      <c r="E116" s="133" t="n"/>
+      <c r="F116" s="133" t="n"/>
+      <c r="G116" s="133">
+        <f>SUM(G117:G117)</f>
+        <v/>
+      </c>
+      <c r="H116" s="133" t="n"/>
+      <c r="I116" s="131" t="n"/>
+    </row>
+    <row r="117" ht="15.75" customHeight="1">
+      <c r="A117" s="125" t="n"/>
+      <c r="B117" s="126" t="inlineStr">
+        <is>
+          <t>Circuito C6 (Alumbrado 3er Piso)</t>
+        </is>
+      </c>
+      <c r="C117" s="127" t="n">
+        <v>2</v>
+      </c>
+      <c r="D117" s="127" t="n">
+        <v>40</v>
+      </c>
+      <c r="E117" s="127" t="n"/>
+      <c r="F117" s="127" t="n"/>
+      <c r="G117" s="127">
+        <f>C117*D117</f>
+        <v/>
+      </c>
+      <c r="H117" s="127" t="n"/>
+      <c r="I117" s="125" t="n"/>
+    </row>
+    <row r="118" ht="15.75" customHeight="1">
+      <c r="A118" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.3.2</t>
+        </is>
+      </c>
+      <c r="B118" s="132" t="inlineStr">
+        <is>
+          <t>Conductor de cobre LSOH 1.5 mm2 (Protección a Tierra Alumbrado)</t>
+        </is>
+      </c>
+      <c r="C118" s="133" t="n"/>
+      <c r="D118" s="133" t="n"/>
+      <c r="E118" s="133" t="n"/>
+      <c r="F118" s="133" t="n"/>
+      <c r="G118" s="133" t="n"/>
+      <c r="H118" s="133">
+        <f>SUM(G119,G121,G123)</f>
+        <v/>
+      </c>
+      <c r="I118" s="131" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="15.75" customHeight="1">
+      <c r="A119" s="131" t="n"/>
+      <c r="B119" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C119" s="133" t="n"/>
+      <c r="D119" s="133" t="n"/>
+      <c r="E119" s="133" t="n"/>
+      <c r="F119" s="133" t="n"/>
+      <c r="G119" s="133">
+        <f>SUM(G120:G120)</f>
+        <v/>
+      </c>
+      <c r="H119" s="133" t="n"/>
+      <c r="I119" s="131" t="n"/>
+    </row>
+    <row r="120" ht="15.75" customHeight="1">
+      <c r="A120" s="125" t="n"/>
+      <c r="B120" s="126" t="inlineStr">
+        <is>
+          <t>Circuito C1 (Alumbrado 1er Piso)</t>
+        </is>
+      </c>
+      <c r="C120" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D120" s="127" t="n">
+        <v>35</v>
+      </c>
+      <c r="E120" s="127" t="n"/>
+      <c r="F120" s="127" t="n"/>
+      <c r="G120" s="127">
+        <f>C120*D120</f>
+        <v/>
+      </c>
+      <c r="H120" s="127" t="n"/>
+      <c r="I120" s="125" t="n"/>
+    </row>
+    <row r="121" ht="15.75" customHeight="1">
+      <c r="A121" s="131" t="n"/>
+      <c r="B121" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C121" s="133" t="n"/>
+      <c r="D121" s="133" t="n"/>
+      <c r="E121" s="133" t="n"/>
+      <c r="F121" s="133" t="n"/>
+      <c r="G121" s="133">
+        <f>SUM(G122:G122)</f>
+        <v/>
+      </c>
+      <c r="H121" s="133" t="n"/>
+      <c r="I121" s="131" t="n"/>
+    </row>
+    <row r="122" ht="15.75" customHeight="1">
+      <c r="A122" s="125" t="n"/>
+      <c r="B122" s="126" t="inlineStr">
+        <is>
+          <t>Circuito C4 (Alumbrado 2do Piso)</t>
+        </is>
+      </c>
+      <c r="C122" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D122" s="127" t="n">
+        <v>35</v>
+      </c>
+      <c r="E122" s="127" t="n"/>
+      <c r="F122" s="127" t="n"/>
+      <c r="G122" s="127">
+        <f>C122*D122</f>
+        <v/>
+      </c>
+      <c r="H122" s="127" t="n"/>
+      <c r="I122" s="125" t="n"/>
+    </row>
+    <row r="123" ht="15.75" customHeight="1">
+      <c r="A123" s="131" t="n"/>
+      <c r="B123" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C123" s="133" t="n"/>
+      <c r="D123" s="133" t="n"/>
+      <c r="E123" s="133" t="n"/>
+      <c r="F123" s="133" t="n"/>
+      <c r="G123" s="133">
+        <f>SUM(G124:G124)</f>
+        <v/>
+      </c>
+      <c r="H123" s="133" t="n"/>
+      <c r="I123" s="131" t="n"/>
+    </row>
+    <row r="124" ht="15.75" customHeight="1">
+      <c r="A124" s="125" t="n"/>
+      <c r="B124" s="126" t="inlineStr">
+        <is>
+          <t>Circuito C6 (Alumbrado 3er Piso)</t>
+        </is>
+      </c>
+      <c r="C124" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" s="127" t="n">
+        <v>40</v>
+      </c>
+      <c r="E124" s="127" t="n"/>
+      <c r="F124" s="127" t="n"/>
+      <c r="G124" s="127">
+        <f>C124*D124</f>
+        <v/>
+      </c>
+      <c r="H124" s="127" t="n"/>
+      <c r="I124" s="125" t="n"/>
+    </row>
+    <row r="125" ht="15.75" customHeight="1">
+      <c r="A125" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.3.3</t>
+        </is>
+      </c>
+      <c r="B125" s="132" t="inlineStr">
+        <is>
+          <t>Conductor de cobre LSOH 2.5 mm2 (Fase+Neutro Tomacorrientes)</t>
+        </is>
+      </c>
+      <c r="C125" s="133" t="n"/>
+      <c r="D125" s="133" t="n"/>
+      <c r="E125" s="133" t="n"/>
+      <c r="F125" s="133" t="n"/>
+      <c r="G125" s="133" t="n"/>
+      <c r="H125" s="133">
+        <f>SUM(G126,G128,G130)</f>
+        <v/>
+      </c>
+      <c r="I125" s="131" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="15.75" customHeight="1">
+      <c r="A126" s="131" t="n"/>
+      <c r="B126" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C126" s="133" t="n"/>
+      <c r="D126" s="133" t="n"/>
+      <c r="E126" s="133" t="n"/>
+      <c r="F126" s="133" t="n"/>
+      <c r="G126" s="133">
+        <f>SUM(G127:G127)</f>
+        <v/>
+      </c>
+      <c r="H126" s="133" t="n"/>
+      <c r="I126" s="131" t="n"/>
+    </row>
+    <row r="127" ht="15.75" customHeight="1">
+      <c r="A127" s="125" t="n"/>
+      <c r="B127" s="126" t="inlineStr">
+        <is>
+          <t>Circuito C2 (Tomacorrientes 1er Piso)</t>
+        </is>
+      </c>
+      <c r="C127" s="127" t="n">
+        <v>2</v>
+      </c>
+      <c r="D127" s="127" t="n">
+        <v>50</v>
+      </c>
+      <c r="E127" s="127" t="n"/>
+      <c r="F127" s="127" t="n"/>
+      <c r="G127" s="127">
+        <f>C127*D127</f>
+        <v/>
+      </c>
+      <c r="H127" s="127" t="n"/>
+      <c r="I127" s="125" t="n"/>
+    </row>
+    <row r="128" ht="15.75" customHeight="1">
+      <c r="A128" s="131" t="n"/>
+      <c r="B128" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C128" s="133" t="n"/>
+      <c r="D128" s="133" t="n"/>
+      <c r="E128" s="133" t="n"/>
+      <c r="F128" s="133" t="n"/>
+      <c r="G128" s="133">
+        <f>SUM(G129:G129)</f>
+        <v/>
+      </c>
+      <c r="H128" s="133" t="n"/>
+      <c r="I128" s="131" t="n"/>
+    </row>
+    <row r="129" ht="15.75" customHeight="1">
+      <c r="A129" s="125" t="n"/>
+      <c r="B129" s="126" t="inlineStr">
+        <is>
+          <t>Circuito C5 (Tomacorrientes 2do Piso)</t>
+        </is>
+      </c>
+      <c r="C129" s="127" t="n">
+        <v>2</v>
+      </c>
+      <c r="D129" s="127" t="n">
+        <v>55</v>
+      </c>
+      <c r="E129" s="127" t="n"/>
+      <c r="F129" s="127" t="n"/>
+      <c r="G129" s="127">
+        <f>C129*D129</f>
+        <v/>
+      </c>
+      <c r="H129" s="127" t="n"/>
+      <c r="I129" s="125" t="n"/>
+    </row>
+    <row r="130" ht="15.75" customHeight="1">
+      <c r="A130" s="131" t="n"/>
+      <c r="B130" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C130" s="133" t="n"/>
+      <c r="D130" s="133" t="n"/>
+      <c r="E130" s="133" t="n"/>
+      <c r="F130" s="133" t="n"/>
+      <c r="G130" s="133">
+        <f>SUM(G131:G131)</f>
+        <v/>
+      </c>
+      <c r="H130" s="133" t="n"/>
+      <c r="I130" s="131" t="n"/>
+    </row>
+    <row r="131" ht="15.75" customHeight="1">
+      <c r="A131" s="125" t="n"/>
+      <c r="B131" s="126" t="inlineStr">
+        <is>
+          <t>Circuito C7 (Tomacorrientes 3er Piso)</t>
+        </is>
+      </c>
+      <c r="C131" s="127" t="n">
+        <v>2</v>
+      </c>
+      <c r="D131" s="127" t="n">
+        <v>45</v>
+      </c>
+      <c r="E131" s="127" t="n"/>
+      <c r="F131" s="127" t="n"/>
+      <c r="G131" s="127">
+        <f>C131*D131</f>
+        <v/>
+      </c>
+      <c r="H131" s="127" t="n"/>
+      <c r="I131" s="125" t="n"/>
+    </row>
+    <row r="132" ht="15.75" customHeight="1">
+      <c r="A132" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.3.4</t>
+        </is>
+      </c>
+      <c r="B132" s="132" t="inlineStr">
+        <is>
+          <t>Conductor de cobre LSOH 2.5 mm2 (Protección a Tierra Tomacorrientes)</t>
+        </is>
+      </c>
+      <c r="C132" s="133" t="n"/>
+      <c r="D132" s="133" t="n"/>
+      <c r="E132" s="133" t="n"/>
+      <c r="F132" s="133" t="n"/>
+      <c r="G132" s="133" t="n"/>
+      <c r="H132" s="133">
+        <f>SUM(G133,G135,G137)</f>
+        <v/>
+      </c>
+      <c r="I132" s="131" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="15.75" customHeight="1">
+      <c r="A133" s="131" t="n"/>
+      <c r="B133" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C133" s="133" t="n"/>
+      <c r="D133" s="133" t="n"/>
+      <c r="E133" s="133" t="n"/>
+      <c r="F133" s="133" t="n"/>
+      <c r="G133" s="133">
+        <f>SUM(G134:G134)</f>
+        <v/>
+      </c>
+      <c r="H133" s="133" t="n"/>
+      <c r="I133" s="131" t="n"/>
+    </row>
+    <row r="134" ht="15.75" customHeight="1">
+      <c r="A134" s="125" t="n"/>
+      <c r="B134" s="126" t="inlineStr">
+        <is>
+          <t>Circuito C2 (Tomacorrientes 1er Piso)</t>
+        </is>
+      </c>
+      <c r="C134" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D134" s="127" t="n">
+        <v>50</v>
+      </c>
+      <c r="E134" s="127" t="n"/>
+      <c r="F134" s="127" t="n"/>
+      <c r="G134" s="127">
+        <f>C134*D134</f>
+        <v/>
+      </c>
+      <c r="H134" s="127" t="n"/>
+      <c r="I134" s="125" t="n"/>
+    </row>
+    <row r="135" ht="15.75" customHeight="1">
+      <c r="A135" s="131" t="n"/>
+      <c r="B135" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C135" s="133" t="n"/>
+      <c r="D135" s="133" t="n"/>
+      <c r="E135" s="133" t="n"/>
+      <c r="F135" s="133" t="n"/>
+      <c r="G135" s="133">
+        <f>SUM(G136:G136)</f>
+        <v/>
+      </c>
+      <c r="H135" s="133" t="n"/>
+      <c r="I135" s="131" t="n"/>
+    </row>
+    <row r="136" ht="15.75" customHeight="1">
+      <c r="A136" s="125" t="n"/>
+      <c r="B136" s="126" t="inlineStr">
+        <is>
+          <t>Circuito C5 (Tomacorrientes 2do Piso)</t>
+        </is>
+      </c>
+      <c r="C136" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D136" s="127" t="n">
+        <v>50</v>
+      </c>
+      <c r="E136" s="127" t="n"/>
+      <c r="F136" s="127" t="n"/>
+      <c r="G136" s="127">
+        <f>C136*D136</f>
+        <v/>
+      </c>
+      <c r="H136" s="127" t="n"/>
+      <c r="I136" s="125" t="n"/>
+    </row>
+    <row r="137" ht="15.75" customHeight="1">
+      <c r="A137" s="131" t="n"/>
+      <c r="B137" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C137" s="133" t="n"/>
+      <c r="D137" s="133" t="n"/>
+      <c r="E137" s="133" t="n"/>
+      <c r="F137" s="133" t="n"/>
+      <c r="G137" s="133">
+        <f>SUM(G138:G138)</f>
+        <v/>
+      </c>
+      <c r="H137" s="133" t="n"/>
+      <c r="I137" s="131" t="n"/>
+    </row>
+    <row r="138" ht="15.75" customHeight="1">
+      <c r="A138" s="125" t="n"/>
+      <c r="B138" s="126" t="inlineStr">
+        <is>
+          <t>Circuito C7 (Tomacorrientes 3er Piso)</t>
+        </is>
+      </c>
+      <c r="C138" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D138" s="127" t="n">
+        <v>50</v>
+      </c>
+      <c r="E138" s="127" t="n"/>
+      <c r="F138" s="127" t="n"/>
+      <c r="G138" s="127">
+        <f>C138*D138</f>
+        <v/>
+      </c>
+      <c r="H138" s="127" t="n"/>
+      <c r="I138" s="125" t="n"/>
+    </row>
+    <row r="139" ht="15.75" customHeight="1">
+      <c r="A139" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.3.5</t>
+        </is>
+      </c>
+      <c r="B139" s="126" t="inlineStr">
+        <is>
+          <t>Conductor de cobre LSOH 2.5 mm2 (Alimentación Electrobomba)</t>
+        </is>
+      </c>
+      <c r="C139" s="127" t="n">
+        <v>35</v>
+      </c>
+      <c r="D139" s="127" t="n"/>
+      <c r="E139" s="127" t="n"/>
+      <c r="F139" s="127" t="n"/>
+      <c r="G139" s="127">
+        <f>C139</f>
+        <v/>
+      </c>
+      <c r="H139" s="127">
+        <f>G139</f>
+        <v/>
+      </c>
+      <c r="I139" s="125" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="15.75" customHeight="1">
+      <c r="A140" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.3.6</t>
+        </is>
+      </c>
+      <c r="B140" s="126" t="inlineStr">
+        <is>
+          <t>Conductor de cobre LSOH 10 mm2 (Alimentador General)</t>
+        </is>
+      </c>
+      <c r="C140" s="127" t="n">
+        <v>60</v>
+      </c>
+      <c r="D140" s="127" t="n"/>
+      <c r="E140" s="127" t="n"/>
+      <c r="F140" s="127" t="n"/>
+      <c r="G140" s="127">
+        <f>C140</f>
+        <v/>
+      </c>
+      <c r="H140" s="127">
+        <f>G140</f>
+        <v/>
+      </c>
+      <c r="I140" s="125" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="15.75" customHeight="1">
+      <c r="A141" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.3.7</t>
+        </is>
+      </c>
+      <c r="B141" s="126" t="inlineStr">
+        <is>
+          <t>Conductor de cobre temple blando 6 mm2 (Conexión Puesta a Tierra)</t>
+        </is>
+      </c>
+      <c r="C141" s="127" t="n">
+        <v>25</v>
+      </c>
+      <c r="D141" s="127" t="n"/>
+      <c r="E141" s="127" t="n"/>
+      <c r="F141" s="127" t="n"/>
+      <c r="G141" s="127">
+        <f>C141</f>
+        <v/>
+      </c>
+      <c r="H141" s="127">
+        <f>G141</f>
+        <v/>
+      </c>
+      <c r="I141" s="125" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="15.75" customHeight="1">
+      <c r="A142" s="122" t="inlineStr">
+        <is>
+          <t>OE.5.2.4</t>
+        </is>
+      </c>
+      <c r="B142" s="123" t="inlineStr">
+        <is>
+          <t>CAJAS DE PASO Y DERIVACION</t>
+        </is>
+      </c>
+      <c r="C142" s="124" t="n"/>
+      <c r="D142" s="124" t="n"/>
+      <c r="E142" s="124" t="n"/>
+      <c r="F142" s="124" t="n"/>
+      <c r="G142" s="124" t="n"/>
+      <c r="H142" s="124" t="n"/>
+      <c r="I142" s="122" t="n"/>
+    </row>
+    <row r="143" ht="15.75" customHeight="1">
+      <c r="A143" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.4.1</t>
+        </is>
+      </c>
+      <c r="B143" s="126" t="inlineStr">
+        <is>
+          <t>Caja de pase rectangular 4"x2" FG (Derivaciones y cambios)</t>
+        </is>
+      </c>
+      <c r="C143" s="127" t="n">
+        <v>6</v>
+      </c>
+      <c r="D143" s="127" t="n"/>
+      <c r="E143" s="127" t="n"/>
+      <c r="F143" s="127" t="n"/>
+      <c r="G143" s="127">
+        <f>C143</f>
+        <v/>
+      </c>
+      <c r="H143" s="127">
+        <f>G143</f>
+        <v/>
+      </c>
+      <c r="I143" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="15.75" customHeight="1">
+      <c r="A144" s="122" t="inlineStr">
+        <is>
+          <t>OE.5.2.6</t>
+        </is>
+      </c>
+      <c r="B144" s="123" t="inlineStr">
+        <is>
+          <t>TABLEROS DE DISTRIBUCION Y DETALLES</t>
+        </is>
+      </c>
+      <c r="C144" s="124" t="n"/>
+      <c r="D144" s="124" t="n"/>
+      <c r="E144" s="124" t="n"/>
+      <c r="F144" s="124" t="n"/>
+      <c r="G144" s="124" t="n"/>
+      <c r="H144" s="124" t="n"/>
+      <c r="I144" s="122" t="n"/>
+    </row>
+    <row r="145" ht="15.75" customHeight="1">
+      <c r="A145" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.6.1</t>
+        </is>
+      </c>
+      <c r="B145" s="126" t="inlineStr">
+        <is>
+          <t>Tablero General TG-01 (12 polos, metálico empotrable, primer piso)</t>
+        </is>
+      </c>
+      <c r="C145" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D145" s="127" t="n"/>
+      <c r="E145" s="127" t="n"/>
+      <c r="F145" s="127" t="n"/>
+      <c r="G145" s="127">
+        <f>C145</f>
+        <v/>
+      </c>
+      <c r="H145" s="127">
+        <f>G145</f>
+        <v/>
+      </c>
+      <c r="I145" s="125" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="15.75" customHeight="1">
+      <c r="A146" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.6.2</t>
+        </is>
+      </c>
+      <c r="B146" s="126" t="inlineStr">
+        <is>
+          <t>Tablero de Distribución TD-01 (8 polos, metálico empotrable, segundo piso)</t>
+        </is>
+      </c>
+      <c r="C146" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D146" s="127" t="n"/>
+      <c r="E146" s="127" t="n"/>
+      <c r="F146" s="127" t="n"/>
+      <c r="G146" s="127">
+        <f>C146</f>
+        <v/>
+      </c>
+      <c r="H146" s="127">
+        <f>G146</f>
+        <v/>
+      </c>
+      <c r="I146" s="125" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="15.75" customHeight="1">
+      <c r="A147" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.6.3</t>
+        </is>
+      </c>
+      <c r="B147" s="126" t="inlineStr">
+        <is>
+          <t>Tablero de Distribución TD-02 (8 polos, metálico empotrable, tercer piso)</t>
+        </is>
+      </c>
+      <c r="C147" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D147" s="127" t="n"/>
+      <c r="E147" s="127" t="n"/>
+      <c r="F147" s="127" t="n"/>
+      <c r="G147" s="127">
+        <f>C147</f>
+        <v/>
+      </c>
+      <c r="H147" s="127">
+        <f>G147</f>
+        <v/>
+      </c>
+      <c r="I147" s="125" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="15.75" customHeight="1">
+      <c r="A148" s="122" t="inlineStr">
+        <is>
+          <t>OE.5.2.8</t>
+        </is>
+      </c>
+      <c r="B148" s="123" t="inlineStr">
+        <is>
+          <t>DISPOSITIVOS DE MANIOBRA Y PROTECCION</t>
+        </is>
+      </c>
+      <c r="C148" s="124" t="n"/>
+      <c r="D148" s="124" t="n"/>
+      <c r="E148" s="124" t="n"/>
+      <c r="F148" s="124" t="n"/>
+      <c r="G148" s="124" t="n"/>
+      <c r="H148" s="124" t="n"/>
+      <c r="I148" s="122" t="n"/>
+    </row>
+    <row r="149" ht="15.75" customHeight="1">
+      <c r="A149" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.8.1</t>
+        </is>
+      </c>
+      <c r="B149" s="126" t="inlineStr">
+        <is>
+          <t>Interruptor simple unipolar (adosar/empotrar, 10A)</t>
+        </is>
+      </c>
+      <c r="C149" s="127" t="n">
+        <v>6</v>
+      </c>
+      <c r="D149" s="127" t="n"/>
+      <c r="E149" s="127" t="n"/>
+      <c r="F149" s="127" t="n"/>
+      <c r="G149" s="127">
+        <f>C149</f>
+        <v/>
+      </c>
+      <c r="H149" s="127">
+        <f>G149</f>
+        <v/>
+      </c>
+      <c r="I149" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="15.75" customHeight="1">
+      <c r="A150" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.8.2</t>
+        </is>
+      </c>
+      <c r="B150" s="126" t="inlineStr">
+        <is>
+          <t>Interruptor de conmutación 3 vías (S3, escaleras)</t>
+        </is>
+      </c>
+      <c r="C150" s="127" t="n">
+        <v>4</v>
+      </c>
+      <c r="D150" s="127" t="n"/>
+      <c r="E150" s="127" t="n"/>
+      <c r="F150" s="127" t="n"/>
+      <c r="G150" s="127">
+        <f>C150</f>
+        <v/>
+      </c>
+      <c r="H150" s="127">
+        <f>G150</f>
+        <v/>
+      </c>
+      <c r="I150" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="15.75" customHeight="1">
+      <c r="A151" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.8.3</t>
+        </is>
+      </c>
+      <c r="B151" s="126" t="inlineStr">
+        <is>
+          <t>Interruptor termomagnetico 2P-10A (Alumbrado)</t>
+        </is>
+      </c>
+      <c r="C151" s="127" t="n">
+        <v>3</v>
+      </c>
+      <c r="D151" s="127" t="n"/>
+      <c r="E151" s="127" t="n"/>
+      <c r="F151" s="127" t="n"/>
+      <c r="G151" s="127">
+        <f>C151</f>
+        <v/>
+      </c>
+      <c r="H151" s="127">
+        <f>G151</f>
+        <v/>
+      </c>
+      <c r="I151" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="15.75" customHeight="1">
+      <c r="A152" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.8.4</t>
+        </is>
+      </c>
+      <c r="B152" s="126" t="inlineStr">
+        <is>
+          <t>Interruptor termomagnetico 2P-16A (Tomacorrientes)</t>
+        </is>
+      </c>
+      <c r="C152" s="127" t="n">
+        <v>5</v>
+      </c>
+      <c r="D152" s="127" t="n"/>
+      <c r="E152" s="127" t="n"/>
+      <c r="F152" s="127" t="n"/>
+      <c r="G152" s="127">
+        <f>C152</f>
+        <v/>
+      </c>
+      <c r="H152" s="127">
+        <f>G152</f>
+        <v/>
+      </c>
+      <c r="I152" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="15.75" customHeight="1">
+      <c r="A153" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.8.5</t>
+        </is>
+      </c>
+      <c r="B153" s="126" t="inlineStr">
+        <is>
+          <t>Interruptor termomagnetico 2P-20A (Cocina / Cargas especiales)</t>
+        </is>
+      </c>
+      <c r="C153" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D153" s="127" t="n"/>
+      <c r="E153" s="127" t="n"/>
+      <c r="F153" s="127" t="n"/>
+      <c r="G153" s="127">
+        <f>C153</f>
+        <v/>
+      </c>
+      <c r="H153" s="127">
+        <f>G153</f>
+        <v/>
+      </c>
+      <c r="I153" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="15.75" customHeight="1">
+      <c r="A154" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.8.6</t>
+        </is>
+      </c>
+      <c r="B154" s="126" t="inlineStr">
+        <is>
+          <t>Interruptor termomagnetico general 2P-40A (TG-01)</t>
+        </is>
+      </c>
+      <c r="C154" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D154" s="127" t="n"/>
+      <c r="E154" s="127" t="n"/>
+      <c r="F154" s="127" t="n"/>
+      <c r="G154" s="127">
+        <f>C154</f>
+        <v/>
+      </c>
+      <c r="H154" s="127">
+        <f>G154</f>
+        <v/>
+      </c>
+      <c r="I154" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="15.75" customHeight="1">
+      <c r="A155" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.8.7</t>
+        </is>
+      </c>
+      <c r="B155" s="126" t="inlineStr">
+        <is>
+          <t>Interruptor diferencial 2P-25A-30mA (Protección personal)</t>
+        </is>
+      </c>
+      <c r="C155" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D155" s="127" t="n"/>
+      <c r="E155" s="127" t="n"/>
+      <c r="F155" s="127" t="n"/>
+      <c r="G155" s="127">
+        <f>C155</f>
+        <v/>
+      </c>
+      <c r="H155" s="127">
+        <f>G155</f>
+        <v/>
+      </c>
+      <c r="I155" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="15.75" customHeight="1">
+      <c r="A156" s="119" t="inlineStr">
+        <is>
+          <t>OE.5.4</t>
+        </is>
+      </c>
+      <c r="B156" s="120" t="inlineStr">
+        <is>
+          <t>INSTALACION DE PUESTA A TIERRA</t>
+        </is>
+      </c>
+      <c r="C156" s="121" t="n"/>
+      <c r="D156" s="121" t="n"/>
+      <c r="E156" s="121" t="n"/>
+      <c r="F156" s="121" t="n"/>
+      <c r="G156" s="121" t="n"/>
+      <c r="H156" s="121" t="n"/>
+      <c r="I156" s="119" t="n"/>
+    </row>
+    <row r="157" ht="15.75" customHeight="1">
+      <c r="A157" s="122" t="inlineStr">
+        <is>
+          <t>OE.5.4.1</t>
+        </is>
+      </c>
+      <c r="B157" s="123" t="inlineStr">
+        <is>
+          <t>PUESTA A TIERRA PAT-1</t>
+        </is>
+      </c>
+      <c r="C157" s="124" t="n"/>
+      <c r="D157" s="124" t="n"/>
+      <c r="E157" s="124" t="n"/>
+      <c r="F157" s="124" t="n"/>
+      <c r="G157" s="124" t="n"/>
+      <c r="H157" s="124" t="n"/>
+      <c r="I157" s="122" t="n"/>
+    </row>
+    <row r="158" ht="15.75" customHeight="1">
+      <c r="A158" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.4.1.1</t>
+        </is>
+      </c>
+      <c r="B158" s="126" t="inlineStr">
+        <is>
+          <t>Varilla de cobre 5/8" x 2.40m, conector, caja registro, gel conductor y accesorios</t>
+        </is>
+      </c>
+      <c r="C158" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D158" s="127" t="n"/>
+      <c r="E158" s="127" t="n"/>
+      <c r="F158" s="127" t="n"/>
+      <c r="G158" s="127">
+        <f>C158</f>
+        <v/>
+      </c>
+      <c r="H158" s="127">
+        <f>G158</f>
+        <v/>
+      </c>
+      <c r="I158" s="125" t="inlineStr">
+        <is>
+          <t>jgo</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="15.75" customHeight="1">
+      <c r="A159" s="119" t="inlineStr">
+        <is>
+          <t>OE.5.5</t>
+        </is>
+      </c>
+      <c r="B159" s="120" t="inlineStr">
+        <is>
+          <t>ARTEFACTOS DE ALUMBRADO</t>
+        </is>
+      </c>
+      <c r="C159" s="121" t="n"/>
+      <c r="D159" s="121" t="n"/>
+      <c r="E159" s="121" t="n"/>
+      <c r="F159" s="121" t="n"/>
+      <c r="G159" s="121" t="n"/>
+      <c r="H159" s="121" t="n"/>
+      <c r="I159" s="119" t="n"/>
+    </row>
+    <row r="160" ht="15.75" customHeight="1">
+      <c r="A160" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.5.1</t>
+        </is>
+      </c>
+      <c r="B160" s="126" t="inlineStr">
+        <is>
+          <t>Luminaria LED interior de adosar 12 W (Iluminación general)</t>
+        </is>
+      </c>
+      <c r="C160" s="127" t="n">
+        <v>19</v>
+      </c>
+      <c r="D160" s="127" t="n"/>
+      <c r="E160" s="127" t="n"/>
+      <c r="F160" s="127" t="n"/>
+      <c r="G160" s="127">
+        <f>C160</f>
+        <v/>
+      </c>
+      <c r="H160" s="127">
+        <f>G160</f>
+        <v/>
+      </c>
+      <c r="I160" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="15.75" customHeight="1">
+      <c r="A161" s="119" t="inlineStr">
         <is>
           <t>OE.5.6</t>
         </is>
       </c>
-      <c r="B94" s="120" t="inlineStr">
+      <c r="B161" s="120" t="inlineStr">
         <is>
           <t>EQUIPOS ELECTRICOS Y MECANICOS</t>
         </is>
       </c>
-      <c r="C94" s="121" t="n"/>
-      <c r="D94" s="121" t="n"/>
-      <c r="E94" s="121" t="n"/>
-      <c r="F94" s="121" t="n"/>
-      <c r="G94" s="121" t="n"/>
-      <c r="H94" s="121" t="n"/>
-      <c r="I94" s="119" t="n"/>
-    </row>
-    <row r="95" ht="15.75" customHeight="1">
-      <c r="A95" s="125" t="inlineStr">
+      <c r="C161" s="121" t="n"/>
+      <c r="D161" s="121" t="n"/>
+      <c r="E161" s="121" t="n"/>
+      <c r="F161" s="121" t="n"/>
+      <c r="G161" s="121" t="n"/>
+      <c r="H161" s="121" t="n"/>
+      <c r="I161" s="119" t="n"/>
+    </row>
+    <row r="162" ht="15.75" customHeight="1">
+      <c r="A162" s="125" t="inlineStr">
         <is>
           <t>OE.5.6.1</t>
         </is>
       </c>
-      <c r="B95" s="126" t="inlineStr">
+      <c r="B162" s="126" t="inlineStr">
         <is>
           <t>Electrobomba monofásica de agua 1 HP, 220V, 60Hz</t>
         </is>
       </c>
-      <c r="C95" s="127" t="n">
+      <c r="C162" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D95" s="127" t="n"/>
-      <c r="E95" s="127" t="n"/>
-      <c r="F95" s="127" t="n"/>
-      <c r="G95" s="127">
-        <f>C95</f>
-        <v/>
-      </c>
-      <c r="H95" s="127">
-        <f>G95</f>
-        <v/>
-      </c>
-      <c r="I95" s="125" t="inlineStr">
+      <c r="D162" s="127" t="n"/>
+      <c r="E162" s="127" t="n"/>
+      <c r="F162" s="127" t="n"/>
+      <c r="G162" s="127">
+        <f>C162</f>
+        <v/>
+      </c>
+      <c r="H162" s="127">
+        <f>G162</f>
+        <v/>
+      </c>
+      <c r="I162" s="125" t="inlineStr">
         <is>
           <t>UND</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="15.75" customHeight="1">
-      <c r="A96" s="119" t="inlineStr">
+    <row r="163" ht="15.75" customHeight="1">
+      <c r="A163" s="119" t="inlineStr">
         <is>
           <t>OE.5.7</t>
         </is>
       </c>
-      <c r="B96" s="120" t="inlineStr">
+      <c r="B163" s="120" t="inlineStr">
         <is>
           <t>PRUEBAS ELECTRICAS</t>
         </is>
       </c>
-      <c r="C96" s="121" t="n"/>
-      <c r="D96" s="121" t="n"/>
-      <c r="E96" s="121" t="n"/>
-      <c r="F96" s="121" t="n"/>
-      <c r="G96" s="121" t="n"/>
-      <c r="H96" s="121" t="n"/>
-      <c r="I96" s="119" t="n"/>
-    </row>
-    <row r="97" ht="15.75" customHeight="1">
-      <c r="A97" s="125" t="inlineStr">
+      <c r="C163" s="121" t="n"/>
+      <c r="D163" s="121" t="n"/>
+      <c r="E163" s="121" t="n"/>
+      <c r="F163" s="121" t="n"/>
+      <c r="G163" s="121" t="n"/>
+      <c r="H163" s="121" t="n"/>
+      <c r="I163" s="119" t="n"/>
+    </row>
+    <row r="164" ht="15.75" customHeight="1">
+      <c r="A164" s="125" t="inlineStr">
         <is>
           <t>OE.5.7.1</t>
         </is>
       </c>
-      <c r="B97" s="126" t="inlineStr">
+      <c r="B164" s="126" t="inlineStr">
         <is>
           <t>Pruebas de aislamiento, continuidad de línea y resistencia de puesta a tierra</t>
         </is>
       </c>
-      <c r="C97" s="127" t="n">
+      <c r="C164" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D97" s="127" t="n"/>
-      <c r="E97" s="127" t="n"/>
-      <c r="F97" s="127" t="n"/>
-      <c r="G97" s="127">
-        <f>C97</f>
-        <v/>
-      </c>
-      <c r="H97" s="127">
-        <f>G97</f>
-        <v/>
-      </c>
-      <c r="I97" s="125" t="inlineStr">
+      <c r="D164" s="127" t="n"/>
+      <c r="E164" s="127" t="n"/>
+      <c r="F164" s="127" t="n"/>
+      <c r="G164" s="127">
+        <f>C164</f>
+        <v/>
+      </c>
+      <c r="H164" s="127">
+        <f>G164</f>
+        <v/>
+      </c>
+      <c r="I164" s="125" t="inlineStr">
         <is>
           <t>glb</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="12.75" customHeight="1"/>
-    <row r="99" ht="12.75" customHeight="1"/>
-    <row r="100" ht="12.75" customHeight="1"/>
-    <row r="101" ht="12.75" customHeight="1"/>
-    <row r="102" ht="12.75" customHeight="1"/>
-    <row r="103" ht="12.75" customHeight="1"/>
-    <row r="104" ht="12.75" customHeight="1"/>
-    <row r="105" ht="12.75" customHeight="1"/>
-    <row r="106" ht="12.75" customHeight="1"/>
-    <row r="107" ht="12.75" customHeight="1"/>
-    <row r="108" ht="12.75" customHeight="1"/>
-    <row r="109" ht="12.75" customHeight="1"/>
-    <row r="110" ht="12.75" customHeight="1"/>
-    <row r="111" ht="12.75" customHeight="1"/>
-    <row r="112" ht="12.75" customHeight="1"/>
-    <row r="113" ht="12.75" customHeight="1"/>
-    <row r="114" ht="12.75" customHeight="1"/>
-    <row r="115" ht="12.75" customHeight="1"/>
-    <row r="116" ht="12.75" customHeight="1"/>
-    <row r="117" ht="12.75" customHeight="1"/>
-    <row r="118" ht="12.75" customHeight="1"/>
-    <row r="119" ht="12.75" customHeight="1"/>
-    <row r="120" ht="12.75" customHeight="1"/>
-    <row r="121" ht="12.75" customHeight="1"/>
-    <row r="122" ht="12.75" customHeight="1"/>
-    <row r="123" ht="12.75" customHeight="1"/>
-    <row r="124" ht="12.75" customHeight="1"/>
-    <row r="125" ht="12.75" customHeight="1"/>
-    <row r="126" ht="12.75" customHeight="1"/>
-    <row r="127" ht="12.75" customHeight="1"/>
-    <row r="128" ht="12.75" customHeight="1"/>
-    <row r="129" ht="12.75" customHeight="1"/>
-    <row r="130" ht="12.75" customHeight="1"/>
-    <row r="131" ht="12.75" customHeight="1"/>
-    <row r="132" ht="12.75" customHeight="1"/>
-    <row r="133" ht="12.75" customHeight="1"/>
-    <row r="134" ht="12.75" customHeight="1"/>
-    <row r="135" ht="12.75" customHeight="1"/>
-    <row r="136" ht="12.75" customHeight="1"/>
-    <row r="137" ht="12.75" customHeight="1"/>
-    <row r="138" ht="12.75" customHeight="1"/>
-    <row r="139" ht="12.75" customHeight="1"/>
-    <row r="140" ht="12.75" customHeight="1"/>
-    <row r="141" ht="12.75" customHeight="1"/>
-    <row r="142" ht="12.75" customHeight="1"/>
-    <row r="143" ht="12.75" customHeight="1"/>
-    <row r="144" ht="12.75" customHeight="1"/>
-    <row r="145" ht="12.75" customHeight="1"/>
-    <row r="146" ht="12.75" customHeight="1"/>
-    <row r="147" ht="12.75" customHeight="1"/>
-    <row r="148" ht="12.75" customHeight="1"/>
-    <row r="149" ht="12.75" customHeight="1"/>
-    <row r="150" ht="12.75" customHeight="1"/>
-    <row r="151" ht="12.75" customHeight="1"/>
-    <row r="152" ht="12.75" customHeight="1"/>
-    <row r="153" ht="12.75" customHeight="1"/>
-    <row r="154" ht="12.75" customHeight="1"/>
-    <row r="155" ht="12.75" customHeight="1"/>
-    <row r="156" ht="12.75" customHeight="1"/>
-    <row r="157" ht="12.75" customHeight="1"/>
-    <row r="158" ht="12.75" customHeight="1"/>
-    <row r="159" ht="24" customHeight="1"/>
-    <row r="160" ht="12.75" customHeight="1"/>
-    <row r="161" ht="12.75" customHeight="1"/>
-    <row r="162" ht="12.75" customHeight="1"/>
-    <row r="163" ht="12.75" customHeight="1"/>
-    <row r="164" ht="12.75" customHeight="1"/>
     <row r="165" ht="12.75" customHeight="1"/>
     <row r="166" ht="12.75" customHeight="1"/>
     <row r="167" ht="12.75" customHeight="1"/>

</xml_diff>

<commit_message>
Sincronizar presupuesto y metrados en Excel, LaTeX y PDF
</commit_message>
<xml_diff>
--- a/proyecto_vivienda_unifamiliar_por_RENZO/metrados/metrados.xlsx
+++ b/proyecto_vivienda_unifamiliar_por_RENZO/metrados/metrados.xlsx
@@ -1098,7 +1098,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M164"/>
+  <dimension ref="A1:M171"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="15" customWidth="1" style="1" min="1" max="1"/>
@@ -1810,97 +1810,96 @@
       <c r="I36" s="125" t="n"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="128" t="inlineStr">
-        <is>
-          <t>OE.5.2.1.2</t>
-        </is>
-      </c>
-      <c r="B37" s="129" t="inlineStr">
-        <is>
-          <t>SALIDA PARA TOMACORRIENTES</t>
-        </is>
-      </c>
-      <c r="C37" s="130" t="n"/>
-      <c r="D37" s="130" t="n"/>
-      <c r="E37" s="130" t="n"/>
-      <c r="F37" s="130" t="n"/>
-      <c r="G37" s="130" t="n"/>
-      <c r="H37" s="130" t="n"/>
-      <c r="I37" s="128" t="n"/>
+      <c r="A37" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.1.1.2</t>
+        </is>
+      </c>
+      <c r="B37" s="132" t="inlineStr">
+        <is>
+          <t>CAJA RECTANGULAR FG 4"x2" - SALIDA PARA INTERRUPTORES</t>
+        </is>
+      </c>
+      <c r="C37" s="133" t="n"/>
+      <c r="D37" s="133" t="n"/>
+      <c r="E37" s="133" t="n"/>
+      <c r="F37" s="133" t="n"/>
+      <c r="G37" s="133" t="n"/>
+      <c r="H37" s="133">
+        <f>SUM(G38,G40,G42)</f>
+        <v/>
+      </c>
+      <c r="I37" s="131" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="131" t="inlineStr">
-        <is>
-          <t>OE.5.2.1.2.1</t>
-        </is>
-      </c>
+      <c r="A38" s="131" t="n"/>
       <c r="B38" s="132" t="inlineStr">
         <is>
-          <t>CAJA RECTANGULAR FG 4"x2" - SALIDA DE TOMACORRIENTE DOBLE CON TIERRA</t>
+          <t>PRIMER NIVEL</t>
         </is>
       </c>
       <c r="C38" s="133" t="n"/>
       <c r="D38" s="133" t="n"/>
       <c r="E38" s="133" t="n"/>
       <c r="F38" s="133" t="n"/>
-      <c r="G38" s="133" t="n"/>
-      <c r="H38" s="133">
-        <f>SUM(G39,G43,G47)</f>
-        <v/>
-      </c>
-      <c r="I38" s="131" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+      <c r="G38" s="133">
+        <f>SUM(C39:C39)</f>
+        <v/>
+      </c>
+      <c r="H38" s="133" t="n"/>
+      <c r="I38" s="131" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="131" t="n"/>
-      <c r="B39" s="132" t="inlineStr">
-        <is>
-          <t>PRIMER NIVEL</t>
-        </is>
-      </c>
-      <c r="C39" s="133" t="n"/>
-      <c r="D39" s="133" t="n"/>
-      <c r="E39" s="133" t="n"/>
-      <c r="F39" s="133" t="n"/>
-      <c r="G39" s="133">
-        <f>SUM(C40:C42)</f>
-        <v/>
-      </c>
-      <c r="H39" s="133" t="n"/>
-      <c r="I39" s="131" t="n"/>
+      <c r="A39" s="125" t="n"/>
+      <c r="B39" s="126" t="inlineStr">
+        <is>
+          <t>Interruptores Simples y de Conmutacion</t>
+        </is>
+      </c>
+      <c r="C39" s="127" t="n">
+        <v>4</v>
+      </c>
+      <c r="D39" s="127" t="n"/>
+      <c r="E39" s="127" t="n"/>
+      <c r="F39" s="127" t="n"/>
+      <c r="G39" s="127">
+        <f>C39</f>
+        <v/>
+      </c>
+      <c r="H39" s="127" t="n"/>
+      <c r="I39" s="125" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="125" t="n"/>
-      <c r="B40" s="126" t="inlineStr">
-        <is>
-          <t>Tienda (Ambiente Frontal)</t>
-        </is>
-      </c>
-      <c r="C40" s="127" t="n">
-        <v>4</v>
-      </c>
-      <c r="D40" s="127" t="n"/>
-      <c r="E40" s="127" t="n"/>
-      <c r="F40" s="127" t="n"/>
-      <c r="G40" s="127">
-        <f>C40</f>
-        <v/>
-      </c>
-      <c r="H40" s="127" t="n"/>
-      <c r="I40" s="125" t="n"/>
+      <c r="A40" s="131" t="n"/>
+      <c r="B40" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C40" s="133" t="n"/>
+      <c r="D40" s="133" t="n"/>
+      <c r="E40" s="133" t="n"/>
+      <c r="F40" s="133" t="n"/>
+      <c r="G40" s="133">
+        <f>SUM(C41:C41)</f>
+        <v/>
+      </c>
+      <c r="H40" s="133" t="n"/>
+      <c r="I40" s="131" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="125" t="n"/>
       <c r="B41" s="126" t="inlineStr">
         <is>
-          <t>Cocina (Uso General)</t>
+          <t>Interruptores Simples y de Conmutacion</t>
         </is>
       </c>
       <c r="C41" s="127" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D41" s="127" t="n"/>
       <c r="E41" s="127" t="n"/>
@@ -1913,130 +1912,135 @@
       <c r="I41" s="125" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="125" t="n"/>
-      <c r="B42" s="126" t="inlineStr">
-        <is>
-          <t>Pasadizo de Acceso</t>
-        </is>
-      </c>
-      <c r="C42" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="127" t="n"/>
-      <c r="E42" s="127" t="n"/>
-      <c r="F42" s="127" t="n"/>
-      <c r="G42" s="127">
-        <f>C42</f>
-        <v/>
-      </c>
-      <c r="H42" s="127" t="n"/>
-      <c r="I42" s="125" t="n"/>
+      <c r="A42" s="131" t="n"/>
+      <c r="B42" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C42" s="133" t="n"/>
+      <c r="D42" s="133" t="n"/>
+      <c r="E42" s="133" t="n"/>
+      <c r="F42" s="133" t="n"/>
+      <c r="G42" s="133">
+        <f>SUM(C43:C43)</f>
+        <v/>
+      </c>
+      <c r="H42" s="133" t="n"/>
+      <c r="I42" s="131" t="n"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="131" t="n"/>
-      <c r="B43" s="132" t="inlineStr">
-        <is>
-          <t>SEGUNDO NIVEL</t>
-        </is>
-      </c>
-      <c r="C43" s="133" t="n"/>
-      <c r="D43" s="133" t="n"/>
-      <c r="E43" s="133" t="n"/>
-      <c r="F43" s="133" t="n"/>
-      <c r="G43" s="133">
-        <f>SUM(C44:C46)</f>
-        <v/>
-      </c>
-      <c r="H43" s="133" t="n"/>
-      <c r="I43" s="131" t="n"/>
+      <c r="A43" s="125" t="n"/>
+      <c r="B43" s="126" t="inlineStr">
+        <is>
+          <t>Interruptores Simples y de Conmutacion</t>
+        </is>
+      </c>
+      <c r="C43" s="127" t="n">
+        <v>3</v>
+      </c>
+      <c r="D43" s="127" t="n"/>
+      <c r="E43" s="127" t="n"/>
+      <c r="F43" s="127" t="n"/>
+      <c r="G43" s="127">
+        <f>C43</f>
+        <v/>
+      </c>
+      <c r="H43" s="127" t="n"/>
+      <c r="I43" s="125" t="n"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="125" t="n"/>
-      <c r="B44" s="126" t="inlineStr">
-        <is>
-          <t>Dormitorio Principal</t>
-        </is>
-      </c>
-      <c r="C44" s="127" t="n">
+      <c r="A44" s="128" t="inlineStr">
+        <is>
+          <t>OE.5.2.1.2</t>
+        </is>
+      </c>
+      <c r="B44" s="129" t="inlineStr">
+        <is>
+          <t>SALIDA PARA TOMACORRIENTES</t>
+        </is>
+      </c>
+      <c r="C44" s="130" t="n"/>
+      <c r="D44" s="130" t="n"/>
+      <c r="E44" s="130" t="n"/>
+      <c r="F44" s="130" t="n"/>
+      <c r="G44" s="130" t="n"/>
+      <c r="H44" s="130" t="n"/>
+      <c r="I44" s="128" t="n"/>
+    </row>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="A45" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.1.2.1</t>
+        </is>
+      </c>
+      <c r="B45" s="132" t="inlineStr">
+        <is>
+          <t>CAJA RECTANGULAR FG 4"x2" - SALIDA DE TOMACORRIENTE DOBLE CON TIERRA</t>
+        </is>
+      </c>
+      <c r="C45" s="133" t="n"/>
+      <c r="D45" s="133" t="n"/>
+      <c r="E45" s="133" t="n"/>
+      <c r="F45" s="133" t="n"/>
+      <c r="G45" s="133" t="n"/>
+      <c r="H45" s="133">
+        <f>SUM(G46,G50,G54)</f>
+        <v/>
+      </c>
+      <c r="I45" s="131" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="131" t="n"/>
+      <c r="B46" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C46" s="133" t="n"/>
+      <c r="D46" s="133" t="n"/>
+      <c r="E46" s="133" t="n"/>
+      <c r="F46" s="133" t="n"/>
+      <c r="G46" s="133">
+        <f>SUM(C47:C49)</f>
+        <v/>
+      </c>
+      <c r="H46" s="133" t="n"/>
+      <c r="I46" s="131" t="n"/>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="A47" s="125" t="n"/>
+      <c r="B47" s="126" t="inlineStr">
+        <is>
+          <t>Tienda (Ambiente Frontal)</t>
+        </is>
+      </c>
+      <c r="C47" s="127" t="n">
         <v>4</v>
       </c>
-      <c r="D44" s="127" t="n"/>
-      <c r="E44" s="127" t="n"/>
-      <c r="F44" s="127" t="n"/>
-      <c r="G44" s="127">
-        <f>C44</f>
-        <v/>
-      </c>
-      <c r="H44" s="127" t="n"/>
-      <c r="I44" s="125" t="n"/>
-    </row>
-    <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="125" t="n"/>
-      <c r="B45" s="126" t="inlineStr">
-        <is>
-          <t>Dormitorio 3</t>
-        </is>
-      </c>
-      <c r="C45" s="127" t="n">
-        <v>2</v>
-      </c>
-      <c r="D45" s="127" t="n"/>
-      <c r="E45" s="127" t="n"/>
-      <c r="F45" s="127" t="n"/>
-      <c r="G45" s="127">
-        <f>C45</f>
-        <v/>
-      </c>
-      <c r="H45" s="127" t="n"/>
-      <c r="I45" s="125" t="n"/>
-    </row>
-    <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="125" t="n"/>
-      <c r="B46" s="126" t="inlineStr">
-        <is>
-          <t>Sala / Hall Común</t>
-        </is>
-      </c>
-      <c r="C46" s="127" t="n">
-        <v>2</v>
-      </c>
-      <c r="D46" s="127" t="n"/>
-      <c r="E46" s="127" t="n"/>
-      <c r="F46" s="127" t="n"/>
-      <c r="G46" s="127">
-        <f>C46</f>
-        <v/>
-      </c>
-      <c r="H46" s="127" t="n"/>
-      <c r="I46" s="125" t="n"/>
-    </row>
-    <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="131" t="n"/>
-      <c r="B47" s="132" t="inlineStr">
-        <is>
-          <t>TERCER NIVEL</t>
-        </is>
-      </c>
-      <c r="C47" s="133" t="n"/>
-      <c r="D47" s="133" t="n"/>
-      <c r="E47" s="133" t="n"/>
-      <c r="F47" s="133" t="n"/>
-      <c r="G47" s="133">
-        <f>SUM(C48:C50)</f>
-        <v/>
-      </c>
-      <c r="H47" s="133" t="n"/>
-      <c r="I47" s="131" t="n"/>
+      <c r="D47" s="127" t="n"/>
+      <c r="E47" s="127" t="n"/>
+      <c r="F47" s="127" t="n"/>
+      <c r="G47" s="127">
+        <f>C47</f>
+        <v/>
+      </c>
+      <c r="H47" s="127" t="n"/>
+      <c r="I47" s="125" t="n"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="125" t="n"/>
       <c r="B48" s="126" t="inlineStr">
         <is>
-          <t>Dormitorio 4</t>
+          <t>Cocina (Uso General)</t>
         </is>
       </c>
       <c r="C48" s="127" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D48" s="127" t="n"/>
       <c r="E48" s="127" t="n"/>
@@ -2052,11 +2056,11 @@
       <c r="A49" s="125" t="n"/>
       <c r="B49" s="126" t="inlineStr">
         <is>
-          <t>Dormitorio 5</t>
+          <t>Pasadizo de Acceso</t>
         </is>
       </c>
       <c r="C49" s="127" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D49" s="127" t="n"/>
       <c r="E49" s="127" t="n"/>
@@ -2069,78 +2073,72 @@
       <c r="I49" s="125" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="125" t="n"/>
-      <c r="B50" s="126" t="inlineStr">
-        <is>
-          <t>Pasadizo / Vestíbulo</t>
-        </is>
-      </c>
-      <c r="C50" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="127" t="n"/>
-      <c r="E50" s="127" t="n"/>
-      <c r="F50" s="127" t="n"/>
-      <c r="G50" s="127">
-        <f>C50</f>
-        <v/>
-      </c>
-      <c r="H50" s="127" t="n"/>
-      <c r="I50" s="125" t="n"/>
+      <c r="A50" s="131" t="n"/>
+      <c r="B50" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C50" s="133" t="n"/>
+      <c r="D50" s="133" t="n"/>
+      <c r="E50" s="133" t="n"/>
+      <c r="F50" s="133" t="n"/>
+      <c r="G50" s="133">
+        <f>SUM(C51:C53)</f>
+        <v/>
+      </c>
+      <c r="H50" s="133" t="n"/>
+      <c r="I50" s="131" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="131" t="inlineStr">
-        <is>
-          <t>OE.5.2.1.2.2</t>
-        </is>
-      </c>
-      <c r="B51" s="132" t="inlineStr">
-        <is>
-          <t>CAJA RECTANGULAR FG 4"x2" - SALIDA DE TOMACORRIENTE DOBLE CON PROTECCION GFCI</t>
-        </is>
-      </c>
-      <c r="C51" s="133" t="n"/>
-      <c r="D51" s="133" t="n"/>
-      <c r="E51" s="133" t="n"/>
-      <c r="F51" s="133" t="n"/>
-      <c r="G51" s="133" t="n"/>
-      <c r="H51" s="133">
-        <f>SUM(G52,G54)</f>
-        <v/>
-      </c>
-      <c r="I51" s="131" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+      <c r="A51" s="125" t="n"/>
+      <c r="B51" s="126" t="inlineStr">
+        <is>
+          <t>Dormitorio Principal</t>
+        </is>
+      </c>
+      <c r="C51" s="127" t="n">
+        <v>4</v>
+      </c>
+      <c r="D51" s="127" t="n"/>
+      <c r="E51" s="127" t="n"/>
+      <c r="F51" s="127" t="n"/>
+      <c r="G51" s="127">
+        <f>C51</f>
+        <v/>
+      </c>
+      <c r="H51" s="127" t="n"/>
+      <c r="I51" s="125" t="n"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="131" t="n"/>
-      <c r="B52" s="132" t="inlineStr">
-        <is>
-          <t>SEGUNDO NIVEL</t>
-        </is>
-      </c>
-      <c r="C52" s="133" t="n"/>
-      <c r="D52" s="133" t="n"/>
-      <c r="E52" s="133" t="n"/>
-      <c r="F52" s="133" t="n"/>
-      <c r="G52" s="133">
-        <f>SUM(C53:C53)</f>
-        <v/>
-      </c>
-      <c r="H52" s="133" t="n"/>
-      <c r="I52" s="131" t="n"/>
+      <c r="A52" s="125" t="n"/>
+      <c r="B52" s="126" t="inlineStr">
+        <is>
+          <t>Dormitorio 3</t>
+        </is>
+      </c>
+      <c r="C52" s="127" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" s="127" t="n"/>
+      <c r="E52" s="127" t="n"/>
+      <c r="F52" s="127" t="n"/>
+      <c r="G52" s="127">
+        <f>C52</f>
+        <v/>
+      </c>
+      <c r="H52" s="127" t="n"/>
+      <c r="I52" s="125" t="n"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="125" t="n"/>
       <c r="B53" s="126" t="inlineStr">
         <is>
-          <t>Baño Completo</t>
+          <t>Sala / Hall Común</t>
         </is>
       </c>
       <c r="C53" s="127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D53" s="127" t="n"/>
       <c r="E53" s="127" t="n"/>
@@ -2164,7 +2162,7 @@
       <c r="E54" s="133" t="n"/>
       <c r="F54" s="133" t="n"/>
       <c r="G54" s="133">
-        <f>SUM(C55:C55)</f>
+        <f>SUM(C55:C57)</f>
         <v/>
       </c>
       <c r="H54" s="133" t="n"/>
@@ -2174,11 +2172,11 @@
       <c r="A55" s="125" t="n"/>
       <c r="B55" s="126" t="inlineStr">
         <is>
-          <t>Baño / Lavandería</t>
+          <t>Dormitorio 4</t>
         </is>
       </c>
       <c r="C55" s="127" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D55" s="127" t="n"/>
       <c r="E55" s="127" t="n"/>
@@ -2191,155 +2189,156 @@
       <c r="I55" s="125" t="n"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="131" t="inlineStr">
-        <is>
-          <t>OE.5.2.1.2.3</t>
-        </is>
-      </c>
-      <c r="B56" s="132" t="inlineStr">
-        <is>
-          <t>CAJA RECTANGULAR FG 4"x2" - SALIDA DE TOMACORRIENTE SERVICIO PESADO 20A</t>
-        </is>
-      </c>
-      <c r="C56" s="133" t="n"/>
-      <c r="D56" s="133" t="n"/>
-      <c r="E56" s="133" t="n"/>
-      <c r="F56" s="133" t="n"/>
-      <c r="G56" s="133" t="n"/>
-      <c r="H56" s="133">
-        <f>SUM(G57,G60)</f>
-        <v/>
-      </c>
-      <c r="I56" s="131" t="inlineStr">
+      <c r="A56" s="125" t="n"/>
+      <c r="B56" s="126" t="inlineStr">
+        <is>
+          <t>Dormitorio 5</t>
+        </is>
+      </c>
+      <c r="C56" s="127" t="n">
+        <v>3</v>
+      </c>
+      <c r="D56" s="127" t="n"/>
+      <c r="E56" s="127" t="n"/>
+      <c r="F56" s="127" t="n"/>
+      <c r="G56" s="127">
+        <f>C56</f>
+        <v/>
+      </c>
+      <c r="H56" s="127" t="n"/>
+      <c r="I56" s="125" t="n"/>
+    </row>
+    <row r="57" ht="15.75" customHeight="1">
+      <c r="A57" s="125" t="n"/>
+      <c r="B57" s="126" t="inlineStr">
+        <is>
+          <t>Pasadizo / Vestíbulo</t>
+        </is>
+      </c>
+      <c r="C57" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" s="127" t="n"/>
+      <c r="E57" s="127" t="n"/>
+      <c r="F57" s="127" t="n"/>
+      <c r="G57" s="127">
+        <f>C57</f>
+        <v/>
+      </c>
+      <c r="H57" s="127" t="n"/>
+      <c r="I57" s="125" t="n"/>
+    </row>
+    <row r="58" ht="15.75" customHeight="1">
+      <c r="A58" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.1.2.2</t>
+        </is>
+      </c>
+      <c r="B58" s="132" t="inlineStr">
+        <is>
+          <t>CAJA RECTANGULAR FG 4"x2" - SALIDA DE TOMACORRIENTE DOBLE CON PROTECCION GFCI</t>
+        </is>
+      </c>
+      <c r="C58" s="133" t="n"/>
+      <c r="D58" s="133" t="n"/>
+      <c r="E58" s="133" t="n"/>
+      <c r="F58" s="133" t="n"/>
+      <c r="G58" s="133" t="n"/>
+      <c r="H58" s="133">
+        <f>SUM(G59,G61)</f>
+        <v/>
+      </c>
+      <c r="I58" s="131" t="inlineStr">
         <is>
           <t>pza</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="131" t="n"/>
-      <c r="B57" s="132" t="inlineStr">
-        <is>
-          <t>PRIMER NIVEL</t>
-        </is>
-      </c>
-      <c r="C57" s="133" t="n"/>
-      <c r="D57" s="133" t="n"/>
-      <c r="E57" s="133" t="n"/>
-      <c r="F57" s="133" t="n"/>
-      <c r="G57" s="133">
-        <f>SUM(C58:C59)</f>
-        <v/>
-      </c>
-      <c r="H57" s="133" t="n"/>
-      <c r="I57" s="131" t="n"/>
-    </row>
-    <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="125" t="n"/>
-      <c r="B58" s="126" t="inlineStr">
-        <is>
-          <t>Cocina (Microondas / Cocina Eléctrica)</t>
-        </is>
-      </c>
-      <c r="C58" s="127" t="n">
+    <row r="59" ht="15.75" customHeight="1">
+      <c r="A59" s="131" t="n"/>
+      <c r="B59" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C59" s="133" t="n"/>
+      <c r="D59" s="133" t="n"/>
+      <c r="E59" s="133" t="n"/>
+      <c r="F59" s="133" t="n"/>
+      <c r="G59" s="133">
+        <f>SUM(C60:C60)</f>
+        <v/>
+      </c>
+      <c r="H59" s="133" t="n"/>
+      <c r="I59" s="131" t="n"/>
+    </row>
+    <row r="60" ht="15.75" customHeight="1">
+      <c r="A60" s="125" t="n"/>
+      <c r="B60" s="126" t="inlineStr">
+        <is>
+          <t>Baño Completo</t>
+        </is>
+      </c>
+      <c r="C60" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D58" s="127" t="n"/>
-      <c r="E58" s="127" t="n"/>
-      <c r="F58" s="127" t="n"/>
-      <c r="G58" s="127">
-        <f>C58</f>
-        <v/>
-      </c>
-      <c r="H58" s="127" t="n"/>
-      <c r="I58" s="125" t="n"/>
-    </row>
-    <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="125" t="n"/>
-      <c r="B59" s="126" t="inlineStr">
-        <is>
-          <t>Bomba de Agua (Servicio)</t>
-        </is>
-      </c>
-      <c r="C59" s="127" t="n">
+      <c r="D60" s="127" t="n"/>
+      <c r="E60" s="127" t="n"/>
+      <c r="F60" s="127" t="n"/>
+      <c r="G60" s="127">
+        <f>C60</f>
+        <v/>
+      </c>
+      <c r="H60" s="127" t="n"/>
+      <c r="I60" s="125" t="n"/>
+    </row>
+    <row r="61" ht="15.75" customHeight="1">
+      <c r="A61" s="131" t="n"/>
+      <c r="B61" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C61" s="133" t="n"/>
+      <c r="D61" s="133" t="n"/>
+      <c r="E61" s="133" t="n"/>
+      <c r="F61" s="133" t="n"/>
+      <c r="G61" s="133">
+        <f>SUM(C62:C62)</f>
+        <v/>
+      </c>
+      <c r="H61" s="133" t="n"/>
+      <c r="I61" s="131" t="n"/>
+    </row>
+    <row r="62" ht="15.75" customHeight="1">
+      <c r="A62" s="125" t="n"/>
+      <c r="B62" s="126" t="inlineStr">
+        <is>
+          <t>Baño / Lavandería</t>
+        </is>
+      </c>
+      <c r="C62" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D59" s="127" t="n"/>
-      <c r="E59" s="127" t="n"/>
-      <c r="F59" s="127" t="n"/>
-      <c r="G59" s="127">
-        <f>C59</f>
-        <v/>
-      </c>
-      <c r="H59" s="127" t="n"/>
-      <c r="I59" s="125" t="n"/>
-    </row>
-    <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="131" t="n"/>
-      <c r="B60" s="132" t="inlineStr">
-        <is>
-          <t>TERCER NIVEL</t>
-        </is>
-      </c>
-      <c r="C60" s="133" t="n"/>
-      <c r="D60" s="133" t="n"/>
-      <c r="E60" s="133" t="n"/>
-      <c r="F60" s="133" t="n"/>
-      <c r="G60" s="133">
-        <f>SUM(C61:C61)</f>
-        <v/>
-      </c>
-      <c r="H60" s="133" t="n"/>
-      <c r="I60" s="131" t="n"/>
-    </row>
-    <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="125" t="n"/>
-      <c r="B61" s="126" t="inlineStr">
-        <is>
-          <t>Lavandería (Lavadora)</t>
-        </is>
-      </c>
-      <c r="C61" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="127" t="n"/>
-      <c r="E61" s="127" t="n"/>
-      <c r="F61" s="127" t="n"/>
-      <c r="G61" s="127">
-        <f>C61</f>
-        <v/>
-      </c>
-      <c r="H61" s="127" t="n"/>
-      <c r="I61" s="125" t="n"/>
-    </row>
-    <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="122" t="inlineStr">
-        <is>
-          <t>OE.5.2.2</t>
-        </is>
-      </c>
-      <c r="B62" s="123" t="inlineStr">
-        <is>
-          <t>CANALIZACIONES, TUBERIAS Y CONDUCTOS</t>
-        </is>
-      </c>
-      <c r="C62" s="124" t="n"/>
-      <c r="D62" s="124" t="n"/>
-      <c r="E62" s="124" t="n"/>
-      <c r="F62" s="124" t="n"/>
-      <c r="G62" s="124" t="n"/>
-      <c r="H62" s="124" t="n"/>
-      <c r="I62" s="122" t="n"/>
+      <c r="D62" s="127" t="n"/>
+      <c r="E62" s="127" t="n"/>
+      <c r="F62" s="127" t="n"/>
+      <c r="G62" s="127">
+        <f>C62</f>
+        <v/>
+      </c>
+      <c r="H62" s="127" t="n"/>
+      <c r="I62" s="125" t="n"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="131" t="inlineStr">
         <is>
-          <t>OE.5.2.2.1</t>
+          <t>OE.5.2.1.2.3</t>
         </is>
       </c>
       <c r="B63" s="132" t="inlineStr">
         <is>
-          <t>Tubería PVC Liviana (PV-L) 3/4" (Canalización Alumbrado)</t>
+          <t>CAJA RECTANGULAR FG 4"x2" - SALIDA DE TOMACORRIENTE SERVICIO PESADO 20A</t>
         </is>
       </c>
       <c r="C63" s="133" t="n"/>
@@ -2348,12 +2347,12 @@
       <c r="F63" s="133" t="n"/>
       <c r="G63" s="133" t="n"/>
       <c r="H63" s="133">
-        <f>SUM(G64,G67,G70)</f>
+        <f>SUM(G64,G67)</f>
         <v/>
       </c>
       <c r="I63" s="131" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>pza</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2368,7 @@
       <c r="E64" s="133" t="n"/>
       <c r="F64" s="133" t="n"/>
       <c r="G64" s="133">
-        <f>SUM(G65:G66)</f>
+        <f>SUM(C65:C66)</f>
         <v/>
       </c>
       <c r="H64" s="133" t="n"/>
@@ -2379,19 +2378,17 @@
       <c r="A65" s="125" t="n"/>
       <c r="B65" s="126" t="inlineStr">
         <is>
-          <t>Recorrido Horizontal (En losa de techo)</t>
+          <t>Cocina (Microondas / Cocina Eléctrica)</t>
         </is>
       </c>
       <c r="C65" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D65" s="127" t="n">
-        <v>35</v>
-      </c>
+      <c r="D65" s="127" t="n"/>
       <c r="E65" s="127" t="n"/>
       <c r="F65" s="127" t="n"/>
       <c r="G65" s="127">
-        <f>C65*D65</f>
+        <f>C65</f>
         <v/>
       </c>
       <c r="H65" s="127" t="n"/>
@@ -2401,19 +2398,17 @@
       <c r="A66" s="125" t="n"/>
       <c r="B66" s="126" t="inlineStr">
         <is>
-          <t>Verticales: Bajadas a Cajas de Interruptores (h = 1.40 m)</t>
+          <t>Bomba de Agua (Servicio)</t>
         </is>
       </c>
       <c r="C66" s="127" t="n">
-        <v>3</v>
-      </c>
-      <c r="D66" s="127" t="n">
-        <v>1.4</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D66" s="127" t="n"/>
       <c r="E66" s="127" t="n"/>
       <c r="F66" s="127" t="n"/>
       <c r="G66" s="127">
-        <f>C66*D66</f>
+        <f>C66</f>
         <v/>
       </c>
       <c r="H66" s="127" t="n"/>
@@ -2423,7 +2418,7 @@
       <c r="A67" s="131" t="n"/>
       <c r="B67" s="132" t="inlineStr">
         <is>
-          <t>SEGUNDO NIVEL</t>
+          <t>TERCER NIVEL</t>
         </is>
       </c>
       <c r="C67" s="133" t="n"/>
@@ -2431,7 +2426,7 @@
       <c r="E67" s="133" t="n"/>
       <c r="F67" s="133" t="n"/>
       <c r="G67" s="133">
-        <f>SUM(G68:G69)</f>
+        <f>SUM(C68:C68)</f>
         <v/>
       </c>
       <c r="H67" s="133" t="n"/>
@@ -2441,98 +2436,97 @@
       <c r="A68" s="125" t="n"/>
       <c r="B68" s="126" t="inlineStr">
         <is>
-          <t>Recorrido Horizontal (En losa de techo)</t>
+          <t>Lavandería (Lavadora)</t>
         </is>
       </c>
       <c r="C68" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D68" s="127" t="n">
-        <v>35</v>
-      </c>
+      <c r="D68" s="127" t="n"/>
       <c r="E68" s="127" t="n"/>
       <c r="F68" s="127" t="n"/>
       <c r="G68" s="127">
-        <f>C68*D68</f>
+        <f>C68</f>
         <v/>
       </c>
       <c r="H68" s="127" t="n"/>
       <c r="I68" s="125" t="n"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="125" t="n"/>
-      <c r="B69" s="126" t="inlineStr">
-        <is>
-          <t>Verticales: Bajadas a Cajas de Interruptores (h = 1.40 m)</t>
-        </is>
-      </c>
-      <c r="C69" s="127" t="n">
-        <v>3</v>
-      </c>
-      <c r="D69" s="127" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="E69" s="127" t="n"/>
-      <c r="F69" s="127" t="n"/>
-      <c r="G69" s="127">
-        <f>C69*D69</f>
-        <v/>
-      </c>
-      <c r="H69" s="127" t="n"/>
-      <c r="I69" s="125" t="n"/>
+      <c r="A69" s="122" t="inlineStr">
+        <is>
+          <t>OE.5.2.2</t>
+        </is>
+      </c>
+      <c r="B69" s="123" t="inlineStr">
+        <is>
+          <t>CANALIZACIONES, TUBERIAS Y CONDUCTOS</t>
+        </is>
+      </c>
+      <c r="C69" s="124" t="n"/>
+      <c r="D69" s="124" t="n"/>
+      <c r="E69" s="124" t="n"/>
+      <c r="F69" s="124" t="n"/>
+      <c r="G69" s="124" t="n"/>
+      <c r="H69" s="124" t="n"/>
+      <c r="I69" s="122" t="n"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="131" t="n"/>
+      <c r="A70" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.2.1</t>
+        </is>
+      </c>
       <c r="B70" s="132" t="inlineStr">
         <is>
-          <t>TERCER NIVEL</t>
+          <t>Tubería PVC Liviana (PV-L) 3/4" (Canalización Alumbrado)</t>
         </is>
       </c>
       <c r="C70" s="133" t="n"/>
       <c r="D70" s="133" t="n"/>
       <c r="E70" s="133" t="n"/>
       <c r="F70" s="133" t="n"/>
-      <c r="G70" s="133">
-        <f>SUM(G71:G72)</f>
-        <v/>
-      </c>
-      <c r="H70" s="133" t="n"/>
-      <c r="I70" s="131" t="n"/>
+      <c r="G70" s="133" t="n"/>
+      <c r="H70" s="133">
+        <f>SUM(G71,G74,G77)</f>
+        <v/>
+      </c>
+      <c r="I70" s="131" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="125" t="n"/>
-      <c r="B71" s="126" t="inlineStr">
-        <is>
-          <t>Recorrido Horizontal (En losa de techo)</t>
-        </is>
-      </c>
-      <c r="C71" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D71" s="127" t="n">
-        <v>36.4</v>
-      </c>
-      <c r="E71" s="127" t="n"/>
-      <c r="F71" s="127" t="n"/>
-      <c r="G71" s="127">
-        <f>C71*D71</f>
-        <v/>
-      </c>
-      <c r="H71" s="127" t="n"/>
-      <c r="I71" s="125" t="n"/>
+      <c r="A71" s="131" t="n"/>
+      <c r="B71" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C71" s="133" t="n"/>
+      <c r="D71" s="133" t="n"/>
+      <c r="E71" s="133" t="n"/>
+      <c r="F71" s="133" t="n"/>
+      <c r="G71" s="133">
+        <f>SUM(G72:G73)</f>
+        <v/>
+      </c>
+      <c r="H71" s="133" t="n"/>
+      <c r="I71" s="131" t="n"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="125" t="n"/>
       <c r="B72" s="126" t="inlineStr">
         <is>
-          <t>Verticales: Bajadas a Cajas de Interruptores (h = 1.40 m)</t>
+          <t>Recorrido Horizontal (En losa de techo)</t>
         </is>
       </c>
       <c r="C72" s="127" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D72" s="127" t="n">
-        <v>1.4</v>
+        <v>35</v>
       </c>
       <c r="E72" s="127" t="n"/>
       <c r="F72" s="127" t="n"/>
@@ -2544,36 +2538,32 @@
       <c r="I72" s="125" t="n"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="131" t="inlineStr">
-        <is>
-          <t>OE.5.2.2.2</t>
-        </is>
-      </c>
-      <c r="B73" s="132" t="inlineStr">
-        <is>
-          <t>Tubería PVC Pesada (PV-P) 3/4" (Canalización Tomacorrientes)</t>
-        </is>
-      </c>
-      <c r="C73" s="133" t="n"/>
-      <c r="D73" s="133" t="n"/>
-      <c r="E73" s="133" t="n"/>
-      <c r="F73" s="133" t="n"/>
-      <c r="G73" s="133" t="n"/>
-      <c r="H73" s="133">
-        <f>SUM(G74,G78,G82)</f>
-        <v/>
-      </c>
-      <c r="I73" s="131" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+      <c r="A73" s="125" t="n"/>
+      <c r="B73" s="126" t="inlineStr">
+        <is>
+          <t>Verticales: Bajadas a Cajas de Interruptores (h = 1.40 m)</t>
+        </is>
+      </c>
+      <c r="C73" s="127" t="n">
+        <v>3</v>
+      </c>
+      <c r="D73" s="127" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E73" s="127" t="n"/>
+      <c r="F73" s="127" t="n"/>
+      <c r="G73" s="127">
+        <f>C73*D73</f>
+        <v/>
+      </c>
+      <c r="H73" s="127" t="n"/>
+      <c r="I73" s="125" t="n"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="131" t="n"/>
       <c r="B74" s="132" t="inlineStr">
         <is>
-          <t>PRIMER NIVEL</t>
+          <t>SEGUNDO NIVEL</t>
         </is>
       </c>
       <c r="C74" s="133" t="n"/>
@@ -2581,7 +2571,7 @@
       <c r="E74" s="133" t="n"/>
       <c r="F74" s="133" t="n"/>
       <c r="G74" s="133">
-        <f>SUM(G75:G77)</f>
+        <f>SUM(G75:G76)</f>
         <v/>
       </c>
       <c r="H74" s="133" t="n"/>
@@ -2591,14 +2581,14 @@
       <c r="A75" s="125" t="n"/>
       <c r="B75" s="126" t="inlineStr">
         <is>
-          <t>Recorrido Horizontal (En contrapiso de piso 1)</t>
+          <t>Recorrido Horizontal (En losa de techo)</t>
         </is>
       </c>
       <c r="C75" s="127" t="n">
         <v>1</v>
       </c>
       <c r="D75" s="127" t="n">
-        <v>35.9</v>
+        <v>35</v>
       </c>
       <c r="E75" s="127" t="n"/>
       <c r="F75" s="127" t="n"/>
@@ -2613,14 +2603,14 @@
       <c r="A76" s="125" t="n"/>
       <c r="B76" s="126" t="inlineStr">
         <is>
-          <t>Verticales: Subidas a Tomacorrientes Dobles (h = 0.30 m)</t>
+          <t>Verticales: Bajadas a Cajas de Interruptores (h = 1.40 m)</t>
         </is>
       </c>
       <c r="C76" s="127" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D76" s="127" t="n">
-        <v>0.3</v>
+        <v>1.4</v>
       </c>
       <c r="E76" s="127" t="n"/>
       <c r="F76" s="127" t="n"/>
@@ -2632,57 +2622,57 @@
       <c r="I76" s="125" t="n"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="125" t="n"/>
-      <c r="B77" s="126" t="inlineStr">
-        <is>
-          <t>Verticales: Subidas a Cocina/Bomba (Especiales h = 1.10 m)</t>
-        </is>
-      </c>
-      <c r="C77" s="127" t="n">
-        <v>5</v>
-      </c>
-      <c r="D77" s="127" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="E77" s="127" t="n"/>
-      <c r="F77" s="127" t="n"/>
-      <c r="G77" s="127">
-        <f>C77*D77</f>
-        <v/>
-      </c>
-      <c r="H77" s="127" t="n"/>
-      <c r="I77" s="125" t="n"/>
+      <c r="A77" s="131" t="n"/>
+      <c r="B77" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C77" s="133" t="n"/>
+      <c r="D77" s="133" t="n"/>
+      <c r="E77" s="133" t="n"/>
+      <c r="F77" s="133" t="n"/>
+      <c r="G77" s="133">
+        <f>SUM(G78:G79)</f>
+        <v/>
+      </c>
+      <c r="H77" s="133" t="n"/>
+      <c r="I77" s="131" t="n"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="131" t="n"/>
-      <c r="B78" s="132" t="inlineStr">
-        <is>
-          <t>SEGUNDO NIVEL</t>
-        </is>
-      </c>
-      <c r="C78" s="133" t="n"/>
-      <c r="D78" s="133" t="n"/>
-      <c r="E78" s="133" t="n"/>
-      <c r="F78" s="133" t="n"/>
-      <c r="G78" s="133">
-        <f>SUM(G79:G81)</f>
-        <v/>
-      </c>
-      <c r="H78" s="133" t="n"/>
-      <c r="I78" s="131" t="n"/>
+      <c r="A78" s="125" t="n"/>
+      <c r="B78" s="126" t="inlineStr">
+        <is>
+          <t>Recorrido Horizontal (En losa de techo)</t>
+        </is>
+      </c>
+      <c r="C78" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D78" s="127" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="E78" s="127" t="n"/>
+      <c r="F78" s="127" t="n"/>
+      <c r="G78" s="127">
+        <f>C78*D78</f>
+        <v/>
+      </c>
+      <c r="H78" s="127" t="n"/>
+      <c r="I78" s="125" t="n"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="125" t="n"/>
       <c r="B79" s="126" t="inlineStr">
         <is>
-          <t>Recorrido Horizontal (En contrapiso de piso 2)</t>
+          <t>Verticales: Bajadas a Cajas de Interruptores (h = 1.40 m)</t>
         </is>
       </c>
       <c r="C79" s="127" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D79" s="127" t="n">
-        <v>50.4</v>
+        <v>1.4</v>
       </c>
       <c r="E79" s="127" t="n"/>
       <c r="F79" s="127" t="n"/>
@@ -2694,79 +2684,83 @@
       <c r="I79" s="125" t="n"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="A80" s="125" t="n"/>
-      <c r="B80" s="126" t="inlineStr">
-        <is>
-          <t>Verticales: Subidas a Tomacorrientes Dobles (h = 0.30 m)</t>
-        </is>
-      </c>
-      <c r="C80" s="127" t="n">
-        <v>8</v>
-      </c>
-      <c r="D80" s="127" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E80" s="127" t="n"/>
-      <c r="F80" s="127" t="n"/>
-      <c r="G80" s="127">
-        <f>C80*D80</f>
-        <v/>
-      </c>
-      <c r="H80" s="127" t="n"/>
-      <c r="I80" s="125" t="n"/>
+      <c r="A80" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.2.2</t>
+        </is>
+      </c>
+      <c r="B80" s="132" t="inlineStr">
+        <is>
+          <t>Tubería PVC Pesada (PV-P) 3/4" (Canalización Tomacorrientes)</t>
+        </is>
+      </c>
+      <c r="C80" s="133" t="n"/>
+      <c r="D80" s="133" t="n"/>
+      <c r="E80" s="133" t="n"/>
+      <c r="F80" s="133" t="n"/>
+      <c r="G80" s="133" t="n"/>
+      <c r="H80" s="133">
+        <f>SUM(G81,G85,G89)</f>
+        <v/>
+      </c>
+      <c r="I80" s="131" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
-      <c r="A81" s="125" t="n"/>
-      <c r="B81" s="126" t="inlineStr">
-        <is>
-          <t>Verticales: Subidas a Baño GFCI (h = 1.10 m)</t>
-        </is>
-      </c>
-      <c r="C81" s="127" t="n">
+      <c r="A81" s="131" t="n"/>
+      <c r="B81" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C81" s="133" t="n"/>
+      <c r="D81" s="133" t="n"/>
+      <c r="E81" s="133" t="n"/>
+      <c r="F81" s="133" t="n"/>
+      <c r="G81" s="133">
+        <f>SUM(G82:G84)</f>
+        <v/>
+      </c>
+      <c r="H81" s="133" t="n"/>
+      <c r="I81" s="131" t="n"/>
+    </row>
+    <row r="82" ht="15.75" customHeight="1">
+      <c r="A82" s="125" t="n"/>
+      <c r="B82" s="126" t="inlineStr">
+        <is>
+          <t>Recorrido Horizontal (En contrapiso de piso 1)</t>
+        </is>
+      </c>
+      <c r="C82" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D81" s="127" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="E81" s="127" t="n"/>
-      <c r="F81" s="127" t="n"/>
-      <c r="G81" s="127">
-        <f>C81*D81</f>
-        <v/>
-      </c>
-      <c r="H81" s="127" t="n"/>
-      <c r="I81" s="125" t="n"/>
-    </row>
-    <row r="82" ht="15.75" customHeight="1">
-      <c r="A82" s="131" t="n"/>
-      <c r="B82" s="132" t="inlineStr">
-        <is>
-          <t>TERCER NIVEL</t>
-        </is>
-      </c>
-      <c r="C82" s="133" t="n"/>
-      <c r="D82" s="133" t="n"/>
-      <c r="E82" s="133" t="n"/>
-      <c r="F82" s="133" t="n"/>
-      <c r="G82" s="133">
-        <f>SUM(G83:G85)</f>
-        <v/>
-      </c>
-      <c r="H82" s="133" t="n"/>
-      <c r="I82" s="131" t="n"/>
+      <c r="D82" s="127" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="E82" s="127" t="n"/>
+      <c r="F82" s="127" t="n"/>
+      <c r="G82" s="127">
+        <f>C82*D82</f>
+        <v/>
+      </c>
+      <c r="H82" s="127" t="n"/>
+      <c r="I82" s="125" t="n"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="125" t="n"/>
       <c r="B83" s="126" t="inlineStr">
         <is>
-          <t>Recorrido Horizontal (En contrapiso de piso 3)</t>
+          <t>Verticales: Subidas a Tomacorrientes Dobles (h = 0.30 m)</t>
         </is>
       </c>
       <c r="C83" s="127" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D83" s="127" t="n">
-        <v>50</v>
+        <v>0.3</v>
       </c>
       <c r="E83" s="127" t="n"/>
       <c r="F83" s="127" t="n"/>
@@ -2781,14 +2775,14 @@
       <c r="A84" s="125" t="n"/>
       <c r="B84" s="126" t="inlineStr">
         <is>
-          <t>Verticales: Subidas a Tomacorrientes Dobles (h = 0.30 m)</t>
+          <t>Verticales: Subidas a Cocina/Bomba (Especiales h = 1.10 m)</t>
         </is>
       </c>
       <c r="C84" s="127" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D84" s="127" t="n">
-        <v>0.3</v>
+        <v>1.1</v>
       </c>
       <c r="E84" s="127" t="n"/>
       <c r="F84" s="127" t="n"/>
@@ -2800,83 +2794,79 @@
       <c r="I84" s="125" t="n"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
-      <c r="A85" s="125" t="n"/>
-      <c r="B85" s="126" t="inlineStr">
-        <is>
-          <t>Verticales: Subidas a Baño/Lavandería (h = 1.10 m)</t>
-        </is>
-      </c>
-      <c r="C85" s="127" t="n">
-        <v>2</v>
-      </c>
-      <c r="D85" s="127" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="E85" s="127" t="n"/>
-      <c r="F85" s="127" t="n"/>
-      <c r="G85" s="127">
-        <f>C85*D85</f>
-        <v/>
-      </c>
-      <c r="H85" s="127" t="n"/>
-      <c r="I85" s="125" t="n"/>
+      <c r="A85" s="131" t="n"/>
+      <c r="B85" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C85" s="133" t="n"/>
+      <c r="D85" s="133" t="n"/>
+      <c r="E85" s="133" t="n"/>
+      <c r="F85" s="133" t="n"/>
+      <c r="G85" s="133">
+        <f>SUM(G86:G88)</f>
+        <v/>
+      </c>
+      <c r="H85" s="133" t="n"/>
+      <c r="I85" s="131" t="n"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="131" t="inlineStr">
-        <is>
-          <t>OE.5.2.2.3</t>
-        </is>
-      </c>
-      <c r="B86" s="132" t="inlineStr">
-        <is>
-          <t>Tubería PVC Pesada (PV-P) 1" (Canalización Alimentador General)</t>
-        </is>
-      </c>
-      <c r="C86" s="133" t="n"/>
-      <c r="D86" s="133" t="n"/>
-      <c r="E86" s="133" t="n"/>
-      <c r="F86" s="133" t="n"/>
-      <c r="G86" s="133" t="n"/>
-      <c r="H86" s="133">
-        <f>SUM(G87)</f>
-        <v/>
-      </c>
-      <c r="I86" s="131" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+      <c r="A86" s="125" t="n"/>
+      <c r="B86" s="126" t="inlineStr">
+        <is>
+          <t>Recorrido Horizontal (En contrapiso de piso 2)</t>
+        </is>
+      </c>
+      <c r="C86" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D86" s="127" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="E86" s="127" t="n"/>
+      <c r="F86" s="127" t="n"/>
+      <c r="G86" s="127">
+        <f>C86*D86</f>
+        <v/>
+      </c>
+      <c r="H86" s="127" t="n"/>
+      <c r="I86" s="125" t="n"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
-      <c r="A87" s="131" t="n"/>
-      <c r="B87" s="132" t="inlineStr">
-        <is>
-          <t>TRAMO PRINCIPAL</t>
-        </is>
-      </c>
-      <c r="C87" s="133" t="n"/>
-      <c r="D87" s="133" t="n"/>
-      <c r="E87" s="133" t="n"/>
-      <c r="F87" s="133" t="n"/>
-      <c r="G87" s="133">
-        <f>SUM(G88:G93)</f>
-        <v/>
-      </c>
-      <c r="H87" s="133" t="n"/>
-      <c r="I87" s="131" t="n"/>
+      <c r="A87" s="125" t="n"/>
+      <c r="B87" s="126" t="inlineStr">
+        <is>
+          <t>Verticales: Subidas a Tomacorrientes Dobles (h = 0.30 m)</t>
+        </is>
+      </c>
+      <c r="C87" s="127" t="n">
+        <v>8</v>
+      </c>
+      <c r="D87" s="127" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E87" s="127" t="n"/>
+      <c r="F87" s="127" t="n"/>
+      <c r="G87" s="127">
+        <f>C87*D87</f>
+        <v/>
+      </c>
+      <c r="H87" s="127" t="n"/>
+      <c r="I87" s="125" t="n"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="125" t="n"/>
       <c r="B88" s="126" t="inlineStr">
         <is>
-          <t>Acometida a Tablero General TG-01 (Horizontal)</t>
+          <t>Verticales: Subidas a Baño GFCI (h = 1.10 m)</t>
         </is>
       </c>
       <c r="C88" s="127" t="n">
         <v>1</v>
       </c>
       <c r="D88" s="127" t="n">
-        <v>6.6</v>
+        <v>1.1</v>
       </c>
       <c r="E88" s="127" t="n"/>
       <c r="F88" s="127" t="n"/>
@@ -2888,39 +2878,35 @@
       <c r="I88" s="125" t="n"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
-      <c r="A89" s="125" t="n"/>
-      <c r="B89" s="126" t="inlineStr">
-        <is>
-          <t>Acometida a TG-01 (Vertical subida h = 1.40 m)</t>
-        </is>
-      </c>
-      <c r="C89" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D89" s="127" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="E89" s="127" t="n"/>
-      <c r="F89" s="127" t="n"/>
-      <c r="G89" s="127">
-        <f>C89*D89</f>
-        <v/>
-      </c>
-      <c r="H89" s="127" t="n"/>
-      <c r="I89" s="125" t="n"/>
+      <c r="A89" s="131" t="n"/>
+      <c r="B89" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C89" s="133" t="n"/>
+      <c r="D89" s="133" t="n"/>
+      <c r="E89" s="133" t="n"/>
+      <c r="F89" s="133" t="n"/>
+      <c r="G89" s="133">
+        <f>SUM(G90:G92)</f>
+        <v/>
+      </c>
+      <c r="H89" s="133" t="n"/>
+      <c r="I89" s="131" t="n"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="125" t="n"/>
       <c r="B90" s="126" t="inlineStr">
         <is>
-          <t>TG-01 a Tablero Distribución TD-01 (Horizontal)</t>
+          <t>Recorrido Horizontal (En contrapiso de piso 3)</t>
         </is>
       </c>
       <c r="C90" s="127" t="n">
         <v>1</v>
       </c>
       <c r="D90" s="127" t="n">
-        <v>7.6</v>
+        <v>50</v>
       </c>
       <c r="E90" s="127" t="n"/>
       <c r="F90" s="127" t="n"/>
@@ -2935,14 +2921,14 @@
       <c r="A91" s="125" t="n"/>
       <c r="B91" s="126" t="inlineStr">
         <is>
-          <t>TG-01 / TD-01 (Vertical subida h = 1.40 m)</t>
+          <t>Verticales: Subidas a Tomacorrientes Dobles (h = 0.30 m)</t>
         </is>
       </c>
       <c r="C91" s="127" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D91" s="127" t="n">
-        <v>1.4</v>
+        <v>0.3</v>
       </c>
       <c r="E91" s="127" t="n"/>
       <c r="F91" s="127" t="n"/>
@@ -2957,14 +2943,14 @@
       <c r="A92" s="125" t="n"/>
       <c r="B92" s="126" t="inlineStr">
         <is>
-          <t>TD-01 a Tablero Distribución TD-02 (Horizontal)</t>
+          <t>Verticales: Subidas a Baño/Lavandería (h = 1.10 m)</t>
         </is>
       </c>
       <c r="C92" s="127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D92" s="127" t="n">
-        <v>6.6</v>
+        <v>1.1</v>
       </c>
       <c r="E92" s="127" t="n"/>
       <c r="F92" s="127" t="n"/>
@@ -2976,162 +2962,176 @@
       <c r="I92" s="125" t="n"/>
     </row>
     <row r="93" ht="15.75" customHeight="1">
-      <c r="A93" s="125" t="n"/>
-      <c r="B93" s="126" t="inlineStr">
-        <is>
-          <t>TD-01 / TD-02 (Vertical subida h = 1.40 m)</t>
-        </is>
-      </c>
-      <c r="C93" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D93" s="127" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="E93" s="127" t="n"/>
-      <c r="F93" s="127" t="n"/>
-      <c r="G93" s="127">
-        <f>C93*D93</f>
-        <v/>
-      </c>
-      <c r="H93" s="127" t="n"/>
-      <c r="I93" s="125" t="n"/>
+      <c r="A93" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.2.3</t>
+        </is>
+      </c>
+      <c r="B93" s="132" t="inlineStr">
+        <is>
+          <t>Tubería PVC Pesada (PV-P) 1" (Canalización Alimentador General)</t>
+        </is>
+      </c>
+      <c r="C93" s="133" t="n"/>
+      <c r="D93" s="133" t="n"/>
+      <c r="E93" s="133" t="n"/>
+      <c r="F93" s="133" t="n"/>
+      <c r="G93" s="133" t="n"/>
+      <c r="H93" s="133">
+        <f>SUM(G94)</f>
+        <v/>
+      </c>
+      <c r="I93" s="131" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="15.75" customHeight="1">
-      <c r="A94" s="131" t="inlineStr">
-        <is>
-          <t>OE.5.2.2.4</t>
-        </is>
-      </c>
+      <c r="A94" s="131" t="n"/>
       <c r="B94" s="132" t="inlineStr">
         <is>
-          <t>Curvas de PVC Pesada (PV-P) 3/4" (Accesorios Tomacorrientes)</t>
+          <t>TRAMO PRINCIPAL</t>
         </is>
       </c>
       <c r="C94" s="133" t="n"/>
       <c r="D94" s="133" t="n"/>
       <c r="E94" s="133" t="n"/>
       <c r="F94" s="133" t="n"/>
-      <c r="G94" s="133" t="n"/>
-      <c r="H94" s="133">
-        <f>SUM(G95,G97,G99)</f>
-        <v/>
-      </c>
-      <c r="I94" s="131" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+      <c r="G94" s="133">
+        <f>SUM(G95:G100)</f>
+        <v/>
+      </c>
+      <c r="H94" s="133" t="n"/>
+      <c r="I94" s="131" t="n"/>
     </row>
     <row r="95" ht="15.75" customHeight="1">
-      <c r="A95" s="131" t="n"/>
-      <c r="B95" s="132" t="inlineStr">
-        <is>
-          <t>PRIMER NIVEL</t>
-        </is>
-      </c>
-      <c r="C95" s="133" t="n"/>
-      <c r="D95" s="133" t="n"/>
-      <c r="E95" s="133" t="n"/>
-      <c r="F95" s="133" t="n"/>
-      <c r="G95" s="133">
-        <f>SUM(C96:C96)</f>
-        <v/>
-      </c>
-      <c r="H95" s="133" t="n"/>
-      <c r="I95" s="131" t="n"/>
+      <c r="A95" s="125" t="n"/>
+      <c r="B95" s="126" t="inlineStr">
+        <is>
+          <t>Acometida a Tablero General TG-01 (Horizontal)</t>
+        </is>
+      </c>
+      <c r="C95" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" s="127" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="E95" s="127" t="n"/>
+      <c r="F95" s="127" t="n"/>
+      <c r="G95" s="127">
+        <f>C95*D95</f>
+        <v/>
+      </c>
+      <c r="H95" s="127" t="n"/>
+      <c r="I95" s="125" t="n"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="125" t="n"/>
       <c r="B96" s="126" t="inlineStr">
         <is>
-          <t>Curvas en subida a cajas de tomacorrientes</t>
+          <t>Acometida a TG-01 (Vertical subida h = 1.40 m)</t>
         </is>
       </c>
       <c r="C96" s="127" t="n">
-        <v>12</v>
-      </c>
-      <c r="D96" s="127" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D96" s="127" t="n">
+        <v>1.4</v>
+      </c>
       <c r="E96" s="127" t="n"/>
       <c r="F96" s="127" t="n"/>
       <c r="G96" s="127">
-        <f>C96</f>
+        <f>C96*D96</f>
         <v/>
       </c>
       <c r="H96" s="127" t="n"/>
       <c r="I96" s="125" t="n"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
-      <c r="A97" s="131" t="n"/>
-      <c r="B97" s="132" t="inlineStr">
-        <is>
-          <t>SEGUNDO NIVEL</t>
-        </is>
-      </c>
-      <c r="C97" s="133" t="n"/>
-      <c r="D97" s="133" t="n"/>
-      <c r="E97" s="133" t="n"/>
-      <c r="F97" s="133" t="n"/>
-      <c r="G97" s="133">
-        <f>SUM(C98:C98)</f>
-        <v/>
-      </c>
-      <c r="H97" s="133" t="n"/>
-      <c r="I97" s="131" t="n"/>
+      <c r="A97" s="125" t="n"/>
+      <c r="B97" s="126" t="inlineStr">
+        <is>
+          <t>TG-01 a Tablero Distribución TD-01 (Horizontal)</t>
+        </is>
+      </c>
+      <c r="C97" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D97" s="127" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="E97" s="127" t="n"/>
+      <c r="F97" s="127" t="n"/>
+      <c r="G97" s="127">
+        <f>C97*D97</f>
+        <v/>
+      </c>
+      <c r="H97" s="127" t="n"/>
+      <c r="I97" s="125" t="n"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="125" t="n"/>
       <c r="B98" s="126" t="inlineStr">
         <is>
-          <t>Curvas en subida a cajas de tomacorrientes</t>
+          <t>TG-01 / TD-01 (Vertical subida h = 1.40 m)</t>
         </is>
       </c>
       <c r="C98" s="127" t="n">
-        <v>18</v>
-      </c>
-      <c r="D98" s="127" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D98" s="127" t="n">
+        <v>1.4</v>
+      </c>
       <c r="E98" s="127" t="n"/>
       <c r="F98" s="127" t="n"/>
       <c r="G98" s="127">
-        <f>C98</f>
+        <f>C98*D98</f>
         <v/>
       </c>
       <c r="H98" s="127" t="n"/>
       <c r="I98" s="125" t="n"/>
     </row>
     <row r="99" ht="15.75" customHeight="1">
-      <c r="A99" s="131" t="n"/>
-      <c r="B99" s="132" t="inlineStr">
-        <is>
-          <t>TERCER NIVEL</t>
-        </is>
-      </c>
-      <c r="C99" s="133" t="n"/>
-      <c r="D99" s="133" t="n"/>
-      <c r="E99" s="133" t="n"/>
-      <c r="F99" s="133" t="n"/>
-      <c r="G99" s="133">
-        <f>SUM(C100:C100)</f>
-        <v/>
-      </c>
-      <c r="H99" s="133" t="n"/>
-      <c r="I99" s="131" t="n"/>
+      <c r="A99" s="125" t="n"/>
+      <c r="B99" s="126" t="inlineStr">
+        <is>
+          <t>TD-01 a Tablero Distribución TD-02 (Horizontal)</t>
+        </is>
+      </c>
+      <c r="C99" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D99" s="127" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="E99" s="127" t="n"/>
+      <c r="F99" s="127" t="n"/>
+      <c r="G99" s="127">
+        <f>C99*D99</f>
+        <v/>
+      </c>
+      <c r="H99" s="127" t="n"/>
+      <c r="I99" s="125" t="n"/>
     </row>
     <row r="100" ht="15.75" customHeight="1">
       <c r="A100" s="125" t="n"/>
       <c r="B100" s="126" t="inlineStr">
         <is>
-          <t>Curvas en subida a cajas de tomacorrientes</t>
+          <t>TD-01 / TD-02 (Vertical subida h = 1.40 m)</t>
         </is>
       </c>
       <c r="C100" s="127" t="n">
-        <v>15</v>
-      </c>
-      <c r="D100" s="127" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D100" s="127" t="n">
+        <v>1.4</v>
+      </c>
       <c r="E100" s="127" t="n"/>
       <c r="F100" s="127" t="n"/>
       <c r="G100" s="127">
-        <f>C100</f>
+        <f>C100*D100</f>
         <v/>
       </c>
       <c r="H100" s="127" t="n"/>
@@ -3140,12 +3140,12 @@
     <row r="101" ht="15.75" customHeight="1">
       <c r="A101" s="131" t="inlineStr">
         <is>
-          <t>OE.5.2.2.5</t>
+          <t>OE.5.2.2.4</t>
         </is>
       </c>
       <c r="B101" s="132" t="inlineStr">
         <is>
-          <t>Curvas de PVC Liviana (PV-L) 3/4" (Accesorios Alumbrado)</t>
+          <t>Curvas de PVC Pesada (PV-P) 3/4" (Accesorios Tomacorrientes)</t>
         </is>
       </c>
       <c r="C101" s="133" t="n"/>
@@ -3185,11 +3185,11 @@
       <c r="A103" s="125" t="n"/>
       <c r="B103" s="126" t="inlineStr">
         <is>
-          <t>Curvas en bajadas a cajas de interruptores</t>
+          <t>Curvas en subida a cajas de tomacorrientes</t>
         </is>
       </c>
       <c r="C103" s="127" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D103" s="127" t="n"/>
       <c r="E103" s="127" t="n"/>
@@ -3223,11 +3223,11 @@
       <c r="A105" s="125" t="n"/>
       <c r="B105" s="126" t="inlineStr">
         <is>
-          <t>Curvas en bajadas a cajas de interruptores</t>
+          <t>Curvas en subida a cajas de tomacorrientes</t>
         </is>
       </c>
       <c r="C105" s="127" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="D105" s="127" t="n"/>
       <c r="E105" s="127" t="n"/>
@@ -3261,11 +3261,11 @@
       <c r="A107" s="125" t="n"/>
       <c r="B107" s="126" t="inlineStr">
         <is>
-          <t>Curvas en bajadas a cajas de interruptores</t>
+          <t>Curvas en subida a cajas de tomacorrientes</t>
         </is>
       </c>
       <c r="C107" s="127" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D107" s="127" t="n"/>
       <c r="E107" s="127" t="n"/>
@@ -3278,241 +3278,235 @@
       <c r="I107" s="125" t="n"/>
     </row>
     <row r="108" ht="15.75" customHeight="1">
-      <c r="A108" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.2.6</t>
-        </is>
-      </c>
-      <c r="B108" s="126" t="inlineStr">
-        <is>
-          <t>Curva PVC Pesada (PV-P) 1" (Accesorios Alimentadores y tableros)</t>
-        </is>
-      </c>
-      <c r="C108" s="127" t="n">
-        <v>6</v>
-      </c>
-      <c r="D108" s="127" t="n"/>
-      <c r="E108" s="127" t="n"/>
-      <c r="F108" s="127" t="n"/>
-      <c r="G108" s="127">
-        <f>C108</f>
-        <v/>
-      </c>
-      <c r="H108" s="127">
-        <f>G108</f>
-        <v/>
-      </c>
-      <c r="I108" s="125" t="inlineStr">
+      <c r="A108" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.2.5</t>
+        </is>
+      </c>
+      <c r="B108" s="132" t="inlineStr">
+        <is>
+          <t>Curvas de PVC Liviana (PV-L) 3/4" (Accesorios Alumbrado)</t>
+        </is>
+      </c>
+      <c r="C108" s="133" t="n"/>
+      <c r="D108" s="133" t="n"/>
+      <c r="E108" s="133" t="n"/>
+      <c r="F108" s="133" t="n"/>
+      <c r="G108" s="133" t="n"/>
+      <c r="H108" s="133">
+        <f>SUM(G109,G111,G113)</f>
+        <v/>
+      </c>
+      <c r="I108" s="131" t="inlineStr">
         <is>
           <t>pza</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15.75" customHeight="1">
-      <c r="A109" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.2.7</t>
-        </is>
-      </c>
-      <c r="B109" s="126" t="inlineStr">
-        <is>
-          <t>Accesorios de canalización (Curvas, uniones, conectores, pegamento)</t>
-        </is>
-      </c>
-      <c r="C109" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D109" s="127" t="n"/>
-      <c r="E109" s="127" t="n"/>
-      <c r="F109" s="127" t="n"/>
-      <c r="G109" s="127">
-        <f>C109</f>
-        <v/>
-      </c>
-      <c r="H109" s="127">
-        <f>G109</f>
-        <v/>
-      </c>
-      <c r="I109" s="125" t="inlineStr">
-        <is>
-          <t>glb</t>
-        </is>
-      </c>
+      <c r="A109" s="131" t="n"/>
+      <c r="B109" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C109" s="133" t="n"/>
+      <c r="D109" s="133" t="n"/>
+      <c r="E109" s="133" t="n"/>
+      <c r="F109" s="133" t="n"/>
+      <c r="G109" s="133">
+        <f>SUM(C110:C110)</f>
+        <v/>
+      </c>
+      <c r="H109" s="133" t="n"/>
+      <c r="I109" s="131" t="n"/>
     </row>
     <row r="110" ht="15.75" customHeight="1">
-      <c r="A110" s="122" t="inlineStr">
-        <is>
-          <t>OE.5.2.3</t>
-        </is>
-      </c>
-      <c r="B110" s="123" t="inlineStr">
-        <is>
-          <t>CONDUCTORES Y CABLES</t>
-        </is>
-      </c>
-      <c r="C110" s="124" t="n"/>
-      <c r="D110" s="124" t="n"/>
-      <c r="E110" s="124" t="n"/>
-      <c r="F110" s="124" t="n"/>
-      <c r="G110" s="124" t="n"/>
-      <c r="H110" s="124" t="n"/>
-      <c r="I110" s="122" t="n"/>
+      <c r="A110" s="125" t="n"/>
+      <c r="B110" s="126" t="inlineStr">
+        <is>
+          <t>Curvas en bajadas a cajas de interruptores</t>
+        </is>
+      </c>
+      <c r="C110" s="127" t="n">
+        <v>4</v>
+      </c>
+      <c r="D110" s="127" t="n"/>
+      <c r="E110" s="127" t="n"/>
+      <c r="F110" s="127" t="n"/>
+      <c r="G110" s="127">
+        <f>C110</f>
+        <v/>
+      </c>
+      <c r="H110" s="127" t="n"/>
+      <c r="I110" s="125" t="n"/>
     </row>
     <row r="111" ht="15.75" customHeight="1">
-      <c r="A111" s="131" t="inlineStr">
-        <is>
-          <t>OE.5.2.3.1</t>
-        </is>
-      </c>
+      <c r="A111" s="131" t="n"/>
       <c r="B111" s="132" t="inlineStr">
         <is>
-          <t>Conductor de cobre LSOH 1.5 mm2 (Fase+Neutro Alumbrado)</t>
+          <t>SEGUNDO NIVEL</t>
         </is>
       </c>
       <c r="C111" s="133" t="n"/>
       <c r="D111" s="133" t="n"/>
       <c r="E111" s="133" t="n"/>
       <c r="F111" s="133" t="n"/>
-      <c r="G111" s="133" t="n"/>
-      <c r="H111" s="133">
-        <f>SUM(G112,G114,G116)</f>
-        <v/>
-      </c>
-      <c r="I111" s="131" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+      <c r="G111" s="133">
+        <f>SUM(C112:C112)</f>
+        <v/>
+      </c>
+      <c r="H111" s="133" t="n"/>
+      <c r="I111" s="131" t="n"/>
     </row>
     <row r="112" ht="15.75" customHeight="1">
-      <c r="A112" s="131" t="n"/>
-      <c r="B112" s="132" t="inlineStr">
-        <is>
-          <t>PRIMER NIVEL</t>
-        </is>
-      </c>
-      <c r="C112" s="133" t="n"/>
-      <c r="D112" s="133" t="n"/>
-      <c r="E112" s="133" t="n"/>
-      <c r="F112" s="133" t="n"/>
-      <c r="G112" s="133">
-        <f>SUM(G113:G113)</f>
-        <v/>
-      </c>
-      <c r="H112" s="133" t="n"/>
-      <c r="I112" s="131" t="n"/>
+      <c r="A112" s="125" t="n"/>
+      <c r="B112" s="126" t="inlineStr">
+        <is>
+          <t>Curvas en bajadas a cajas de interruptores</t>
+        </is>
+      </c>
+      <c r="C112" s="127" t="n">
+        <v>4</v>
+      </c>
+      <c r="D112" s="127" t="n"/>
+      <c r="E112" s="127" t="n"/>
+      <c r="F112" s="127" t="n"/>
+      <c r="G112" s="127">
+        <f>C112</f>
+        <v/>
+      </c>
+      <c r="H112" s="127" t="n"/>
+      <c r="I112" s="125" t="n"/>
     </row>
     <row r="113" ht="15.75" customHeight="1">
-      <c r="A113" s="125" t="n"/>
-      <c r="B113" s="126" t="inlineStr">
-        <is>
-          <t>Circuito C1 (Alumbrado 1er Piso)</t>
-        </is>
-      </c>
-      <c r="C113" s="127" t="n">
-        <v>2</v>
-      </c>
-      <c r="D113" s="127" t="n">
-        <v>40</v>
-      </c>
-      <c r="E113" s="127" t="n"/>
-      <c r="F113" s="127" t="n"/>
-      <c r="G113" s="127">
-        <f>C113*D113</f>
-        <v/>
-      </c>
-      <c r="H113" s="127" t="n"/>
-      <c r="I113" s="125" t="n"/>
+      <c r="A113" s="131" t="n"/>
+      <c r="B113" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C113" s="133" t="n"/>
+      <c r="D113" s="133" t="n"/>
+      <c r="E113" s="133" t="n"/>
+      <c r="F113" s="133" t="n"/>
+      <c r="G113" s="133">
+        <f>SUM(C114:C114)</f>
+        <v/>
+      </c>
+      <c r="H113" s="133" t="n"/>
+      <c r="I113" s="131" t="n"/>
     </row>
     <row r="114" ht="15.75" customHeight="1">
-      <c r="A114" s="131" t="n"/>
-      <c r="B114" s="132" t="inlineStr">
-        <is>
-          <t>SEGUNDO NIVEL</t>
-        </is>
-      </c>
-      <c r="C114" s="133" t="n"/>
-      <c r="D114" s="133" t="n"/>
-      <c r="E114" s="133" t="n"/>
-      <c r="F114" s="133" t="n"/>
-      <c r="G114" s="133">
-        <f>SUM(G115:G115)</f>
-        <v/>
-      </c>
-      <c r="H114" s="133" t="n"/>
-      <c r="I114" s="131" t="n"/>
+      <c r="A114" s="125" t="n"/>
+      <c r="B114" s="126" t="inlineStr">
+        <is>
+          <t>Curvas en bajadas a cajas de interruptores</t>
+        </is>
+      </c>
+      <c r="C114" s="127" t="n">
+        <v>4</v>
+      </c>
+      <c r="D114" s="127" t="n"/>
+      <c r="E114" s="127" t="n"/>
+      <c r="F114" s="127" t="n"/>
+      <c r="G114" s="127">
+        <f>C114</f>
+        <v/>
+      </c>
+      <c r="H114" s="127" t="n"/>
+      <c r="I114" s="125" t="n"/>
     </row>
     <row r="115" ht="15.75" customHeight="1">
-      <c r="A115" s="125" t="n"/>
+      <c r="A115" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.2.6</t>
+        </is>
+      </c>
       <c r="B115" s="126" t="inlineStr">
         <is>
-          <t>Circuito C4 (Alumbrado 2do Piso)</t>
+          <t>Curva PVC Pesada (PV-P) 1" (Accesorios Alimentadores y tableros)</t>
         </is>
       </c>
       <c r="C115" s="127" t="n">
-        <v>2</v>
-      </c>
-      <c r="D115" s="127" t="n">
-        <v>40</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="D115" s="127" t="n"/>
       <c r="E115" s="127" t="n"/>
       <c r="F115" s="127" t="n"/>
       <c r="G115" s="127">
-        <f>C115*D115</f>
-        <v/>
-      </c>
-      <c r="H115" s="127" t="n"/>
-      <c r="I115" s="125" t="n"/>
+        <f>C115</f>
+        <v/>
+      </c>
+      <c r="H115" s="127">
+        <f>G115</f>
+        <v/>
+      </c>
+      <c r="I115" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="15.75" customHeight="1">
-      <c r="A116" s="131" t="n"/>
-      <c r="B116" s="132" t="inlineStr">
-        <is>
-          <t>TERCER NIVEL</t>
-        </is>
-      </c>
-      <c r="C116" s="133" t="n"/>
-      <c r="D116" s="133" t="n"/>
-      <c r="E116" s="133" t="n"/>
-      <c r="F116" s="133" t="n"/>
-      <c r="G116" s="133">
-        <f>SUM(G117:G117)</f>
-        <v/>
-      </c>
-      <c r="H116" s="133" t="n"/>
-      <c r="I116" s="131" t="n"/>
+      <c r="A116" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.2.7</t>
+        </is>
+      </c>
+      <c r="B116" s="126" t="inlineStr">
+        <is>
+          <t>Accesorios de canalización (Curvas, uniones, conectores, pegamento)</t>
+        </is>
+      </c>
+      <c r="C116" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D116" s="127" t="n"/>
+      <c r="E116" s="127" t="n"/>
+      <c r="F116" s="127" t="n"/>
+      <c r="G116" s="127">
+        <f>C116</f>
+        <v/>
+      </c>
+      <c r="H116" s="127">
+        <f>G116</f>
+        <v/>
+      </c>
+      <c r="I116" s="125" t="inlineStr">
+        <is>
+          <t>glb</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="15.75" customHeight="1">
-      <c r="A117" s="125" t="n"/>
-      <c r="B117" s="126" t="inlineStr">
-        <is>
-          <t>Circuito C6 (Alumbrado 3er Piso)</t>
-        </is>
-      </c>
-      <c r="C117" s="127" t="n">
-        <v>2</v>
-      </c>
-      <c r="D117" s="127" t="n">
-        <v>40</v>
-      </c>
-      <c r="E117" s="127" t="n"/>
-      <c r="F117" s="127" t="n"/>
-      <c r="G117" s="127">
-        <f>C117*D117</f>
-        <v/>
-      </c>
-      <c r="H117" s="127" t="n"/>
-      <c r="I117" s="125" t="n"/>
+      <c r="A117" s="122" t="inlineStr">
+        <is>
+          <t>OE.5.2.3</t>
+        </is>
+      </c>
+      <c r="B117" s="123" t="inlineStr">
+        <is>
+          <t>CONDUCTORES Y CABLES</t>
+        </is>
+      </c>
+      <c r="C117" s="124" t="n"/>
+      <c r="D117" s="124" t="n"/>
+      <c r="E117" s="124" t="n"/>
+      <c r="F117" s="124" t="n"/>
+      <c r="G117" s="124" t="n"/>
+      <c r="H117" s="124" t="n"/>
+      <c r="I117" s="122" t="n"/>
     </row>
     <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="131" t="inlineStr">
         <is>
-          <t>OE.5.2.3.2</t>
+          <t>OE.5.2.3.1</t>
         </is>
       </c>
       <c r="B118" s="132" t="inlineStr">
         <is>
-          <t>Conductor de cobre LSOH 1.5 mm2 (Protección a Tierra Alumbrado)</t>
+          <t>Conductor de cobre LSOH 1.5 mm2 (Fase+Neutro Alumbrado)</t>
         </is>
       </c>
       <c r="C118" s="133" t="n"/>
@@ -3556,10 +3550,10 @@
         </is>
       </c>
       <c r="C120" s="127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D120" s="127" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E120" s="127" t="n"/>
       <c r="F120" s="127" t="n"/>
@@ -3596,10 +3590,10 @@
         </is>
       </c>
       <c r="C122" s="127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D122" s="127" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E122" s="127" t="n"/>
       <c r="F122" s="127" t="n"/>
@@ -3636,7 +3630,7 @@
         </is>
       </c>
       <c r="C124" s="127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D124" s="127" t="n">
         <v>40</v>
@@ -3653,12 +3647,12 @@
     <row r="125" ht="15.75" customHeight="1">
       <c r="A125" s="131" t="inlineStr">
         <is>
-          <t>OE.5.2.3.3</t>
+          <t>OE.5.2.3.2</t>
         </is>
       </c>
       <c r="B125" s="132" t="inlineStr">
         <is>
-          <t>Conductor de cobre LSOH 2.5 mm2 (Fase+Neutro Tomacorrientes)</t>
+          <t>Conductor de cobre LSOH 1.5 mm2 (Protección a Tierra Alumbrado)</t>
         </is>
       </c>
       <c r="C125" s="133" t="n"/>
@@ -3698,14 +3692,14 @@
       <c r="A127" s="125" t="n"/>
       <c r="B127" s="126" t="inlineStr">
         <is>
-          <t>Circuito C2 (Tomacorrientes 1er Piso)</t>
+          <t>Circuito C1 (Alumbrado 1er Piso)</t>
         </is>
       </c>
       <c r="C127" s="127" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D127" s="127" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E127" s="127" t="n"/>
       <c r="F127" s="127" t="n"/>
@@ -3738,14 +3732,14 @@
       <c r="A129" s="125" t="n"/>
       <c r="B129" s="126" t="inlineStr">
         <is>
-          <t>Circuito C5 (Tomacorrientes 2do Piso)</t>
+          <t>Circuito C4 (Alumbrado 2do Piso)</t>
         </is>
       </c>
       <c r="C129" s="127" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D129" s="127" t="n">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="E129" s="127" t="n"/>
       <c r="F129" s="127" t="n"/>
@@ -3778,14 +3772,14 @@
       <c r="A131" s="125" t="n"/>
       <c r="B131" s="126" t="inlineStr">
         <is>
-          <t>Circuito C7 (Tomacorrientes 3er Piso)</t>
+          <t>Circuito C6 (Alumbrado 3er Piso)</t>
         </is>
       </c>
       <c r="C131" s="127" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D131" s="127" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E131" s="127" t="n"/>
       <c r="F131" s="127" t="n"/>
@@ -3799,12 +3793,12 @@
     <row r="132" ht="15.75" customHeight="1">
       <c r="A132" s="131" t="inlineStr">
         <is>
-          <t>OE.5.2.3.4</t>
+          <t>OE.5.2.3.3</t>
         </is>
       </c>
       <c r="B132" s="132" t="inlineStr">
         <is>
-          <t>Conductor de cobre LSOH 2.5 mm2 (Protección a Tierra Tomacorrientes)</t>
+          <t>Conductor de cobre LSOH 2.5 mm2 (Fase+Neutro Tomacorrientes)</t>
         </is>
       </c>
       <c r="C132" s="133" t="n"/>
@@ -3848,7 +3842,7 @@
         </is>
       </c>
       <c r="C134" s="127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D134" s="127" t="n">
         <v>50</v>
@@ -3888,10 +3882,10 @@
         </is>
       </c>
       <c r="C136" s="127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D136" s="127" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E136" s="127" t="n"/>
       <c r="F136" s="127" t="n"/>
@@ -3928,10 +3922,10 @@
         </is>
       </c>
       <c r="C138" s="127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D138" s="127" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E138" s="127" t="n"/>
       <c r="F138" s="127" t="n"/>
@@ -3943,211 +3937,164 @@
       <c r="I138" s="125" t="n"/>
     </row>
     <row r="139" ht="15.75" customHeight="1">
-      <c r="A139" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.3.5</t>
-        </is>
-      </c>
-      <c r="B139" s="126" t="inlineStr">
-        <is>
-          <t>Conductor de cobre LSOH 2.5 mm2 (Alimentación Electrobomba)</t>
-        </is>
-      </c>
-      <c r="C139" s="127" t="n">
-        <v>35</v>
-      </c>
-      <c r="D139" s="127" t="n"/>
-      <c r="E139" s="127" t="n"/>
-      <c r="F139" s="127" t="n"/>
-      <c r="G139" s="127">
-        <f>C139</f>
-        <v/>
-      </c>
-      <c r="H139" s="127">
-        <f>G139</f>
-        <v/>
-      </c>
-      <c r="I139" s="125" t="inlineStr">
+      <c r="A139" s="131" t="inlineStr">
+        <is>
+          <t>OE.5.2.3.4</t>
+        </is>
+      </c>
+      <c r="B139" s="132" t="inlineStr">
+        <is>
+          <t>Conductor de cobre LSOH 2.5 mm2 (Protección a Tierra Tomacorrientes)</t>
+        </is>
+      </c>
+      <c r="C139" s="133" t="n"/>
+      <c r="D139" s="133" t="n"/>
+      <c r="E139" s="133" t="n"/>
+      <c r="F139" s="133" t="n"/>
+      <c r="G139" s="133" t="n"/>
+      <c r="H139" s="133">
+        <f>SUM(G140,G142,G144)</f>
+        <v/>
+      </c>
+      <c r="I139" s="131" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
     </row>
     <row r="140" ht="15.75" customHeight="1">
-      <c r="A140" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.3.6</t>
-        </is>
-      </c>
-      <c r="B140" s="126" t="inlineStr">
-        <is>
-          <t>Conductor de cobre LSOH 10 mm2 (Alimentador General)</t>
-        </is>
-      </c>
-      <c r="C140" s="127" t="n">
-        <v>60</v>
-      </c>
-      <c r="D140" s="127" t="n"/>
-      <c r="E140" s="127" t="n"/>
-      <c r="F140" s="127" t="n"/>
-      <c r="G140" s="127">
-        <f>C140</f>
-        <v/>
-      </c>
-      <c r="H140" s="127">
-        <f>G140</f>
-        <v/>
-      </c>
-      <c r="I140" s="125" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+      <c r="A140" s="131" t="n"/>
+      <c r="B140" s="132" t="inlineStr">
+        <is>
+          <t>PRIMER NIVEL</t>
+        </is>
+      </c>
+      <c r="C140" s="133" t="n"/>
+      <c r="D140" s="133" t="n"/>
+      <c r="E140" s="133" t="n"/>
+      <c r="F140" s="133" t="n"/>
+      <c r="G140" s="133">
+        <f>SUM(G141:G141)</f>
+        <v/>
+      </c>
+      <c r="H140" s="133" t="n"/>
+      <c r="I140" s="131" t="n"/>
     </row>
     <row r="141" ht="15.75" customHeight="1">
-      <c r="A141" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.3.7</t>
-        </is>
-      </c>
+      <c r="A141" s="125" t="n"/>
       <c r="B141" s="126" t="inlineStr">
         <is>
-          <t>Conductor de cobre temple blando 6 mm2 (Conexión Puesta a Tierra)</t>
+          <t>Circuito C2 (Tomacorrientes 1er Piso)</t>
         </is>
       </c>
       <c r="C141" s="127" t="n">
-        <v>25</v>
-      </c>
-      <c r="D141" s="127" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D141" s="127" t="n">
+        <v>50</v>
+      </c>
       <c r="E141" s="127" t="n"/>
       <c r="F141" s="127" t="n"/>
       <c r="G141" s="127">
-        <f>C141</f>
-        <v/>
-      </c>
-      <c r="H141" s="127">
-        <f>G141</f>
-        <v/>
-      </c>
-      <c r="I141" s="125" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+        <f>C141*D141</f>
+        <v/>
+      </c>
+      <c r="H141" s="127" t="n"/>
+      <c r="I141" s="125" t="n"/>
     </row>
     <row r="142" ht="15.75" customHeight="1">
-      <c r="A142" s="122" t="inlineStr">
-        <is>
-          <t>OE.5.2.4</t>
-        </is>
-      </c>
-      <c r="B142" s="123" t="inlineStr">
-        <is>
-          <t>CAJAS DE PASO Y DERIVACION</t>
-        </is>
-      </c>
-      <c r="C142" s="124" t="n"/>
-      <c r="D142" s="124" t="n"/>
-      <c r="E142" s="124" t="n"/>
-      <c r="F142" s="124" t="n"/>
-      <c r="G142" s="124" t="n"/>
-      <c r="H142" s="124" t="n"/>
-      <c r="I142" s="122" t="n"/>
+      <c r="A142" s="131" t="n"/>
+      <c r="B142" s="132" t="inlineStr">
+        <is>
+          <t>SEGUNDO NIVEL</t>
+        </is>
+      </c>
+      <c r="C142" s="133" t="n"/>
+      <c r="D142" s="133" t="n"/>
+      <c r="E142" s="133" t="n"/>
+      <c r="F142" s="133" t="n"/>
+      <c r="G142" s="133">
+        <f>SUM(G143:G143)</f>
+        <v/>
+      </c>
+      <c r="H142" s="133" t="n"/>
+      <c r="I142" s="131" t="n"/>
     </row>
     <row r="143" ht="15.75" customHeight="1">
-      <c r="A143" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.4.1</t>
-        </is>
-      </c>
+      <c r="A143" s="125" t="n"/>
       <c r="B143" s="126" t="inlineStr">
         <is>
-          <t>Caja de pase rectangular 4"x2" FG (Derivaciones y cambios)</t>
+          <t>Circuito C5 (Tomacorrientes 2do Piso)</t>
         </is>
       </c>
       <c r="C143" s="127" t="n">
-        <v>6</v>
-      </c>
-      <c r="D143" s="127" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D143" s="127" t="n">
+        <v>50</v>
+      </c>
       <c r="E143" s="127" t="n"/>
       <c r="F143" s="127" t="n"/>
       <c r="G143" s="127">
-        <f>C143</f>
-        <v/>
-      </c>
-      <c r="H143" s="127">
-        <f>G143</f>
-        <v/>
-      </c>
-      <c r="I143" s="125" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+        <f>C143*D143</f>
+        <v/>
+      </c>
+      <c r="H143" s="127" t="n"/>
+      <c r="I143" s="125" t="n"/>
     </row>
     <row r="144" ht="15.75" customHeight="1">
-      <c r="A144" s="122" t="inlineStr">
-        <is>
-          <t>OE.5.2.6</t>
-        </is>
-      </c>
-      <c r="B144" s="123" t="inlineStr">
-        <is>
-          <t>TABLEROS DE DISTRIBUCION Y DETALLES</t>
-        </is>
-      </c>
-      <c r="C144" s="124" t="n"/>
-      <c r="D144" s="124" t="n"/>
-      <c r="E144" s="124" t="n"/>
-      <c r="F144" s="124" t="n"/>
-      <c r="G144" s="124" t="n"/>
-      <c r="H144" s="124" t="n"/>
-      <c r="I144" s="122" t="n"/>
+      <c r="A144" s="131" t="n"/>
+      <c r="B144" s="132" t="inlineStr">
+        <is>
+          <t>TERCER NIVEL</t>
+        </is>
+      </c>
+      <c r="C144" s="133" t="n"/>
+      <c r="D144" s="133" t="n"/>
+      <c r="E144" s="133" t="n"/>
+      <c r="F144" s="133" t="n"/>
+      <c r="G144" s="133">
+        <f>SUM(G145:G145)</f>
+        <v/>
+      </c>
+      <c r="H144" s="133" t="n"/>
+      <c r="I144" s="131" t="n"/>
     </row>
     <row r="145" ht="15.75" customHeight="1">
-      <c r="A145" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.6.1</t>
-        </is>
-      </c>
+      <c r="A145" s="125" t="n"/>
       <c r="B145" s="126" t="inlineStr">
         <is>
-          <t>Tablero General TG-01 (12 polos, metálico empotrable, primer piso)</t>
+          <t>Circuito C7 (Tomacorrientes 3er Piso)</t>
         </is>
       </c>
       <c r="C145" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D145" s="127" t="n"/>
+      <c r="D145" s="127" t="n">
+        <v>50</v>
+      </c>
       <c r="E145" s="127" t="n"/>
       <c r="F145" s="127" t="n"/>
       <c r="G145" s="127">
-        <f>C145</f>
-        <v/>
-      </c>
-      <c r="H145" s="127">
-        <f>G145</f>
-        <v/>
-      </c>
-      <c r="I145" s="125" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
+        <f>C145*D145</f>
+        <v/>
+      </c>
+      <c r="H145" s="127" t="n"/>
+      <c r="I145" s="125" t="n"/>
     </row>
     <row r="146" ht="15.75" customHeight="1">
       <c r="A146" s="125" t="inlineStr">
         <is>
-          <t>OE.5.2.6.2</t>
+          <t>OE.5.2.3.5</t>
         </is>
       </c>
       <c r="B146" s="126" t="inlineStr">
         <is>
-          <t>Tablero de Distribución TD-01 (8 polos, metálico empotrable, segundo piso)</t>
+          <t>Conductor de cobre LSOH 2.5 mm2 (Alimentación Electrobomba)</t>
         </is>
       </c>
       <c r="C146" s="127" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="D146" s="127" t="n"/>
       <c r="E146" s="127" t="n"/>
@@ -4162,23 +4109,23 @@
       </c>
       <c r="I146" s="125" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="147" ht="15.75" customHeight="1">
       <c r="A147" s="125" t="inlineStr">
         <is>
-          <t>OE.5.2.6.3</t>
+          <t>OE.5.2.3.6</t>
         </is>
       </c>
       <c r="B147" s="126" t="inlineStr">
         <is>
-          <t>Tablero de Distribución TD-02 (8 polos, metálico empotrable, tercer piso)</t>
+          <t>Conductor de cobre LSOH 10 mm2 (Alimentador General)</t>
         </is>
       </c>
       <c r="C147" s="127" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="D147" s="127" t="n"/>
       <c r="E147" s="127" t="n"/>
@@ -4193,73 +4140,73 @@
       </c>
       <c r="I147" s="125" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="148" ht="15.75" customHeight="1">
-      <c r="A148" s="122" t="inlineStr">
-        <is>
-          <t>OE.5.2.8</t>
-        </is>
-      </c>
-      <c r="B148" s="123" t="inlineStr">
-        <is>
-          <t>DISPOSITIVOS DE MANIOBRA Y PROTECCION</t>
-        </is>
-      </c>
-      <c r="C148" s="124" t="n"/>
-      <c r="D148" s="124" t="n"/>
-      <c r="E148" s="124" t="n"/>
-      <c r="F148" s="124" t="n"/>
-      <c r="G148" s="124" t="n"/>
-      <c r="H148" s="124" t="n"/>
-      <c r="I148" s="122" t="n"/>
+      <c r="A148" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.3.7</t>
+        </is>
+      </c>
+      <c r="B148" s="126" t="inlineStr">
+        <is>
+          <t>Conductor de cobre temple blando 6 mm2 (Conexión Puesta a Tierra)</t>
+        </is>
+      </c>
+      <c r="C148" s="127" t="n">
+        <v>25</v>
+      </c>
+      <c r="D148" s="127" t="n"/>
+      <c r="E148" s="127" t="n"/>
+      <c r="F148" s="127" t="n"/>
+      <c r="G148" s="127">
+        <f>C148</f>
+        <v/>
+      </c>
+      <c r="H148" s="127">
+        <f>G148</f>
+        <v/>
+      </c>
+      <c r="I148" s="125" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="15.75" customHeight="1">
-      <c r="A149" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.8.1</t>
-        </is>
-      </c>
-      <c r="B149" s="126" t="inlineStr">
-        <is>
-          <t>Interruptor simple unipolar (adosar/empotrar, 10A)</t>
-        </is>
-      </c>
-      <c r="C149" s="127" t="n">
-        <v>6</v>
-      </c>
-      <c r="D149" s="127" t="n"/>
-      <c r="E149" s="127" t="n"/>
-      <c r="F149" s="127" t="n"/>
-      <c r="G149" s="127">
-        <f>C149</f>
-        <v/>
-      </c>
-      <c r="H149" s="127">
-        <f>G149</f>
-        <v/>
-      </c>
-      <c r="I149" s="125" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+      <c r="A149" s="122" t="inlineStr">
+        <is>
+          <t>OE.5.2.4</t>
+        </is>
+      </c>
+      <c r="B149" s="123" t="inlineStr">
+        <is>
+          <t>CAJAS DE PASO Y DERIVACION</t>
+        </is>
+      </c>
+      <c r="C149" s="124" t="n"/>
+      <c r="D149" s="124" t="n"/>
+      <c r="E149" s="124" t="n"/>
+      <c r="F149" s="124" t="n"/>
+      <c r="G149" s="124" t="n"/>
+      <c r="H149" s="124" t="n"/>
+      <c r="I149" s="122" t="n"/>
     </row>
     <row r="150" ht="15.75" customHeight="1">
       <c r="A150" s="125" t="inlineStr">
         <is>
-          <t>OE.5.2.8.2</t>
+          <t>OE.5.2.4.1</t>
         </is>
       </c>
       <c r="B150" s="126" t="inlineStr">
         <is>
-          <t>Interruptor de conmutación 3 vías (S3, escaleras)</t>
+          <t>Caja de pase rectangular 4"x2" FG (Derivaciones y cambios)</t>
         </is>
       </c>
       <c r="C150" s="127" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D150" s="127" t="n"/>
       <c r="E150" s="127" t="n"/>
@@ -4279,49 +4226,37 @@
       </c>
     </row>
     <row r="151" ht="15.75" customHeight="1">
-      <c r="A151" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.8.3</t>
-        </is>
-      </c>
-      <c r="B151" s="126" t="inlineStr">
-        <is>
-          <t>Interruptor termomagnetico 2P-10A (Alumbrado)</t>
-        </is>
-      </c>
-      <c r="C151" s="127" t="n">
-        <v>3</v>
-      </c>
-      <c r="D151" s="127" t="n"/>
-      <c r="E151" s="127" t="n"/>
-      <c r="F151" s="127" t="n"/>
-      <c r="G151" s="127">
-        <f>C151</f>
-        <v/>
-      </c>
-      <c r="H151" s="127">
-        <f>G151</f>
-        <v/>
-      </c>
-      <c r="I151" s="125" t="inlineStr">
-        <is>
-          <t>pza</t>
-        </is>
-      </c>
+      <c r="A151" s="122" t="inlineStr">
+        <is>
+          <t>OE.5.2.6</t>
+        </is>
+      </c>
+      <c r="B151" s="123" t="inlineStr">
+        <is>
+          <t>TABLEROS DE DISTRIBUCION Y DETALLES</t>
+        </is>
+      </c>
+      <c r="C151" s="124" t="n"/>
+      <c r="D151" s="124" t="n"/>
+      <c r="E151" s="124" t="n"/>
+      <c r="F151" s="124" t="n"/>
+      <c r="G151" s="124" t="n"/>
+      <c r="H151" s="124" t="n"/>
+      <c r="I151" s="122" t="n"/>
     </row>
     <row r="152" ht="15.75" customHeight="1">
       <c r="A152" s="125" t="inlineStr">
         <is>
-          <t>OE.5.2.8.4</t>
+          <t>OE.5.2.6.1</t>
         </is>
       </c>
       <c r="B152" s="126" t="inlineStr">
         <is>
-          <t>Interruptor termomagnetico 2P-16A (Tomacorrientes)</t>
+          <t>Tablero General TG-01 (12 polos, metálico empotrable, primer piso)</t>
         </is>
       </c>
       <c r="C152" s="127" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D152" s="127" t="n"/>
       <c r="E152" s="127" t="n"/>
@@ -4336,19 +4271,19 @@
       </c>
       <c r="I152" s="125" t="inlineStr">
         <is>
-          <t>pza</t>
+          <t>u</t>
         </is>
       </c>
     </row>
     <row r="153" ht="15.75" customHeight="1">
       <c r="A153" s="125" t="inlineStr">
         <is>
-          <t>OE.5.2.8.5</t>
+          <t>OE.5.2.6.2</t>
         </is>
       </c>
       <c r="B153" s="126" t="inlineStr">
         <is>
-          <t>Interruptor termomagnetico 2P-20A (Cocina / Cargas especiales)</t>
+          <t>Tablero de Distribución TD-01 (8 polos, metálico empotrable, segundo piso)</t>
         </is>
       </c>
       <c r="C153" s="127" t="n">
@@ -4367,19 +4302,19 @@
       </c>
       <c r="I153" s="125" t="inlineStr">
         <is>
-          <t>pza</t>
+          <t>u</t>
         </is>
       </c>
     </row>
     <row r="154" ht="15.75" customHeight="1">
       <c r="A154" s="125" t="inlineStr">
         <is>
-          <t>OE.5.2.8.6</t>
+          <t>OE.5.2.6.3</t>
         </is>
       </c>
       <c r="B154" s="126" t="inlineStr">
         <is>
-          <t>Interruptor termomagnetico general 2P-40A (TG-01)</t>
+          <t>Tablero de Distribución TD-02 (8 polos, metálico empotrable, tercer piso)</t>
         </is>
       </c>
       <c r="C154" s="127" t="n">
@@ -4398,92 +4333,104 @@
       </c>
       <c r="I154" s="125" t="inlineStr">
         <is>
+          <t>u</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="15.75" customHeight="1">
+      <c r="A155" s="122" t="inlineStr">
+        <is>
+          <t>OE.5.2.8</t>
+        </is>
+      </c>
+      <c r="B155" s="123" t="inlineStr">
+        <is>
+          <t>DISPOSITIVOS DE MANIOBRA Y PROTECCION</t>
+        </is>
+      </c>
+      <c r="C155" s="124" t="n"/>
+      <c r="D155" s="124" t="n"/>
+      <c r="E155" s="124" t="n"/>
+      <c r="F155" s="124" t="n"/>
+      <c r="G155" s="124" t="n"/>
+      <c r="H155" s="124" t="n"/>
+      <c r="I155" s="122" t="n"/>
+    </row>
+    <row r="156" ht="15.75" customHeight="1">
+      <c r="A156" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.8.1</t>
+        </is>
+      </c>
+      <c r="B156" s="126" t="inlineStr">
+        <is>
+          <t>Interruptor simple unipolar (adosar/empotrar, 10A)</t>
+        </is>
+      </c>
+      <c r="C156" s="127" t="n">
+        <v>6</v>
+      </c>
+      <c r="D156" s="127" t="n"/>
+      <c r="E156" s="127" t="n"/>
+      <c r="F156" s="127" t="n"/>
+      <c r="G156" s="127">
+        <f>C156</f>
+        <v/>
+      </c>
+      <c r="H156" s="127">
+        <f>G156</f>
+        <v/>
+      </c>
+      <c r="I156" s="125" t="inlineStr">
+        <is>
           <t>pza</t>
         </is>
       </c>
     </row>
-    <row r="155" ht="15.75" customHeight="1">
-      <c r="A155" s="125" t="inlineStr">
-        <is>
-          <t>OE.5.2.8.7</t>
-        </is>
-      </c>
-      <c r="B155" s="126" t="inlineStr">
-        <is>
-          <t>Interruptor diferencial 2P-25A-30mA (Protección personal)</t>
-        </is>
-      </c>
-      <c r="C155" s="127" t="n">
-        <v>1</v>
-      </c>
-      <c r="D155" s="127" t="n"/>
-      <c r="E155" s="127" t="n"/>
-      <c r="F155" s="127" t="n"/>
-      <c r="G155" s="127">
-        <f>C155</f>
-        <v/>
-      </c>
-      <c r="H155" s="127">
-        <f>G155</f>
-        <v/>
-      </c>
-      <c r="I155" s="125" t="inlineStr">
+    <row r="157" ht="15.75" customHeight="1">
+      <c r="A157" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.8.2</t>
+        </is>
+      </c>
+      <c r="B157" s="126" t="inlineStr">
+        <is>
+          <t>Interruptor de conmutación 3 vías (S3, escaleras)</t>
+        </is>
+      </c>
+      <c r="C157" s="127" t="n">
+        <v>4</v>
+      </c>
+      <c r="D157" s="127" t="n"/>
+      <c r="E157" s="127" t="n"/>
+      <c r="F157" s="127" t="n"/>
+      <c r="G157" s="127">
+        <f>C157</f>
+        <v/>
+      </c>
+      <c r="H157" s="127">
+        <f>G157</f>
+        <v/>
+      </c>
+      <c r="I157" s="125" t="inlineStr">
         <is>
           <t>pza</t>
         </is>
       </c>
-    </row>
-    <row r="156" ht="15.75" customHeight="1">
-      <c r="A156" s="119" t="inlineStr">
-        <is>
-          <t>OE.5.4</t>
-        </is>
-      </c>
-      <c r="B156" s="120" t="inlineStr">
-        <is>
-          <t>INSTALACION DE PUESTA A TIERRA</t>
-        </is>
-      </c>
-      <c r="C156" s="121" t="n"/>
-      <c r="D156" s="121" t="n"/>
-      <c r="E156" s="121" t="n"/>
-      <c r="F156" s="121" t="n"/>
-      <c r="G156" s="121" t="n"/>
-      <c r="H156" s="121" t="n"/>
-      <c r="I156" s="119" t="n"/>
-    </row>
-    <row r="157" ht="15.75" customHeight="1">
-      <c r="A157" s="122" t="inlineStr">
-        <is>
-          <t>OE.5.4.1</t>
-        </is>
-      </c>
-      <c r="B157" s="123" t="inlineStr">
-        <is>
-          <t>PUESTA A TIERRA PAT-1</t>
-        </is>
-      </c>
-      <c r="C157" s="124" t="n"/>
-      <c r="D157" s="124" t="n"/>
-      <c r="E157" s="124" t="n"/>
-      <c r="F157" s="124" t="n"/>
-      <c r="G157" s="124" t="n"/>
-      <c r="H157" s="124" t="n"/>
-      <c r="I157" s="122" t="n"/>
     </row>
     <row r="158" ht="15.75" customHeight="1">
       <c r="A158" s="125" t="inlineStr">
         <is>
-          <t>OE.5.4.1.1</t>
+          <t>OE.5.2.8.3</t>
         </is>
       </c>
       <c r="B158" s="126" t="inlineStr">
         <is>
-          <t>Varilla de cobre 5/8" x 2.40m, conector, caja registro, gel conductor y accesorios</t>
+          <t>Interruptor termomagnetico 2P-10A (Alumbrado)</t>
         </is>
       </c>
       <c r="C158" s="127" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D158" s="127" t="n"/>
       <c r="E158" s="127" t="n"/>
@@ -4498,42 +4445,54 @@
       </c>
       <c r="I158" s="125" t="inlineStr">
         <is>
-          <t>jgo</t>
+          <t>pza</t>
         </is>
       </c>
     </row>
     <row r="159" ht="15.75" customHeight="1">
-      <c r="A159" s="119" t="inlineStr">
-        <is>
-          <t>OE.5.5</t>
-        </is>
-      </c>
-      <c r="B159" s="120" t="inlineStr">
-        <is>
-          <t>ARTEFACTOS DE ALUMBRADO</t>
-        </is>
-      </c>
-      <c r="C159" s="121" t="n"/>
-      <c r="D159" s="121" t="n"/>
-      <c r="E159" s="121" t="n"/>
-      <c r="F159" s="121" t="n"/>
-      <c r="G159" s="121" t="n"/>
-      <c r="H159" s="121" t="n"/>
-      <c r="I159" s="119" t="n"/>
+      <c r="A159" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.8.4</t>
+        </is>
+      </c>
+      <c r="B159" s="126" t="inlineStr">
+        <is>
+          <t>Interruptor termomagnetico 2P-16A (Tomacorrientes)</t>
+        </is>
+      </c>
+      <c r="C159" s="127" t="n">
+        <v>5</v>
+      </c>
+      <c r="D159" s="127" t="n"/>
+      <c r="E159" s="127" t="n"/>
+      <c r="F159" s="127" t="n"/>
+      <c r="G159" s="127">
+        <f>C159</f>
+        <v/>
+      </c>
+      <c r="H159" s="127">
+        <f>G159</f>
+        <v/>
+      </c>
+      <c r="I159" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
     </row>
     <row r="160" ht="15.75" customHeight="1">
       <c r="A160" s="125" t="inlineStr">
         <is>
-          <t>OE.5.5.1</t>
+          <t>OE.5.2.8.5</t>
         </is>
       </c>
       <c r="B160" s="126" t="inlineStr">
         <is>
-          <t>Luminaria LED interior de adosar 12 W (Iluminación general)</t>
+          <t>Interruptor termomagnetico 2P-20A (Cocina / Cargas especiales)</t>
         </is>
       </c>
       <c r="C160" s="127" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D160" s="127" t="n"/>
       <c r="E160" s="127" t="n"/>
@@ -4553,33 +4512,45 @@
       </c>
     </row>
     <row r="161" ht="15.75" customHeight="1">
-      <c r="A161" s="119" t="inlineStr">
-        <is>
-          <t>OE.5.6</t>
-        </is>
-      </c>
-      <c r="B161" s="120" t="inlineStr">
-        <is>
-          <t>EQUIPOS ELECTRICOS Y MECANICOS</t>
-        </is>
-      </c>
-      <c r="C161" s="121" t="n"/>
-      <c r="D161" s="121" t="n"/>
-      <c r="E161" s="121" t="n"/>
-      <c r="F161" s="121" t="n"/>
-      <c r="G161" s="121" t="n"/>
-      <c r="H161" s="121" t="n"/>
-      <c r="I161" s="119" t="n"/>
+      <c r="A161" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.2.8.6</t>
+        </is>
+      </c>
+      <c r="B161" s="126" t="inlineStr">
+        <is>
+          <t>Interruptor termomagnetico general 2P-40A (TG-01)</t>
+        </is>
+      </c>
+      <c r="C161" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D161" s="127" t="n"/>
+      <c r="E161" s="127" t="n"/>
+      <c r="F161" s="127" t="n"/>
+      <c r="G161" s="127">
+        <f>C161</f>
+        <v/>
+      </c>
+      <c r="H161" s="127">
+        <f>G161</f>
+        <v/>
+      </c>
+      <c r="I161" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="15.75" customHeight="1">
       <c r="A162" s="125" t="inlineStr">
         <is>
-          <t>OE.5.6.1</t>
+          <t>OE.5.2.8.7</t>
         </is>
       </c>
       <c r="B162" s="126" t="inlineStr">
         <is>
-          <t>Electrobomba monofásica de agua 1 HP, 220V, 60Hz</t>
+          <t>Interruptor diferencial 2P-25A-30mA (Protección personal)</t>
         </is>
       </c>
       <c r="C162" s="127" t="n">
@@ -4598,19 +4569,19 @@
       </c>
       <c r="I162" s="125" t="inlineStr">
         <is>
-          <t>UND</t>
+          <t>pza</t>
         </is>
       </c>
     </row>
     <row r="163" ht="15.75" customHeight="1">
       <c r="A163" s="119" t="inlineStr">
         <is>
-          <t>OE.5.7</t>
+          <t>OE.5.4</t>
         </is>
       </c>
       <c r="B163" s="120" t="inlineStr">
         <is>
-          <t>PRUEBAS ELECTRICAS</t>
+          <t>INSTALACION DE PUESTA A TIERRA</t>
         </is>
       </c>
       <c r="C163" s="121" t="n"/>
@@ -4622,43 +4593,205 @@
       <c r="I163" s="119" t="n"/>
     </row>
     <row r="164" ht="15.75" customHeight="1">
-      <c r="A164" s="125" t="inlineStr">
+      <c r="A164" s="122" t="inlineStr">
+        <is>
+          <t>OE.5.4.1</t>
+        </is>
+      </c>
+      <c r="B164" s="123" t="inlineStr">
+        <is>
+          <t>PUESTA A TIERRA PAT-1</t>
+        </is>
+      </c>
+      <c r="C164" s="124" t="n"/>
+      <c r="D164" s="124" t="n"/>
+      <c r="E164" s="124" t="n"/>
+      <c r="F164" s="124" t="n"/>
+      <c r="G164" s="124" t="n"/>
+      <c r="H164" s="124" t="n"/>
+      <c r="I164" s="122" t="n"/>
+    </row>
+    <row r="165" ht="15.75" customHeight="1">
+      <c r="A165" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.4.1.1</t>
+        </is>
+      </c>
+      <c r="B165" s="126" t="inlineStr">
+        <is>
+          <t>Varilla de cobre 5/8" x 2.40m, conector, caja registro, gel conductor y accesorios</t>
+        </is>
+      </c>
+      <c r="C165" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D165" s="127" t="n"/>
+      <c r="E165" s="127" t="n"/>
+      <c r="F165" s="127" t="n"/>
+      <c r="G165" s="127">
+        <f>C165</f>
+        <v/>
+      </c>
+      <c r="H165" s="127">
+        <f>G165</f>
+        <v/>
+      </c>
+      <c r="I165" s="125" t="inlineStr">
+        <is>
+          <t>jgo</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="15.75" customHeight="1">
+      <c r="A166" s="119" t="inlineStr">
+        <is>
+          <t>OE.5.5</t>
+        </is>
+      </c>
+      <c r="B166" s="120" t="inlineStr">
+        <is>
+          <t>ARTEFACTOS DE ALUMBRADO</t>
+        </is>
+      </c>
+      <c r="C166" s="121" t="n"/>
+      <c r="D166" s="121" t="n"/>
+      <c r="E166" s="121" t="n"/>
+      <c r="F166" s="121" t="n"/>
+      <c r="G166" s="121" t="n"/>
+      <c r="H166" s="121" t="n"/>
+      <c r="I166" s="119" t="n"/>
+    </row>
+    <row r="167" ht="15.75" customHeight="1">
+      <c r="A167" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.5.1</t>
+        </is>
+      </c>
+      <c r="B167" s="126" t="inlineStr">
+        <is>
+          <t>Luminaria LED interior de adosar 12 W (Iluminación general)</t>
+        </is>
+      </c>
+      <c r="C167" s="127" t="n">
+        <v>19</v>
+      </c>
+      <c r="D167" s="127" t="n"/>
+      <c r="E167" s="127" t="n"/>
+      <c r="F167" s="127" t="n"/>
+      <c r="G167" s="127">
+        <f>C167</f>
+        <v/>
+      </c>
+      <c r="H167" s="127">
+        <f>G167</f>
+        <v/>
+      </c>
+      <c r="I167" s="125" t="inlineStr">
+        <is>
+          <t>pza</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="15.75" customHeight="1">
+      <c r="A168" s="119" t="inlineStr">
+        <is>
+          <t>OE.5.6</t>
+        </is>
+      </c>
+      <c r="B168" s="120" t="inlineStr">
+        <is>
+          <t>EQUIPOS ELECTRICOS Y MECANICOS</t>
+        </is>
+      </c>
+      <c r="C168" s="121" t="n"/>
+      <c r="D168" s="121" t="n"/>
+      <c r="E168" s="121" t="n"/>
+      <c r="F168" s="121" t="n"/>
+      <c r="G168" s="121" t="n"/>
+      <c r="H168" s="121" t="n"/>
+      <c r="I168" s="119" t="n"/>
+    </row>
+    <row r="169" ht="15.75" customHeight="1">
+      <c r="A169" s="125" t="inlineStr">
+        <is>
+          <t>OE.5.6.1</t>
+        </is>
+      </c>
+      <c r="B169" s="126" t="inlineStr">
+        <is>
+          <t>Electrobomba monofásica de agua 1 HP, 220V, 60Hz</t>
+        </is>
+      </c>
+      <c r="C169" s="127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D169" s="127" t="n"/>
+      <c r="E169" s="127" t="n"/>
+      <c r="F169" s="127" t="n"/>
+      <c r="G169" s="127">
+        <f>C169</f>
+        <v/>
+      </c>
+      <c r="H169" s="127">
+        <f>G169</f>
+        <v/>
+      </c>
+      <c r="I169" s="125" t="inlineStr">
+        <is>
+          <t>UND</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="15.75" customHeight="1">
+      <c r="A170" s="119" t="inlineStr">
+        <is>
+          <t>OE.5.7</t>
+        </is>
+      </c>
+      <c r="B170" s="120" t="inlineStr">
+        <is>
+          <t>PRUEBAS ELECTRICAS</t>
+        </is>
+      </c>
+      <c r="C170" s="121" t="n"/>
+      <c r="D170" s="121" t="n"/>
+      <c r="E170" s="121" t="n"/>
+      <c r="F170" s="121" t="n"/>
+      <c r="G170" s="121" t="n"/>
+      <c r="H170" s="121" t="n"/>
+      <c r="I170" s="119" t="n"/>
+    </row>
+    <row r="171" ht="15.75" customHeight="1">
+      <c r="A171" s="125" t="inlineStr">
         <is>
           <t>OE.5.7.1</t>
         </is>
       </c>
-      <c r="B164" s="126" t="inlineStr">
+      <c r="B171" s="126" t="inlineStr">
         <is>
           <t>Pruebas de aislamiento, continuidad de línea y resistencia de puesta a tierra</t>
         </is>
       </c>
-      <c r="C164" s="127" t="n">
+      <c r="C171" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D164" s="127" t="n"/>
-      <c r="E164" s="127" t="n"/>
-      <c r="F164" s="127" t="n"/>
-      <c r="G164" s="127">
-        <f>C164</f>
-        <v/>
-      </c>
-      <c r="H164" s="127">
-        <f>G164</f>
-        <v/>
-      </c>
-      <c r="I164" s="125" t="inlineStr">
+      <c r="D171" s="127" t="n"/>
+      <c r="E171" s="127" t="n"/>
+      <c r="F171" s="127" t="n"/>
+      <c r="G171" s="127">
+        <f>C171</f>
+        <v/>
+      </c>
+      <c r="H171" s="127">
+        <f>G171</f>
+        <v/>
+      </c>
+      <c r="I171" s="125" t="inlineStr">
         <is>
           <t>glb</t>
         </is>
       </c>
     </row>
-    <row r="165" ht="12.75" customHeight="1"/>
-    <row r="166" ht="12.75" customHeight="1"/>
-    <row r="167" ht="12.75" customHeight="1"/>
-    <row r="168" ht="12.75" customHeight="1"/>
-    <row r="169" ht="12.75" customHeight="1"/>
-    <row r="170" ht="12.75" customHeight="1"/>
-    <row r="171" ht="12.75" customHeight="1"/>
     <row r="172" ht="12.75" customHeight="1"/>
     <row r="173" ht="12.75" customHeight="1"/>
     <row r="174" ht="12.75" customHeight="1"/>

</xml_diff>